<commit_message>
feat: implement 20-column financial schema with dynamic margins and live pricing formulas
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -82,7 +82,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -93,11 +93,23 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="4" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="3" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -464,22 +476,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M37"/>
+  <dimension ref="A1:T37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="45" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="45" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="48" customWidth="1" min="8" max="8"/>
+    <col width="48" customWidth="1" min="9" max="9"/>
+    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="17" customWidth="1" min="11" max="11"/>
+    <col width="15" customWidth="1" min="12" max="12"/>
+    <col width="14" customWidth="1" min="13" max="13"/>
+    <col width="12" customWidth="1" min="14" max="14"/>
+    <col width="12" customWidth="1" min="15" max="15"/>
+    <col width="12" customWidth="1" min="16" max="16"/>
+    <col width="16" customWidth="1" min="17" max="17"/>
+    <col width="48" customWidth="1" min="18" max="18"/>
+    <col width="48" customWidth="1" min="19" max="19"/>
+    <col width="48" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,27 +544,62 @@
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>Price (CNY)</t>
+          <t>Local Image Path</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Stock</t>
+          <t>product price</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Weight (kg)</t>
+          <t>china delivery</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>Image URL</t>
+          <t>air shipping</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>Local Image Path</t>
+          <t>bd delivery</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>packaging</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>printing</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>other</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>landing cost</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>margin</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>sell price</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>max discount</t>
         </is>
       </c>
     </row>
@@ -580,7 +634,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G2" s="2" t="inlineStr">
+      <c r="G2" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -590,90 +644,124 @@
           <t>https://moveon.global/BD_en/products/0000000TPCI3HYH3-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-independent-station-15spod13t-semi-hosted-civi4/1AD8305263723979</t>
         </is>
       </c>
-      <c r="I2" s="3" t="inlineStr">
-        <is>
-          <t>113.64</t>
-        </is>
-      </c>
-      <c r="J2" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K2" s="3" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01OU8KPT1RM1GtpDyQH_!!2206506402096-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="inlineStr"/>
+      <c r="I2" s="2" t="inlineStr"/>
+      <c r="J2" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q2" s="4">
+        <f>SUM(J2:P2)</f>
+        <v/>
+      </c>
+      <c r="R2" s="4">
+        <f>IF(Q2&lt;300, Q2*1.4, IF(Q2&lt;400, Q2*1.33, Q2*1.25))</f>
+        <v/>
+      </c>
+      <c r="S2" s="5">
+        <f>INT(R2/100)*100 + IF(MOD(ROUND(R2,0),100)&lt;25, 0, IF(MOD(ROUND(R2,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T2" s="4">
+        <f>IF(S2&lt;300, 0, MIN(99, IF(S2&lt;500, S2*7%, IF(S2&lt;700, S2*12%, S2*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="4" t="inlineStr">
+      <c r="A3" s="6" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max Phone Case, Magnetic, Transparent, with Lens Film</t>
         </is>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>18PM-TPUM-CR-N</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="7" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>Cherry Red Magnetic Style</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F3" s="5" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G3" s="4" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="H3" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000P47PA9R8D-suitable-for-iphone-18-pro-max-phone-case-magnetic-transparent-with-apple-17-lens-film-full-coverage-and-a-simple-drop-resistant-design/1AD8373708955104</t>
         </is>
       </c>
-      <c r="I3" s="5" t="inlineStr">
-        <is>
-          <t>295.48</t>
-        </is>
-      </c>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>4979</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L3" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01AKWeWYQ63VC2R3rs_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M3" s="4" t="inlineStr"/>
+      <c r="I3" s="6" t="inlineStr"/>
+      <c r="J3" s="8" t="n">
+        <v>345.8</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>24.61</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>35.01</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P3" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="8">
+        <f>SUM(J3:P3)</f>
+        <v/>
+      </c>
+      <c r="R3" s="8">
+        <f>IF(Q3&lt;300, Q3*1.4, IF(Q3&lt;400, Q3*1.33, Q3*1.25))</f>
+        <v/>
+      </c>
+      <c r="S3" s="9">
+        <f>INT(R3/100)*100 + IF(MOD(ROUND(R3,0),100)&lt;25, 0, IF(MOD(ROUND(R3,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T3" s="8">
+        <f>IF(S3&lt;300, 0, MIN(99, IF(S3&lt;500, S3*7%, IF(S3&lt;700, S3*12%, S3*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -706,7 +794,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G4" s="2" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -716,90 +804,124 @@
           <t>https://moveon.global/BD_en/products/0000000P47PA9R8D-suitable-for-iphone-18-pro-max-phone-case-magnetic-transparent-with-apple-17-lens-film-full-coverage-and-a-simple-drop-resistant-design/1AD8373708955104</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>295.48</t>
-        </is>
-      </c>
-      <c r="J4" s="3" t="inlineStr">
-        <is>
-          <t>4979</t>
-        </is>
-      </c>
-      <c r="K4" s="3" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01AKWeWYQ63VC2R3rs_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="inlineStr"/>
+      <c r="I4" s="2" t="inlineStr"/>
+      <c r="J4" s="4" t="n">
+        <v>345.8</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>24.61</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>35.01</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q4" s="4">
+        <f>SUM(J4:P4)</f>
+        <v/>
+      </c>
+      <c r="R4" s="4">
+        <f>IF(Q4&lt;300, Q4*1.4, IF(Q4&lt;400, Q4*1.33, Q4*1.25))</f>
+        <v/>
+      </c>
+      <c r="S4" s="5">
+        <f>INT(R4/100)*100 + IF(MOD(ROUND(R4,0),100)&lt;25, 0, IF(MOD(ROUND(R4,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T4" s="4">
+        <f>IF(S4&lt;300, 0, MIN(99, IF(S4&lt;500, S4*7%, IF(S4&lt;700, S4*12%, S4*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>T4P-AC-BG-N</t>
         </is>
       </c>
-      <c r="C5" s="5" t="inlineStr">
+      <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="7" t="inlineStr">
         <is>
           <t>Black -Green</t>
         </is>
       </c>
-      <c r="E5" s="5" t="inlineStr">
+      <c r="E5" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F5" s="5" t="inlineStr">
+      <c r="F5" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G5" s="4" t="inlineStr">
+      <c r="G5" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H5" s="4" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I5" s="5" t="inlineStr">
-        <is>
-          <t>136.37</t>
-        </is>
-      </c>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>4999</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
-      </c>
-      <c r="L5" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01DmquW2fJYHE1chua_!!2221354516123-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M5" s="4" t="inlineStr"/>
+      <c r="I5" s="6" t="inlineStr"/>
+      <c r="J5" s="8" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="8">
+        <f>SUM(J5:P5)</f>
+        <v/>
+      </c>
+      <c r="R5" s="8">
+        <f>IF(Q5&lt;300, Q5*1.4, IF(Q5&lt;400, Q5*1.33, Q5*1.25))</f>
+        <v/>
+      </c>
+      <c r="S5" s="9">
+        <f>INT(R5/100)*100 + IF(MOD(ROUND(R5,0),100)&lt;25, 0, IF(MOD(ROUND(R5,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T5" s="8">
+        <f>IF(S5&lt;300, 0, MIN(99, IF(S5&lt;500, S5*7%, IF(S5&lt;700, S5*12%, S5*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -832,7 +954,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G6" s="2" t="inlineStr">
+      <c r="G6" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -842,90 +964,124 @@
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I6" s="3" t="inlineStr">
-        <is>
-          <t>136.37</t>
-        </is>
-      </c>
-      <c r="J6" s="3" t="inlineStr">
-        <is>
-          <t>4999</t>
-        </is>
-      </c>
-      <c r="K6" s="3" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01DmquW2fJYHE1chua_!!2221354516123-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="inlineStr"/>
+      <c r="I6" s="2" t="inlineStr"/>
+      <c r="J6" s="4" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="4">
+        <f>SUM(J6:P6)</f>
+        <v/>
+      </c>
+      <c r="R6" s="4">
+        <f>IF(Q6&lt;300, Q6*1.4, IF(Q6&lt;400, Q6*1.33, Q6*1.25))</f>
+        <v/>
+      </c>
+      <c r="S6" s="5">
+        <f>INT(R6/100)*100 + IF(MOD(ROUND(R6,0),100)&lt;25, 0, IF(MOD(ROUND(R6,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T6" s="4">
+        <f>IF(S6&lt;300, 0, MIN(99, IF(S6&lt;500, S6*7%, IF(S6&lt;700, S6*12%, S6*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="6" t="inlineStr">
         <is>
           <t>Redmi  Turbo4 Pro Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>T4P-AC-BB-N</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="7" t="inlineStr">
         <is>
           <t>Black -Blue</t>
         </is>
       </c>
-      <c r="E7" s="5" t="inlineStr">
+      <c r="E7" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F7" s="5" t="inlineStr">
+      <c r="F7" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G7" s="4" t="inlineStr">
+      <c r="G7" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H7" s="4" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I7" s="5" t="inlineStr">
-        <is>
-          <t>136.37</t>
-        </is>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>4999</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
-      </c>
-      <c r="L7" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01DmquW2fJYHE1chua_!!2221354516123-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M7" s="4" t="inlineStr"/>
+      <c r="I7" s="6" t="inlineStr"/>
+      <c r="J7" s="8" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q7" s="8">
+        <f>SUM(J7:P7)</f>
+        <v/>
+      </c>
+      <c r="R7" s="8">
+        <f>IF(Q7&lt;300, Q7*1.4, IF(Q7&lt;400, Q7*1.33, Q7*1.25))</f>
+        <v/>
+      </c>
+      <c r="S7" s="9">
+        <f>INT(R7/100)*100 + IF(MOD(ROUND(R7,0),100)&lt;25, 0, IF(MOD(ROUND(R7,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T7" s="8">
+        <f>IF(S7&lt;300, 0, MIN(99, IF(S7&lt;500, S7*7%, IF(S7&lt;700, S7*12%, S7*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -950,7 +1106,7 @@
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Redmi Turbo 4 </t>
+          <t>Redmi Turbo 4</t>
         </is>
       </c>
       <c r="F8" s="3" t="inlineStr">
@@ -958,7 +1114,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G8" s="2" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -968,86 +1124,120 @@
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I8" s="3" t="inlineStr">
-        <is>
-          <t>136.37</t>
-        </is>
-      </c>
-      <c r="J8" s="3" t="inlineStr">
-        <is>
-          <t>4999</t>
-        </is>
-      </c>
-      <c r="K8" s="3" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01DmquW2fJYHE1chua_!!2221354516123-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="inlineStr"/>
+      <c r="I8" s="2" t="inlineStr"/>
+      <c r="J8" s="4" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="4">
+        <f>SUM(J8:P8)</f>
+        <v/>
+      </c>
+      <c r="R8" s="4">
+        <f>IF(Q8&lt;300, Q8*1.4, IF(Q8&lt;400, Q8*1.33, Q8*1.25))</f>
+        <v/>
+      </c>
+      <c r="S8" s="5">
+        <f>INT(R8/100)*100 + IF(MOD(ROUND(R8,0),100)&lt;25, 0, IF(MOD(ROUND(R8,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T8" s="4">
+        <f>IF(S8&lt;300, 0, MIN(99, IF(S8&lt;500, S8*7%, IF(S8&lt;700, S8*12%, S8*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>T4-AC-BB-N</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="7" t="inlineStr">
         <is>
           <t>Black -Blue</t>
         </is>
       </c>
-      <c r="E9" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Redmi Turbo 4 </t>
-        </is>
-      </c>
-      <c r="F9" s="5" t="inlineStr">
+      <c r="E9" s="7" t="inlineStr">
+        <is>
+          <t>Redmi Turbo 4</t>
+        </is>
+      </c>
+      <c r="F9" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr"/>
-      <c r="H9" s="4" t="inlineStr">
+      <c r="G9" s="7" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I9" s="5" t="inlineStr">
-        <is>
-          <t>136.37</t>
-        </is>
-      </c>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>4999</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr">
-        <is>
-          <t>0.006</t>
-        </is>
-      </c>
-      <c r="L9" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01DmquW2fJYHE1chua_!!2221354516123-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M9" s="4" t="inlineStr"/>
+      <c r="I9" s="6" t="inlineStr"/>
+      <c r="J9" s="8" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M9" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="8">
+        <f>SUM(J9:P9)</f>
+        <v/>
+      </c>
+      <c r="R9" s="8">
+        <f>IF(Q9&lt;300, Q9*1.4, IF(Q9&lt;400, Q9*1.33, Q9*1.25))</f>
+        <v/>
+      </c>
+      <c r="S9" s="9">
+        <f>INT(R9/100)*100 + IF(MOD(ROUND(R9,0),100)&lt;25, 0, IF(MOD(ROUND(R9,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T9" s="8">
+        <f>IF(S9&lt;300, 0, MIN(99, IF(S9&lt;500, S9*7%, IF(S9&lt;700, S9*12%, S9*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1080,7 +1270,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G10" s="2" t="inlineStr">
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1090,90 +1280,124 @@
           <t>https://moveon.global/BD_en/products/0000000O0R0QIE2O-jit-one-piece-dropshippinggalaxys25-phone-case-semi-managed-s24-fully-managed-s24fe-aliexpress/1AD8304920318534</t>
         </is>
       </c>
-      <c r="I10" s="3" t="inlineStr">
-        <is>
-          <t>90.92</t>
-        </is>
-      </c>
-      <c r="J10" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K10" s="3" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN0123uXdf1RM1GtTzUvX_!!2206506402096-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr"/>
+      <c r="I10" s="2" t="inlineStr"/>
+      <c r="J10" s="4" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="4">
+        <f>SUM(J10:P10)</f>
+        <v/>
+      </c>
+      <c r="R10" s="4">
+        <f>IF(Q10&lt;300, Q10*1.4, IF(Q10&lt;400, Q10*1.33, Q10*1.25))</f>
+        <v/>
+      </c>
+      <c r="S10" s="5">
+        <f>INT(R10/100)*100 + IF(MOD(ROUND(R10,0),100)&lt;25, 0, IF(MOD(ROUND(R10,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T10" s="4">
+        <f>IF(S10&lt;300, 0, MIN(99, IF(S10&lt;500, S10*7%, IF(S10&lt;700, S10*12%, S10*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="11">
-      <c r="A11" s="4" t="inlineStr">
+      <c r="A11" s="6" t="inlineStr">
         <is>
           <t>RedmiTurbo 4 Pro Tempered Glass Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>T4P-TG-WP-N</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="7" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="7" t="inlineStr">
         <is>
           <t>White Print</t>
         </is>
       </c>
-      <c r="E11" s="5" t="inlineStr">
+      <c r="E11" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F11" s="5" t="inlineStr">
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H11" s="4" t="inlineStr">
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I11" s="5" t="inlineStr">
-        <is>
-          <t>113.64</t>
-        </is>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="L11" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01Qig4Ng1RM1GaafrvV_!!2206506402096-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M11" s="4" t="inlineStr"/>
+      <c r="I11" s="6" t="inlineStr"/>
+      <c r="J11" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P11" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="8">
+        <f>SUM(J11:P11)</f>
+        <v/>
+      </c>
+      <c r="R11" s="8">
+        <f>IF(Q11&lt;300, Q11*1.4, IF(Q11&lt;400, Q11*1.33, Q11*1.25))</f>
+        <v/>
+      </c>
+      <c r="S11" s="9">
+        <f>INT(R11/100)*100 + IF(MOD(ROUND(R11,0),100)&lt;25, 0, IF(MOD(ROUND(R11,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T11" s="8">
+        <f>IF(S11&lt;300, 0, MIN(99, IF(S11&lt;500, S11*7%, IF(S11&lt;700, S11*12%, S11*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -1206,7 +1430,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G12" s="2" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1216,90 +1440,124 @@
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I12" s="3" t="inlineStr">
-        <is>
-          <t>113.64</t>
-        </is>
-      </c>
-      <c r="J12" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K12" s="3" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01Qig4Ng1RM1GaafrvV_!!2206506402096-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="I12" s="2" t="inlineStr"/>
+      <c r="J12" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="4">
+        <f>SUM(J12:P12)</f>
+        <v/>
+      </c>
+      <c r="R12" s="4">
+        <f>IF(Q12&lt;300, Q12*1.4, IF(Q12&lt;400, Q12*1.33, Q12*1.25))</f>
+        <v/>
+      </c>
+      <c r="S12" s="5">
+        <f>INT(R12/100)*100 + IF(MOD(ROUND(R12,0),100)&lt;25, 0, IF(MOD(ROUND(R12,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T12" s="4">
+        <f>IF(S12&lt;300, 0, MIN(99, IF(S12&lt;500, S12*7%, IF(S12&lt;700, S12*12%, S12*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="13">
-      <c r="A13" s="4" t="inlineStr">
+      <c r="A13" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B13" s="5" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>T4P-TG-WP-N</t>
         </is>
       </c>
-      <c r="C13" s="5" t="inlineStr">
+      <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr">
+      <c r="D13" s="7" t="inlineStr">
         <is>
           <t>White Print</t>
         </is>
       </c>
-      <c r="E13" s="5" t="inlineStr">
+      <c r="E13" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F13" s="5" t="inlineStr">
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G13" s="4" t="inlineStr">
+      <c r="G13" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H13" s="4" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I13" s="5" t="inlineStr">
-        <is>
-          <t>113.64</t>
-        </is>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="L13" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01Qig4Ng1RM1GaafrvV_!!2206506402096-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M13" s="4" t="inlineStr"/>
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P13" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="8">
+        <f>SUM(J13:P13)</f>
+        <v/>
+      </c>
+      <c r="R13" s="8">
+        <f>IF(Q13&lt;300, Q13*1.4, IF(Q13&lt;400, Q13*1.33, Q13*1.25))</f>
+        <v/>
+      </c>
+      <c r="S13" s="9">
+        <f>INT(R13/100)*100 + IF(MOD(ROUND(R13,0),100)&lt;25, 0, IF(MOD(ROUND(R13,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T13" s="8">
+        <f>IF(S13&lt;300, 0, MIN(99, IF(S13&lt;500, S13*7%, IF(S13&lt;700, S13*12%, S13*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1332,7 +1590,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G14" s="2" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1342,95 +1600,129 @@
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I14" s="3" t="inlineStr">
-        <is>
-          <t>113.64</t>
-        </is>
-      </c>
-      <c r="J14" s="3" t="inlineStr">
-        <is>
-          <t>100</t>
-        </is>
-      </c>
-      <c r="K14" s="3" t="inlineStr">
-        <is>
-          <t>0.01</t>
-        </is>
-      </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01Qig4Ng1RM1GaafrvV_!!2206506402096-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="inlineStr"/>
+      <c r="I14" s="2" t="inlineStr"/>
+      <c r="J14" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="4">
+        <f>SUM(J14:P14)</f>
+        <v/>
+      </c>
+      <c r="R14" s="4">
+        <f>IF(Q14&lt;300, Q14*1.4, IF(Q14&lt;400, Q14*1.33, Q14*1.25))</f>
+        <v/>
+      </c>
+      <c r="S14" s="5">
+        <f>INT(R14/100)*100 + IF(MOD(ROUND(R14,0),100)&lt;25, 0, IF(MOD(ROUND(R14,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T14" s="4">
+        <f>IF(S14&lt;300, 0, MIN(99, IF(S14&lt;500, S14*7%, IF(S14&lt;700, S14*12%, S14*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" s="4" t="inlineStr">
+      <c r="A15" s="6" t="inlineStr">
         <is>
           <t>Honor 600 Skin Protective Case</t>
         </is>
       </c>
-      <c r="B15" s="5" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>H600-SKn-G-N</t>
         </is>
       </c>
-      <c r="C15" s="5" t="inlineStr">
+      <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Skin</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr">
+      <c r="D15" s="7" t="inlineStr">
         <is>
           <t>Grey</t>
         </is>
       </c>
-      <c r="E15" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Honor 600 </t>
-        </is>
-      </c>
-      <c r="F15" s="5" t="inlineStr">
+      <c r="E15" s="7" t="inlineStr">
+        <is>
+          <t>Honor 600</t>
+        </is>
+      </c>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H15" s="4" t="inlineStr">
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/000000074X6RUVK3-suitable-for-honor-600-phone-case-honor-600-pro-international-version-carbon-fiber-pattern-leather-protective-cover-back-shell-type/1AD8348014988676</t>
         </is>
       </c>
-      <c r="I15" s="5" t="inlineStr">
-        <is>
-          <t>125.01</t>
-        </is>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>29993</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L15" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01elBfvZ1ui7GYuoAXj_!!2212501536070-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M15" s="4" t="inlineStr"/>
+      <c r="I15" s="6" t="inlineStr"/>
+      <c r="J15" s="8" t="n">
+        <v>146.3</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="M15" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P15" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q15" s="8">
+        <f>SUM(J15:P15)</f>
+        <v/>
+      </c>
+      <c r="R15" s="8">
+        <f>IF(Q15&lt;300, Q15*1.4, IF(Q15&lt;400, Q15*1.33, Q15*1.25))</f>
+        <v/>
+      </c>
+      <c r="S15" s="9">
+        <f>INT(R15/100)*100 + IF(MOD(ROUND(R15,0),100)&lt;25, 0, IF(MOD(ROUND(R15,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T15" s="8">
+        <f>IF(S15&lt;300, 0, MIN(99, IF(S15&lt;500, S15*7%, IF(S15&lt;700, S15*12%, S15*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Honor 600 Pro Skin Protective Case </t>
+          <t>Honor 600 Pro Skin Protective Case</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
@@ -1458,7 +1750,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G16" s="2" t="inlineStr">
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1468,90 +1760,124 @@
           <t>https://moveon.global/BD_en/products/000000074X6RUVK3-suitable-for-honor-600-phone-case-honor-600-pro-international-version-carbon-fiber-pattern-leather-protective-cover-back-shell-type/1AD8348014988676</t>
         </is>
       </c>
-      <c r="I16" s="3" t="inlineStr">
-        <is>
-          <t>125.01</t>
-        </is>
-      </c>
-      <c r="J16" s="3" t="inlineStr">
-        <is>
-          <t>29992</t>
-        </is>
-      </c>
-      <c r="K16" s="3" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01elBfvZ1ui7GYuoAXj_!!2212501536070-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="inlineStr"/>
+      <c r="I16" s="2" t="inlineStr"/>
+      <c r="J16" s="4" t="n">
+        <v>146.3</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="4">
+        <f>SUM(J16:P16)</f>
+        <v/>
+      </c>
+      <c r="R16" s="4">
+        <f>IF(Q16&lt;300, Q16*1.4, IF(Q16&lt;400, Q16*1.33, Q16*1.25))</f>
+        <v/>
+      </c>
+      <c r="S16" s="5">
+        <f>INT(R16/100)*100 + IF(MOD(ROUND(R16,0),100)&lt;25, 0, IF(MOD(ROUND(R16,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T16" s="4">
+        <f>IF(S16&lt;300, 0, MIN(99, IF(S16&lt;500, S16*7%, IF(S16&lt;700, S16*12%, S16*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Samsung Galaxy S26 Ultra Wood Grain Magnetic Case </t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>S26U-PW-B-N</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C17" s="7" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D17" s="7" t="inlineStr">
         <is>
           <t>Poplar Wood Grain</t>
         </is>
       </c>
-      <c r="E17" s="5" t="inlineStr">
+      <c r="E17" s="7" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
-      <c r="F17" s="5" t="inlineStr">
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G17" s="4" t="inlineStr">
+      <c r="G17" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H17" s="4" t="inlineStr">
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
         </is>
       </c>
-      <c r="I17" s="5" t="inlineStr">
-        <is>
-          <t>215.93</t>
-        </is>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>4989</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L17" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01iUQW781rBBsKxOkkY_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M17" s="4" t="inlineStr"/>
+      <c r="I17" s="6" t="inlineStr"/>
+      <c r="J17" s="8" t="n">
+        <v>252.7</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>18.09</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q17" s="8">
+        <f>SUM(J17:P17)</f>
+        <v/>
+      </c>
+      <c r="R17" s="8">
+        <f>IF(Q17&lt;300, Q17*1.4, IF(Q17&lt;400, Q17*1.33, Q17*1.25))</f>
+        <v/>
+      </c>
+      <c r="S17" s="9">
+        <f>INT(R17/100)*100 + IF(MOD(ROUND(R17,0),100)&lt;25, 0, IF(MOD(ROUND(R17,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T17" s="8">
+        <f>IF(S17&lt;300, 0, MIN(99, IF(S17&lt;500, S17*7%, IF(S17&lt;700, S17*12%, S17*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1584,7 +1910,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G18" s="2" t="inlineStr">
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1594,95 +1920,129 @@
           <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
         </is>
       </c>
-      <c r="I18" s="3" t="inlineStr">
-        <is>
-          <t>215.93</t>
-        </is>
-      </c>
-      <c r="J18" s="3" t="inlineStr">
-        <is>
-          <t>4989</t>
-        </is>
-      </c>
-      <c r="K18" s="3" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01iUQW781rBBsKxOkkY_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="inlineStr"/>
+      <c r="I18" s="2" t="inlineStr"/>
+      <c r="J18" s="4" t="n">
+        <v>252.7</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>18.09</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q18" s="4">
+        <f>SUM(J18:P18)</f>
+        <v/>
+      </c>
+      <c r="R18" s="4">
+        <f>IF(Q18&lt;300, Q18*1.4, IF(Q18&lt;400, Q18*1.33, Q18*1.25))</f>
+        <v/>
+      </c>
+      <c r="S18" s="5">
+        <f>INT(R18/100)*100 + IF(MOD(ROUND(R18,0),100)&lt;25, 0, IF(MOD(ROUND(R18,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T18" s="4">
+        <f>IF(S18&lt;300, 0, MIN(99, IF(S18&lt;500, S18*7%, IF(S18&lt;700, S18*12%, S18*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="19">
-      <c r="A19" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Samsung Galaxy S26 Ultra Magnetic Invisible Bracket </t>
-        </is>
-      </c>
-      <c r="B19" s="5" t="inlineStr">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra Magnetic Invisible Bracket</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>S26U-MI-B-N</t>
         </is>
       </c>
-      <c r="C19" s="5" t="inlineStr">
+      <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Metal lens frame Acrylic / TPU</t>
         </is>
       </c>
-      <c r="D19" s="5" t="inlineStr">
+      <c r="D19" s="7" t="inlineStr">
         <is>
           <t>Black – Magnetic Invisible Bracket</t>
         </is>
       </c>
-      <c r="E19" s="5" t="inlineStr">
+      <c r="E19" s="7" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
-      <c r="F19" s="5" t="inlineStr">
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G19" s="4" t="inlineStr">
+      <c r="G19" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H19" s="4" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000PWJ01ZSK1-metal-invisible-lens-bracket-suitable-for-samsung-s26ultra-magnetic-phone-case-s25fe-transparent-s24plus-case/1AC5307428543960</t>
         </is>
       </c>
-      <c r="I19" s="5" t="inlineStr">
-        <is>
-          <t>227.06</t>
-        </is>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>9956</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L19" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01TEB9pF1RWYE0j8rua_!!2207694312119-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M19" s="4" t="inlineStr"/>
+      <c r="I19" s="6" t="inlineStr"/>
+      <c r="J19" s="8" t="n">
+        <v>265.74</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P19" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q19" s="8">
+        <f>SUM(J19:P19)</f>
+        <v/>
+      </c>
+      <c r="R19" s="8">
+        <f>IF(Q19&lt;300, Q19*1.4, IF(Q19&lt;400, Q19*1.33, Q19*1.25))</f>
+        <v/>
+      </c>
+      <c r="S19" s="9">
+        <f>INT(R19/100)*100 + IF(MOD(ROUND(R19,0),100)&lt;25, 0, IF(MOD(ROUND(R19,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T19" s="8">
+        <f>IF(S19&lt;300, 0, MIN(99, IF(S19&lt;500, S19*7%, IF(S19&lt;700, S19*12%, S19*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPhone 18 Pro Magnetic Acrylic Case </t>
+          <t>iPhone 18 Pro Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -1710,7 +2070,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G20" s="2" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1720,95 +2080,129 @@
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I20" s="3" t="inlineStr">
-        <is>
-          <t>74.55</t>
-        </is>
-      </c>
-      <c r="J20" s="3" t="inlineStr">
-        <is>
-          <t>8788</t>
-        </is>
-      </c>
-      <c r="K20" s="3" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01Fr0azo1MyspxaybHL_!!2209951271504-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr"/>
+      <c r="I20" s="2" t="inlineStr"/>
+      <c r="J20" s="4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q20" s="4">
+        <f>SUM(J20:P20)</f>
+        <v/>
+      </c>
+      <c r="R20" s="4">
+        <f>IF(Q20&lt;300, Q20*1.4, IF(Q20&lt;400, Q20*1.33, Q20*1.25))</f>
+        <v/>
+      </c>
+      <c r="S20" s="5">
+        <f>INT(R20/100)*100 + IF(MOD(ROUND(R20,0),100)&lt;25, 0, IF(MOD(ROUND(R20,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T20" s="4">
+        <f>IF(S20&lt;300, 0, MIN(99, IF(S20&lt;500, S20*7%, IF(S20&lt;700, S20*12%, S20*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">iPhone 18  Pro Max Magnetic Acrylic Case </t>
-        </is>
-      </c>
-      <c r="B21" s="5" t="inlineStr">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>iPhone 18  Pro Max Magnetic Acrylic Case</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>18PM-AC-M-R-N</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C21" s="7" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D21" s="7" t="inlineStr">
         <is>
           <t>Wine Red</t>
         </is>
       </c>
-      <c r="E21" s="5" t="inlineStr">
+      <c r="E21" s="7" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F21" s="5" t="inlineStr">
+      <c r="F21" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H21" s="4" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I21" s="5" t="inlineStr">
-        <is>
-          <t>74.55</t>
-        </is>
-      </c>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>8788</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L21" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01Fr0azo1MyspxaybHL_!!2209951271504-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M21" s="4" t="inlineStr"/>
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="8" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L21" s="8" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O21" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P21" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q21" s="8">
+        <f>SUM(J21:P21)</f>
+        <v/>
+      </c>
+      <c r="R21" s="8">
+        <f>IF(Q21&lt;300, Q21*1.4, IF(Q21&lt;400, Q21*1.33, Q21*1.25))</f>
+        <v/>
+      </c>
+      <c r="S21" s="9">
+        <f>INT(R21/100)*100 + IF(MOD(ROUND(R21,0),100)&lt;25, 0, IF(MOD(ROUND(R21,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T21" s="8">
+        <f>IF(S21&lt;300, 0, MIN(99, IF(S21&lt;500, S21*7%, IF(S21&lt;700, S21*12%, S21*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPhone 18  Pro  Magnetic Acrylic Case </t>
+          <t>iPhone 18  Pro  Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
@@ -1828,7 +2222,7 @@
       </c>
       <c r="E22" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPhone 18 Pro </t>
+          <t>iPhone 18 Pro</t>
         </is>
       </c>
       <c r="F22" s="3" t="inlineStr">
@@ -1836,7 +2230,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G22" s="2" t="inlineStr">
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1846,95 +2240,129 @@
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I22" s="3" t="inlineStr">
-        <is>
-          <t>74.55</t>
-        </is>
-      </c>
-      <c r="J22" s="3" t="inlineStr">
-        <is>
-          <t>9431</t>
-        </is>
-      </c>
-      <c r="K22" s="3" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L22" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01nhCNBb1MyspxgzA8C_!!2209951271504-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="I22" s="2" t="inlineStr"/>
+      <c r="J22" s="4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q22" s="4">
+        <f>SUM(J22:P22)</f>
+        <v/>
+      </c>
+      <c r="R22" s="4">
+        <f>IF(Q22&lt;300, Q22*1.4, IF(Q22&lt;400, Q22*1.33, Q22*1.25))</f>
+        <v/>
+      </c>
+      <c r="S22" s="5">
+        <f>INT(R22/100)*100 + IF(MOD(ROUND(R22,0),100)&lt;25, 0, IF(MOD(ROUND(R22,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T22" s="4">
+        <f>IF(S22&lt;300, 0, MIN(99, IF(S22&lt;500, S22*7%, IF(S22&lt;700, S22*12%, S22*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="4" t="inlineStr">
-        <is>
-          <t xml:space="preserve">iPhone 17 Pro Max Magnetic Acrylic Case </t>
-        </is>
-      </c>
-      <c r="B23" s="5" t="inlineStr">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>17PM-AC-M-O-N</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C23" s="7" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D23" s="7" t="inlineStr">
         <is>
           <t>Orange</t>
         </is>
       </c>
-      <c r="E23" s="5" t="inlineStr">
+      <c r="E23" s="7" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max</t>
         </is>
       </c>
-      <c r="F23" s="5" t="inlineStr">
+      <c r="F23" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H23" s="4" t="inlineStr">
+      <c r="H23" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I23" s="5" t="inlineStr">
-        <is>
-          <t>74.55</t>
-        </is>
-      </c>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>9962</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L23" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN013gBwfe1MyspxBvQ13_!!2209951271504-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M23" s="4" t="inlineStr"/>
+      <c r="I23" s="6" t="inlineStr"/>
+      <c r="J23" s="8" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q23" s="8">
+        <f>SUM(J23:P23)</f>
+        <v/>
+      </c>
+      <c r="R23" s="8">
+        <f>IF(Q23&lt;300, Q23*1.4, IF(Q23&lt;400, Q23*1.33, Q23*1.25))</f>
+        <v/>
+      </c>
+      <c r="S23" s="9">
+        <f>INT(R23/100)*100 + IF(MOD(ROUND(R23,0),100)&lt;25, 0, IF(MOD(ROUND(R23,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T23" s="8">
+        <f>IF(S23&lt;300, 0, MIN(99, IF(S23&lt;500, S23*7%, IF(S23&lt;700, S23*12%, S23*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPhone 17 Pro Max Magnetic Acrylic Case </t>
+          <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
@@ -1962,7 +2390,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G24" s="2" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -1972,90 +2400,124 @@
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I24" s="3" t="inlineStr">
-        <is>
-          <t>74.55</t>
-        </is>
-      </c>
-      <c r="J24" s="3" t="inlineStr">
-        <is>
-          <t>9981</t>
-        </is>
-      </c>
-      <c r="K24" s="3" t="inlineStr">
-        <is>
-          <t>0.035</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01MnsOtu1MyspxEDb37_!!2209951271504-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr"/>
+      <c r="I24" s="2" t="inlineStr"/>
+      <c r="J24" s="4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q24" s="4">
+        <f>SUM(J24:P24)</f>
+        <v/>
+      </c>
+      <c r="R24" s="4">
+        <f>IF(Q24&lt;300, Q24*1.4, IF(Q24&lt;400, Q24*1.33, Q24*1.25))</f>
+        <v/>
+      </c>
+      <c r="S24" s="5">
+        <f>INT(R24/100)*100 + IF(MOD(ROUND(R24,0),100)&lt;25, 0, IF(MOD(ROUND(R24,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T24" s="4">
+        <f>IF(S24&lt;300, 0, MIN(99, IF(S24&lt;500, S24*7%, IF(S24&lt;700, S24*12%, S24*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="25">
-      <c r="A25" s="4" t="inlineStr">
+      <c r="A25" s="6" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max Hard Shell Case with Lens Film</t>
         </is>
       </c>
-      <c r="B25" s="5" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>18PM-HS-S-N</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C25" s="7" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D25" s="7" t="inlineStr">
         <is>
           <t>Elegant Silver</t>
         </is>
       </c>
-      <c r="E25" s="5" t="inlineStr">
+      <c r="E25" s="7" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F25" s="5" t="inlineStr">
+      <c r="F25" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H25" s="4" t="inlineStr">
+      <c r="H25" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I25" s="5" t="inlineStr">
-        <is>
-          <t>102.28</t>
-        </is>
-      </c>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>4996</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L25" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01uOyImB1rBBtW8oevg_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M25" s="4" t="inlineStr"/>
+      <c r="I25" s="6" t="inlineStr"/>
+      <c r="J25" s="8" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L25" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O25" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P25" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q25" s="8">
+        <f>SUM(J25:P25)</f>
+        <v/>
+      </c>
+      <c r="R25" s="8">
+        <f>IF(Q25&lt;300, Q25*1.4, IF(Q25&lt;400, Q25*1.33, Q25*1.25))</f>
+        <v/>
+      </c>
+      <c r="S25" s="9">
+        <f>INT(R25/100)*100 + IF(MOD(ROUND(R25,0),100)&lt;25, 0, IF(MOD(ROUND(R25,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T25" s="8">
+        <f>IF(S25&lt;300, 0, MIN(99, IF(S25&lt;500, S25*7%, IF(S25&lt;700, S25*12%, S25*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2080,7 +2542,7 @@
       </c>
       <c r="E26" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPhone 18 Pro </t>
+          <t>iPhone 18 Pro</t>
         </is>
       </c>
       <c r="F26" s="3" t="inlineStr">
@@ -2088,7 +2550,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G26" s="2" t="inlineStr">
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -2098,90 +2560,124 @@
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I26" s="3" t="inlineStr">
-        <is>
-          <t>102.28</t>
-        </is>
-      </c>
-      <c r="J26" s="3" t="inlineStr">
-        <is>
-          <t>4996</t>
-        </is>
-      </c>
-      <c r="K26" s="3" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L26" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01uOyImB1rBBtW8oevg_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M26" s="2" t="inlineStr"/>
+      <c r="I26" s="2" t="inlineStr"/>
+      <c r="J26" s="4" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P26" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q26" s="4">
+        <f>SUM(J26:P26)</f>
+        <v/>
+      </c>
+      <c r="R26" s="4">
+        <f>IF(Q26&lt;300, Q26*1.4, IF(Q26&lt;400, Q26*1.33, Q26*1.25))</f>
+        <v/>
+      </c>
+      <c r="S26" s="5">
+        <f>INT(R26/100)*100 + IF(MOD(ROUND(R26,0),100)&lt;25, 0, IF(MOD(ROUND(R26,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T26" s="4">
+        <f>IF(S26&lt;300, 0, MIN(99, IF(S26&lt;500, S26*7%, IF(S26&lt;700, S26*12%, S26*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="27">
-      <c r="A27" s="4" t="inlineStr">
+      <c r="A27" s="6" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max Hard Shell Case with Lens Film</t>
         </is>
       </c>
-      <c r="B27" s="5" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>17PM-HS-S-N</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C27" s="7" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D27" s="7" t="inlineStr">
         <is>
           <t>Elegant Silver</t>
         </is>
       </c>
-      <c r="E27" s="5" t="inlineStr">
+      <c r="E27" s="7" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max</t>
         </is>
       </c>
-      <c r="F27" s="5" t="inlineStr">
+      <c r="F27" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G27" s="4" t="inlineStr">
+      <c r="G27" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H27" s="4" t="inlineStr">
+      <c r="H27" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I27" s="5" t="inlineStr">
-        <is>
-          <t>102.28</t>
-        </is>
-      </c>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>4998</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L27" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01uOyImB1rBBtW8oevg_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M27" s="4" t="inlineStr"/>
+      <c r="I27" s="6" t="inlineStr"/>
+      <c r="J27" s="8" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O27" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P27" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q27" s="8">
+        <f>SUM(J27:P27)</f>
+        <v/>
+      </c>
+      <c r="R27" s="8">
+        <f>IF(Q27&lt;300, Q27*1.4, IF(Q27&lt;400, Q27*1.33, Q27*1.25))</f>
+        <v/>
+      </c>
+      <c r="S27" s="9">
+        <f>INT(R27/100)*100 + IF(MOD(ROUND(R27,0),100)&lt;25, 0, IF(MOD(ROUND(R27,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T27" s="8">
+        <f>IF(S27&lt;300, 0, MIN(99, IF(S27&lt;500, S27*7%, IF(S27&lt;700, S27*12%, S27*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2206,7 +2702,7 @@
       </c>
       <c r="E28" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">iPhone 17 Pro </t>
+          <t>iPhone 17 Pro</t>
         </is>
       </c>
       <c r="F28" s="3" t="inlineStr">
@@ -2214,7 +2710,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G28" s="2" t="inlineStr">
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -2224,93 +2720,127 @@
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I28" s="3" t="inlineStr">
-        <is>
-          <t>102.28</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr">
-        <is>
-          <t>4998</t>
-        </is>
-      </c>
-      <c r="K28" s="3" t="inlineStr">
-        <is>
-          <t>0.04</t>
-        </is>
-      </c>
-      <c r="L28" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01uOyImB1rBBtW8oevg_!!2220284465592-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M28" s="2" t="inlineStr"/>
+      <c r="I28" s="2" t="inlineStr"/>
+      <c r="J28" s="4" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q28" s="4">
+        <f>SUM(J28:P28)</f>
+        <v/>
+      </c>
+      <c r="R28" s="4">
+        <f>IF(Q28&lt;300, Q28*1.4, IF(Q28&lt;400, Q28*1.33, Q28*1.25))</f>
+        <v/>
+      </c>
+      <c r="S28" s="5">
+        <f>INT(R28/100)*100 + IF(MOD(ROUND(R28,0),100)&lt;25, 0, IF(MOD(ROUND(R28,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T28" s="4">
+        <f>IF(S28&lt;300, 0, MIN(99, IF(S28&lt;500, S28*7%, IF(S28&lt;700, S28*12%, S28*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="29">
-      <c r="A29" s="4" t="inlineStr">
+      <c r="A29" s="6" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B29" s="5" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>RN8-SIL-WT-S</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D29" s="7" t="inlineStr">
         <is>
           <t>Antique White</t>
         </is>
       </c>
-      <c r="E29" s="5" t="inlineStr">
+      <c r="E29" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F29" s="5" t="inlineStr">
+      <c r="F29" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G29" s="4" t="inlineStr">
+      <c r="G29" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H29" s="4" t="inlineStr">
+      <c r="H29" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I29" s="5" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>9998</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L29" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01TNlHH71MfBnvHBAoS_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M29" s="4" t="inlineStr">
+      <c r="I29" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S.jpg</t>
         </is>
+      </c>
+      <c r="J29" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O29" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P29" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q29" s="8">
+        <f>SUM(J29:P29)</f>
+        <v/>
+      </c>
+      <c r="R29" s="8">
+        <f>IF(Q29&lt;300, Q29*1.4, IF(Q29&lt;400, Q29*1.33, Q29*1.25))</f>
+        <v/>
+      </c>
+      <c r="S29" s="9">
+        <f>INT(R29/100)*100 + IF(MOD(ROUND(R29,0),100)&lt;25, 0, IF(MOD(ROUND(R29,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T29" s="8">
+        <f>IF(S29&lt;300, 0, MIN(99, IF(S29&lt;500, S29*7%, IF(S29&lt;700, S29*12%, S29*15%))))</f>
+        <v/>
       </c>
     </row>
     <row r="30">
@@ -2344,7 +2874,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G30" s="2" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -2354,97 +2884,131 @@
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I30" s="3" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J30" s="3" t="inlineStr">
-        <is>
-          <t>9996</t>
-        </is>
-      </c>
-      <c r="K30" s="3" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L30" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01AKY4o41MfBnvIEHe1_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M30" s="2" t="inlineStr">
+      <c r="I30" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
       </c>
+      <c r="J30" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O30" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P30" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="4">
+        <f>SUM(J30:P30)</f>
+        <v/>
+      </c>
+      <c r="R30" s="4">
+        <f>IF(Q30&lt;300, Q30*1.4, IF(Q30&lt;400, Q30*1.33, Q30*1.25))</f>
+        <v/>
+      </c>
+      <c r="S30" s="5">
+        <f>INT(R30/100)*100 + IF(MOD(ROUND(R30,0),100)&lt;25, 0, IF(MOD(ROUND(R30,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T30" s="4">
+        <f>IF(S30&lt;300, 0, MIN(99, IF(S30&lt;500, S30*7%, IF(S30&lt;700, S30*12%, S30*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="31">
-      <c r="A31" s="4" t="inlineStr">
+      <c r="A31" s="6" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B31" s="5" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>RN8-SIL-GN-S</t>
         </is>
       </c>
-      <c r="C31" s="5" t="inlineStr">
+      <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D31" s="7" t="inlineStr">
         <is>
           <t>Dark Night Green</t>
         </is>
       </c>
-      <c r="E31" s="5" t="inlineStr">
+      <c r="E31" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F31" s="5" t="inlineStr">
+      <c r="F31" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H31" s="4" t="inlineStr">
+      <c r="H31" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I31" s="5" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="K31" s="5" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L31" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01AxiBJ81MfBnx6raHX_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M31" s="4" t="inlineStr">
+      <c r="I31" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S.jpg</t>
         </is>
+      </c>
+      <c r="J31" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K31" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L31" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M31" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N31" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O31" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P31" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="8">
+        <f>SUM(J31:P31)</f>
+        <v/>
+      </c>
+      <c r="R31" s="8">
+        <f>IF(Q31&lt;300, Q31*1.4, IF(Q31&lt;400, Q31*1.33, Q31*1.25))</f>
+        <v/>
+      </c>
+      <c r="S31" s="9">
+        <f>INT(R31/100)*100 + IF(MOD(ROUND(R31,0),100)&lt;25, 0, IF(MOD(ROUND(R31,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T31" s="8">
+        <f>IF(S31&lt;300, 0, MIN(99, IF(S31&lt;500, S31*7%, IF(S31&lt;700, S31*12%, S31*15%))))</f>
+        <v/>
       </c>
     </row>
     <row r="32">
@@ -2478,7 +3042,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G32" s="2" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -2488,97 +3052,131 @@
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I32" s="3" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J32" s="3" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="K32" s="3" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L32" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01PowUqU1MfBnvNoSsN_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M32" s="2" t="inlineStr">
+      <c r="I32" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S.jpg</t>
         </is>
       </c>
+      <c r="J32" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="4">
+        <f>SUM(J32:P32)</f>
+        <v/>
+      </c>
+      <c r="R32" s="4">
+        <f>IF(Q32&lt;300, Q32*1.4, IF(Q32&lt;400, Q32*1.33, Q32*1.25))</f>
+        <v/>
+      </c>
+      <c r="S32" s="5">
+        <f>INT(R32/100)*100 + IF(MOD(ROUND(R32,0),100)&lt;25, 0, IF(MOD(ROUND(R32,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T32" s="4">
+        <f>IF(S32&lt;300, 0, MIN(99, IF(S32&lt;500, S32*7%, IF(S32&lt;700, S32*12%, S32*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="33">
-      <c r="A33" s="4" t="inlineStr">
+      <c r="A33" s="6" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B33" s="5" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>RN8-SIL-BK-S</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D33" s="7" t="inlineStr">
         <is>
           <t>Classic Black</t>
         </is>
       </c>
-      <c r="E33" s="5" t="inlineStr">
+      <c r="E33" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F33" s="5" t="inlineStr">
+      <c r="F33" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H33" s="4" t="inlineStr">
+      <c r="H33" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I33" s="5" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>9996</t>
-        </is>
-      </c>
-      <c r="K33" s="5" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L33" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01HQAxzE1MfBnvVtrzk_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M33" s="4" t="inlineStr">
+      <c r="I33" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S.jpg</t>
         </is>
+      </c>
+      <c r="J33" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K33" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L33" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O33" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P33" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q33" s="8">
+        <f>SUM(J33:P33)</f>
+        <v/>
+      </c>
+      <c r="R33" s="8">
+        <f>IF(Q33&lt;300, Q33*1.4, IF(Q33&lt;400, Q33*1.33, Q33*1.25))</f>
+        <v/>
+      </c>
+      <c r="S33" s="9">
+        <f>INT(R33/100)*100 + IF(MOD(ROUND(R33,0),100)&lt;25, 0, IF(MOD(ROUND(R33,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T33" s="8">
+        <f>IF(S33&lt;300, 0, MIN(99, IF(S33&lt;500, S33*7%, IF(S33&lt;700, S33*12%, S33*15%))))</f>
+        <v/>
       </c>
     </row>
     <row r="34">
@@ -2612,7 +3210,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G34" s="2" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -2622,97 +3220,131 @@
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I34" s="3" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J34" s="3" t="inlineStr">
-        <is>
-          <t>10000</t>
-        </is>
-      </c>
-      <c r="K34" s="3" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01ld4Pco1MfBnvMZe4H_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
+      <c r="I34" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
       </c>
+      <c r="J34" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O34" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P34" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q34" s="4">
+        <f>SUM(J34:P34)</f>
+        <v/>
+      </c>
+      <c r="R34" s="4">
+        <f>IF(Q34&lt;300, Q34*1.4, IF(Q34&lt;400, Q34*1.33, Q34*1.25))</f>
+        <v/>
+      </c>
+      <c r="S34" s="5">
+        <f>INT(R34/100)*100 + IF(MOD(ROUND(R34,0),100)&lt;25, 0, IF(MOD(ROUND(R34,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T34" s="4">
+        <f>IF(S34&lt;300, 0, MIN(99, IF(S34&lt;500, S34*7%, IF(S34&lt;700, S34*12%, S34*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+      <c r="A35" s="6" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B35" s="5" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>RN8-SIL-RD-S</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C35" s="7" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D35" s="7" t="inlineStr">
         <is>
           <t>Camellia Red</t>
         </is>
       </c>
-      <c r="E35" s="5" t="inlineStr">
+      <c r="E35" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F35" s="5" t="inlineStr">
+      <c r="F35" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G35" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H35" s="4" t="inlineStr">
+      <c r="H35" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I35" s="5" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>9998</t>
-        </is>
-      </c>
-      <c r="K35" s="5" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L35" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN01jZ2ScP1MfBnvWMTkJ_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M35" s="4" t="inlineStr">
+      <c r="I35" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-RD-S.jpg</t>
         </is>
+      </c>
+      <c r="J35" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O35" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P35" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q35" s="8">
+        <f>SUM(J35:P35)</f>
+        <v/>
+      </c>
+      <c r="R35" s="8">
+        <f>IF(Q35&lt;300, Q35*1.4, IF(Q35&lt;400, Q35*1.33, Q35*1.25))</f>
+        <v/>
+      </c>
+      <c r="S35" s="9">
+        <f>INT(R35/100)*100 + IF(MOD(ROUND(R35,0),100)&lt;25, 0, IF(MOD(ROUND(R35,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T35" s="8">
+        <f>IF(S35&lt;300, 0, MIN(99, IF(S35&lt;500, S35*7%, IF(S35&lt;700, S35*12%, S35*15%))))</f>
+        <v/>
       </c>
     </row>
     <row r="36">
@@ -2746,7 +3378,7 @@
           <t>No</t>
         </is>
       </c>
-      <c r="G36" s="2" t="inlineStr">
+      <c r="G36" s="3" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
@@ -2756,97 +3388,131 @@
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I36" s="3" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J36" s="3" t="inlineStr">
-        <is>
-          <t>9999</t>
-        </is>
-      </c>
-      <c r="K36" s="3" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L36" s="2" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN014QYZ9C1MfBnvZ22Lo_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M36" s="2" t="inlineStr">
+      <c r="I36" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-TL-S.jpg</t>
         </is>
       </c>
+      <c r="J36" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O36" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P36" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q36" s="4">
+        <f>SUM(J36:P36)</f>
+        <v/>
+      </c>
+      <c r="R36" s="4">
+        <f>IF(Q36&lt;300, Q36*1.4, IF(Q36&lt;400, Q36*1.33, Q36*1.25))</f>
+        <v/>
+      </c>
+      <c r="S36" s="5">
+        <f>INT(R36/100)*100 + IF(MOD(ROUND(R36,0),100)&lt;25, 0, IF(MOD(ROUND(R36,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T36" s="4">
+        <f>IF(S36&lt;300, 0, MIN(99, IF(S36&lt;500, S36*7%, IF(S36&lt;700, S36*12%, S36*15%))))</f>
+        <v/>
+      </c>
     </row>
     <row r="37">
-      <c r="A37" s="4" t="inlineStr">
+      <c r="A37" s="6" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B37" s="5" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>RN8-SIL-CL-C</t>
         </is>
       </c>
-      <c r="C37" s="5" t="inlineStr">
+      <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D37" s="5" t="inlineStr">
+      <c r="D37" s="7" t="inlineStr">
         <is>
           <t>Transparent</t>
         </is>
       </c>
-      <c r="E37" s="5" t="inlineStr">
+      <c r="E37" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F37" s="5" t="inlineStr">
+      <c r="F37" s="7" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="G37" s="4" t="inlineStr">
+      <c r="G37" s="7" t="inlineStr">
         <is>
           <t>Link</t>
         </is>
       </c>
-      <c r="H37" s="4" t="inlineStr">
+      <c r="H37" s="6" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I37" s="5" t="inlineStr">
-        <is>
-          <t>34.09</t>
-        </is>
-      </c>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>9993</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr">
-        <is>
-          <t>0.03</t>
-        </is>
-      </c>
-      <c r="L37" s="4" t="inlineStr">
-        <is>
-          <t>https://cbu01.alicdn.com/img/ibank/O1CN016Xira71MfBnvVuk5t_!!2222442441461-0-cib.jpg</t>
-        </is>
-      </c>
-      <c r="M37" s="4" t="inlineStr">
+      <c r="I37" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-CL-C.jpg</t>
         </is>
+      </c>
+      <c r="J37" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O37" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P37" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q37" s="8">
+        <f>SUM(J37:P37)</f>
+        <v/>
+      </c>
+      <c r="R37" s="8">
+        <f>IF(Q37&lt;300, Q37*1.4, IF(Q37&lt;400, Q37*1.33, Q37*1.25))</f>
+        <v/>
+      </c>
+      <c r="S37" s="9">
+        <f>INT(R37/100)*100 + IF(MOD(ROUND(R37,0),100)&lt;25, 0, IF(MOD(ROUND(R37,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T37" s="8">
+        <f>IF(S37&lt;300, 0, MIN(99, IF(S37&lt;500, S37*7%, IF(S37&lt;700, S37*12%, S37*15%))))</f>
+        <v/>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat: sync inventory.xlsx and automate Excel update and Git push after product processing
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T37"/>
+  <dimension ref="A1:T39"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -645,26 +645,40 @@
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="4" t="n">
-        <v>133</v>
-      </c>
-      <c r="K2" s="4" t="n">
-        <v>11.7</v>
-      </c>
-      <c r="L2" s="4" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="M2" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N2" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O2" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P2" s="4" t="n">
-        <v>0</v>
+      <c r="J2" s="4" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K2" s="4" t="inlineStr">
+        <is>
+          <t>11.7</t>
+        </is>
+      </c>
+      <c r="L2" s="4" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="M2" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N2" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O2" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P2" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q2" s="4">
         <f>SUM(J2:P2)</f>
@@ -725,26 +739,40 @@
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="8" t="n">
-        <v>345.8</v>
-      </c>
-      <c r="K3" s="8" t="n">
-        <v>24.61</v>
-      </c>
-      <c r="L3" s="8" t="n">
-        <v>35.01</v>
-      </c>
-      <c r="M3" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N3" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O3" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P3" s="8" t="n">
-        <v>0</v>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>345.8</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>24.61</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>35.01</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O3" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q3" s="8">
         <f>SUM(J3:P3)</f>
@@ -805,26 +833,40 @@
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="4" t="n">
-        <v>345.8</v>
-      </c>
-      <c r="K4" s="4" t="n">
-        <v>24.61</v>
-      </c>
-      <c r="L4" s="4" t="n">
-        <v>35.01</v>
-      </c>
-      <c r="M4" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N4" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O4" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P4" s="4" t="n">
-        <v>0</v>
+      <c r="J4" s="4" t="inlineStr">
+        <is>
+          <t>345.8</t>
+        </is>
+      </c>
+      <c r="K4" s="4" t="inlineStr">
+        <is>
+          <t>24.61</t>
+        </is>
+      </c>
+      <c r="L4" s="4" t="inlineStr">
+        <is>
+          <t>35.01</t>
+        </is>
+      </c>
+      <c r="M4" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N4" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O4" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P4" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q4" s="4">
         <f>SUM(J4:P4)</f>
@@ -885,26 +927,40 @@
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="8" t="n">
-        <v>159.6</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="L5" s="8" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="M5" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N5" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O5" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P5" s="8" t="n">
-        <v>0</v>
+      <c r="J5" s="8" t="inlineStr">
+        <is>
+          <t>159.6</t>
+        </is>
+      </c>
+      <c r="K5" s="8" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="L5" s="8" t="inlineStr">
+        <is>
+          <t>51.2</t>
+        </is>
+      </c>
+      <c r="M5" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N5" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O5" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P5" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q5" s="8">
         <f>SUM(J5:P5)</f>
@@ -965,26 +1021,40 @@
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="4" t="n">
-        <v>159.6</v>
-      </c>
-      <c r="K6" s="4" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="L6" s="4" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="M6" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N6" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O6" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P6" s="4" t="n">
-        <v>0</v>
+      <c r="J6" s="4" t="inlineStr">
+        <is>
+          <t>159.6</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="L6" s="4" t="inlineStr">
+        <is>
+          <t>51.2</t>
+        </is>
+      </c>
+      <c r="M6" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N6" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O6" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P6" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q6" s="4">
         <f>SUM(J6:P6)</f>
@@ -1045,26 +1115,40 @@
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="8" t="n">
-        <v>159.6</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="L7" s="8" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="M7" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N7" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O7" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P7" s="8" t="n">
-        <v>0</v>
+      <c r="J7" s="8" t="inlineStr">
+        <is>
+          <t>159.6</t>
+        </is>
+      </c>
+      <c r="K7" s="8" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="L7" s="8" t="inlineStr">
+        <is>
+          <t>51.2</t>
+        </is>
+      </c>
+      <c r="M7" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N7" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O7" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P7" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q7" s="8">
         <f>SUM(J7:P7)</f>
@@ -1125,26 +1209,40 @@
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="4" t="n">
-        <v>159.6</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="L8" s="4" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="M8" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O8" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P8" s="4" t="n">
-        <v>0</v>
+      <c r="J8" s="4" t="inlineStr">
+        <is>
+          <t>159.6</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="L8" s="4" t="inlineStr">
+        <is>
+          <t>51.2</t>
+        </is>
+      </c>
+      <c r="M8" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N8" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O8" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P8" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q8" s="4">
         <f>SUM(J8:P8)</f>
@@ -1201,26 +1299,40 @@
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="8" t="n">
-        <v>159.6</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>2.66</v>
-      </c>
-      <c r="L9" s="8" t="n">
-        <v>51.2</v>
-      </c>
-      <c r="M9" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N9" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O9" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P9" s="8" t="n">
-        <v>0</v>
+      <c r="J9" s="8" t="inlineStr">
+        <is>
+          <t>159.6</t>
+        </is>
+      </c>
+      <c r="K9" s="8" t="inlineStr">
+        <is>
+          <t>2.66</t>
+        </is>
+      </c>
+      <c r="L9" s="8" t="inlineStr">
+        <is>
+          <t>51.2</t>
+        </is>
+      </c>
+      <c r="M9" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N9" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O9" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P9" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q9" s="8">
         <f>SUM(J9:P9)</f>
@@ -1281,26 +1393,40 @@
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="4" t="n">
-        <v>106.4</v>
-      </c>
-      <c r="K10" s="4" t="n">
-        <v>9.039999999999999</v>
-      </c>
-      <c r="L10" s="4" t="n">
-        <v>54.6</v>
-      </c>
-      <c r="M10" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N10" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O10" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P10" s="4" t="n">
-        <v>0</v>
+      <c r="J10" s="4" t="inlineStr">
+        <is>
+          <t>106.4</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>9.04</t>
+        </is>
+      </c>
+      <c r="L10" s="4" t="inlineStr">
+        <is>
+          <t>54.6</t>
+        </is>
+      </c>
+      <c r="M10" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N10" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O10" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P10" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q10" s="4">
         <f>SUM(J10:P10)</f>
@@ -1361,26 +1487,40 @@
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="8" t="n">
-        <v>133</v>
-      </c>
-      <c r="K11" s="8" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="L11" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="M11" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O11" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P11" s="8" t="n">
-        <v>0</v>
+      <c r="J11" s="8" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K11" s="8" t="inlineStr">
+        <is>
+          <t>11.44</t>
+        </is>
+      </c>
+      <c r="L11" s="8" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="M11" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N11" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O11" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P11" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q11" s="8">
         <f>SUM(J11:P11)</f>
@@ -1441,26 +1581,40 @@
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="4" t="n">
-        <v>133</v>
-      </c>
-      <c r="K12" s="4" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="L12" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="M12" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N12" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O12" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P12" s="4" t="n">
-        <v>0</v>
+      <c r="J12" s="4" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>11.44</t>
+        </is>
+      </c>
+      <c r="L12" s="4" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="M12" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N12" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O12" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P12" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q12" s="4">
         <f>SUM(J12:P12)</f>
@@ -1521,26 +1675,40 @@
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="8" t="n">
-        <v>133</v>
-      </c>
-      <c r="K13" s="8" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="L13" s="8" t="n">
-        <v>56</v>
-      </c>
-      <c r="M13" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N13" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O13" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P13" s="8" t="n">
-        <v>0</v>
+      <c r="J13" s="8" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K13" s="8" t="inlineStr">
+        <is>
+          <t>11.44</t>
+        </is>
+      </c>
+      <c r="L13" s="8" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="M13" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N13" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O13" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P13" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q13" s="8">
         <f>SUM(J13:P13)</f>
@@ -1601,26 +1769,40 @@
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="4" t="n">
-        <v>133</v>
-      </c>
-      <c r="K14" s="4" t="n">
-        <v>11.44</v>
-      </c>
-      <c r="L14" s="4" t="n">
-        <v>56</v>
-      </c>
-      <c r="M14" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N14" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O14" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P14" s="4" t="n">
-        <v>0</v>
+      <c r="J14" s="4" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>11.44</t>
+        </is>
+      </c>
+      <c r="L14" s="4" t="inlineStr">
+        <is>
+          <t>56.0</t>
+        </is>
+      </c>
+      <c r="M14" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N14" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O14" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P14" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q14" s="4">
         <f>SUM(J14:P14)</f>
@@ -1681,26 +1863,40 @@
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="8" t="n">
-        <v>146.3</v>
-      </c>
-      <c r="K15" s="8" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="L15" s="8" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="M15" s="8" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N15" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O15" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P15" s="8" t="n">
-        <v>0</v>
+      <c r="J15" s="8" t="inlineStr">
+        <is>
+          <t>146.3</t>
+        </is>
+      </c>
+      <c r="K15" s="8" t="inlineStr">
+        <is>
+          <t>79.8</t>
+        </is>
+      </c>
+      <c r="L15" s="8" t="inlineStr">
+        <is>
+          <t>87.5</t>
+        </is>
+      </c>
+      <c r="M15" s="8" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N15" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O15" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P15" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q15" s="8">
         <f>SUM(J15:P15)</f>
@@ -1761,26 +1957,40 @@
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="4" t="n">
-        <v>146.3</v>
-      </c>
-      <c r="K16" s="4" t="n">
-        <v>79.8</v>
-      </c>
-      <c r="L16" s="4" t="n">
-        <v>87.5</v>
-      </c>
-      <c r="M16" s="4" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N16" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O16" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P16" s="4" t="n">
-        <v>0</v>
+      <c r="J16" s="4" t="inlineStr">
+        <is>
+          <t>146.3</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>79.8</t>
+        </is>
+      </c>
+      <c r="L16" s="4" t="inlineStr">
+        <is>
+          <t>87.5</t>
+        </is>
+      </c>
+      <c r="M16" s="4" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N16" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O16" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P16" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q16" s="4">
         <f>SUM(J16:P16)</f>
@@ -1841,26 +2051,40 @@
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="8" t="n">
-        <v>252.7</v>
-      </c>
-      <c r="K17" s="8" t="n">
-        <v>18.09</v>
-      </c>
-      <c r="L17" s="8" t="n">
-        <v>35</v>
-      </c>
-      <c r="M17" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N17" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O17" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P17" s="8" t="n">
-        <v>0</v>
+      <c r="J17" s="8" t="inlineStr">
+        <is>
+          <t>252.7</t>
+        </is>
+      </c>
+      <c r="K17" s="8" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
+      <c r="L17" s="8" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="M17" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N17" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O17" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P17" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q17" s="8">
         <f>SUM(J17:P17)</f>
@@ -1921,26 +2145,40 @@
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="4" t="n">
-        <v>252.7</v>
-      </c>
-      <c r="K18" s="4" t="n">
-        <v>18.09</v>
-      </c>
-      <c r="L18" s="4" t="n">
-        <v>35</v>
-      </c>
-      <c r="M18" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N18" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O18" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P18" s="4" t="n">
-        <v>0</v>
+      <c r="J18" s="4" t="inlineStr">
+        <is>
+          <t>252.7</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>18.09</t>
+        </is>
+      </c>
+      <c r="L18" s="4" t="inlineStr">
+        <is>
+          <t>35.0</t>
+        </is>
+      </c>
+      <c r="M18" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N18" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O18" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P18" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q18" s="4">
         <f>SUM(J18:P18)</f>
@@ -2001,26 +2239,40 @@
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="8" t="n">
-        <v>265.74</v>
-      </c>
-      <c r="K19" s="8" t="n">
-        <v>50.2</v>
-      </c>
-      <c r="L19" s="8" t="n">
-        <v>80</v>
-      </c>
-      <c r="M19" s="8" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N19" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O19" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P19" s="8" t="n">
-        <v>0</v>
+      <c r="J19" s="8" t="inlineStr">
+        <is>
+          <t>265.74</t>
+        </is>
+      </c>
+      <c r="K19" s="8" t="inlineStr">
+        <is>
+          <t>50.2</t>
+        </is>
+      </c>
+      <c r="L19" s="8" t="inlineStr">
+        <is>
+          <t>80.0</t>
+        </is>
+      </c>
+      <c r="M19" s="8" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N19" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O19" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P19" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q19" s="8">
         <f>SUM(J19:P19)</f>
@@ -2081,26 +2333,40 @@
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="4" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="K20" s="4" t="n">
-        <v>16.55</v>
-      </c>
-      <c r="L20" s="4" t="n">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="M20" s="4" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N20" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O20" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P20" s="4" t="n">
-        <v>0</v>
+      <c r="J20" s="4" t="inlineStr">
+        <is>
+          <t>87.25</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>16.55</t>
+        </is>
+      </c>
+      <c r="L20" s="4" t="inlineStr">
+        <is>
+          <t>81.6</t>
+        </is>
+      </c>
+      <c r="M20" s="4" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N20" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O20" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P20" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q20" s="4">
         <f>SUM(J20:P20)</f>
@@ -2161,26 +2427,40 @@
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="8" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="K21" s="8" t="n">
-        <v>16.55</v>
-      </c>
-      <c r="L21" s="8" t="n">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="M21" s="8" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N21" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O21" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P21" s="8" t="n">
-        <v>0</v>
+      <c r="J21" s="8" t="inlineStr">
+        <is>
+          <t>87.25</t>
+        </is>
+      </c>
+      <c r="K21" s="8" t="inlineStr">
+        <is>
+          <t>16.55</t>
+        </is>
+      </c>
+      <c r="L21" s="8" t="inlineStr">
+        <is>
+          <t>81.6</t>
+        </is>
+      </c>
+      <c r="M21" s="8" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N21" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O21" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P21" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q21" s="8">
         <f>SUM(J21:P21)</f>
@@ -2241,26 +2521,40 @@
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="4" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="K22" s="4" t="n">
-        <v>16.55</v>
-      </c>
-      <c r="L22" s="4" t="n">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="M22" s="4" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N22" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O22" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P22" s="4" t="n">
-        <v>0</v>
+      <c r="J22" s="4" t="inlineStr">
+        <is>
+          <t>87.25</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>16.55</t>
+        </is>
+      </c>
+      <c r="L22" s="4" t="inlineStr">
+        <is>
+          <t>81.6</t>
+        </is>
+      </c>
+      <c r="M22" s="4" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N22" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O22" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P22" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q22" s="4">
         <f>SUM(J22:P22)</f>
@@ -2321,26 +2615,40 @@
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
-      <c r="J23" s="8" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="K23" s="8" t="n">
-        <v>16.55</v>
-      </c>
-      <c r="L23" s="8" t="n">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="M23" s="8" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N23" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O23" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P23" s="8" t="n">
-        <v>0</v>
+      <c r="J23" s="8" t="inlineStr">
+        <is>
+          <t>87.25</t>
+        </is>
+      </c>
+      <c r="K23" s="8" t="inlineStr">
+        <is>
+          <t>16.55</t>
+        </is>
+      </c>
+      <c r="L23" s="8" t="inlineStr">
+        <is>
+          <t>81.6</t>
+        </is>
+      </c>
+      <c r="M23" s="8" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N23" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O23" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P23" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q23" s="8">
         <f>SUM(J23:P23)</f>
@@ -2401,26 +2709,40 @@
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="4" t="n">
-        <v>87.25</v>
-      </c>
-      <c r="K24" s="4" t="n">
-        <v>16.55</v>
-      </c>
-      <c r="L24" s="4" t="n">
-        <v>81.59999999999999</v>
-      </c>
-      <c r="M24" s="4" t="n">
-        <v>5.09</v>
-      </c>
-      <c r="N24" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O24" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P24" s="4" t="n">
-        <v>0</v>
+      <c r="J24" s="4" t="inlineStr">
+        <is>
+          <t>87.25</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>16.55</t>
+        </is>
+      </c>
+      <c r="L24" s="4" t="inlineStr">
+        <is>
+          <t>81.6</t>
+        </is>
+      </c>
+      <c r="M24" s="4" t="inlineStr">
+        <is>
+          <t>5.09</t>
+        </is>
+      </c>
+      <c r="N24" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O24" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P24" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q24" s="4">
         <f>SUM(J24:P24)</f>
@@ -2481,26 +2803,40 @@
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
-      <c r="J25" s="8" t="n">
-        <v>119.7</v>
-      </c>
-      <c r="K25" s="8" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="L25" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="M25" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N25" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O25" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P25" s="8" t="n">
-        <v>0</v>
+      <c r="J25" s="8" t="inlineStr">
+        <is>
+          <t>119.7</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+      <c r="L25" s="8" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="M25" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N25" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O25" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P25" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q25" s="8">
         <f>SUM(J25:P25)</f>
@@ -2561,26 +2897,40 @@
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="4" t="n">
-        <v>119.7</v>
-      </c>
-      <c r="K26" s="4" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="L26" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="M26" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N26" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O26" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P26" s="4" t="n">
-        <v>0</v>
+      <c r="J26" s="4" t="inlineStr">
+        <is>
+          <t>119.7</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+      <c r="L26" s="4" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="M26" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N26" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O26" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P26" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q26" s="4">
         <f>SUM(J26:P26)</f>
@@ -2641,26 +2991,40 @@
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
-      <c r="J27" s="8" t="n">
-        <v>119.7</v>
-      </c>
-      <c r="K27" s="8" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="L27" s="8" t="n">
-        <v>38</v>
-      </c>
-      <c r="M27" s="8" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N27" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O27" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P27" s="8" t="n">
-        <v>0</v>
+      <c r="J27" s="8" t="inlineStr">
+        <is>
+          <t>119.7</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+      <c r="L27" s="8" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="M27" s="8" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N27" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O27" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P27" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q27" s="8">
         <f>SUM(J27:P27)</f>
@@ -2721,26 +3085,40 @@
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="4" t="n">
-        <v>119.7</v>
-      </c>
-      <c r="K28" s="4" t="n">
-        <v>8.75</v>
-      </c>
-      <c r="L28" s="4" t="n">
-        <v>38</v>
-      </c>
-      <c r="M28" s="4" t="n">
-        <v>2.54</v>
-      </c>
-      <c r="N28" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O28" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P28" s="4" t="n">
-        <v>0</v>
+      <c r="J28" s="4" t="inlineStr">
+        <is>
+          <t>119.7</t>
+        </is>
+      </c>
+      <c r="K28" s="4" t="inlineStr">
+        <is>
+          <t>8.75</t>
+        </is>
+      </c>
+      <c r="L28" s="4" t="inlineStr">
+        <is>
+          <t>38.0</t>
+        </is>
+      </c>
+      <c r="M28" s="4" t="inlineStr">
+        <is>
+          <t>2.54</t>
+        </is>
+      </c>
+      <c r="N28" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O28" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P28" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q28" s="4">
         <f>SUM(J28:P28)</f>
@@ -2805,26 +3183,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S.jpg</t>
         </is>
       </c>
-      <c r="J29" s="8" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K29" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="L29" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M29" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N29" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O29" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P29" s="8" t="n">
-        <v>0</v>
+      <c r="J29" s="8" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K29" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L29" s="8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M29" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N29" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O29" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P29" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q29" s="8">
         <f>SUM(J29:P29)</f>
@@ -2889,26 +3281,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
       </c>
-      <c r="J30" s="4" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K30" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L30" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M30" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N30" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O30" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P30" s="4" t="n">
-        <v>0</v>
+      <c r="J30" s="4" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K30" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L30" s="4" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M30" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N30" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O30" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P30" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q30" s="4">
         <f>SUM(J30:P30)</f>
@@ -2973,26 +3379,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S.jpg</t>
         </is>
       </c>
-      <c r="J31" s="8" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K31" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="L31" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M31" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N31" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O31" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P31" s="8" t="n">
-        <v>0</v>
+      <c r="J31" s="8" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K31" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L31" s="8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M31" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N31" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O31" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P31" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q31" s="8">
         <f>SUM(J31:P31)</f>
@@ -3057,26 +3477,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S.jpg</t>
         </is>
       </c>
-      <c r="J32" s="4" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K32" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L32" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M32" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N32" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O32" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P32" s="4" t="n">
-        <v>0</v>
+      <c r="J32" s="4" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K32" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L32" s="4" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M32" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N32" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O32" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P32" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q32" s="4">
         <f>SUM(J32:P32)</f>
@@ -3141,26 +3575,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S.jpg</t>
         </is>
       </c>
-      <c r="J33" s="8" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K33" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="L33" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M33" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N33" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O33" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P33" s="8" t="n">
-        <v>0</v>
+      <c r="J33" s="8" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K33" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L33" s="8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M33" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N33" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O33" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P33" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q33" s="8">
         <f>SUM(J33:P33)</f>
@@ -3225,26 +3673,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
       </c>
-      <c r="J34" s="4" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K34" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L34" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M34" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N34" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O34" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P34" s="4" t="n">
-        <v>0</v>
+      <c r="J34" s="4" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K34" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L34" s="4" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M34" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N34" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O34" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P34" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q34" s="4">
         <f>SUM(J34:P34)</f>
@@ -3309,26 +3771,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-RD-S.jpg</t>
         </is>
       </c>
-      <c r="J35" s="8" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K35" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="L35" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M35" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N35" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O35" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P35" s="8" t="n">
-        <v>0</v>
+      <c r="J35" s="8" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K35" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L35" s="8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M35" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N35" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O35" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P35" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q35" s="8">
         <f>SUM(J35:P35)</f>
@@ -3393,26 +3869,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-TL-S.jpg</t>
         </is>
       </c>
-      <c r="J36" s="4" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K36" s="4" t="n">
-        <v>10</v>
-      </c>
-      <c r="L36" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M36" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N36" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O36" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P36" s="4" t="n">
-        <v>0</v>
+      <c r="J36" s="4" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K36" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L36" s="4" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M36" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N36" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O36" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P36" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q36" s="4">
         <f>SUM(J36:P36)</f>
@@ -3477,26 +3967,40 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-CL-C.jpg</t>
         </is>
       </c>
-      <c r="J37" s="8" t="n">
-        <v>39.9</v>
-      </c>
-      <c r="K37" s="8" t="n">
-        <v>10</v>
-      </c>
-      <c r="L37" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M37" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N37" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O37" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P37" s="8" t="n">
-        <v>0</v>
+      <c r="J37" s="8" t="inlineStr">
+        <is>
+          <t>39.9</t>
+        </is>
+      </c>
+      <c r="K37" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L37" s="8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M37" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N37" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O37" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P37" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q37" s="8">
         <f>SUM(J37:P37)</f>
@@ -3512,6 +4016,202 @@
       </c>
       <c r="T37" s="8">
         <f>IF(S37&lt;300, 0, MIN(99, IF(S37&lt;500, S37*7%, IF(S37&lt;700, S37*12%, S37*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>RN8-TPU-WT-M</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>Transparent White</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H38" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
+        </is>
+      </c>
+      <c r="I38" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8/TPU/sku/RN8-TPU-WT-M.jpg</t>
+        </is>
+      </c>
+      <c r="J38" s="4" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K38" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L38" s="4" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M38" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N38" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O38" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P38" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="Q38" s="4">
+        <f>SUM(J38:P38)</f>
+        <v/>
+      </c>
+      <c r="R38" s="4">
+        <f>IF(Q38&lt;300, Q38*1.4, IF(Q38&lt;400, Q38*1.33, Q38*1.25))</f>
+        <v/>
+      </c>
+      <c r="S38" s="5">
+        <f>INT(R38/100)*100 + IF(MOD(ROUND(R38,0),100)&lt;25, 0, IF(MOD(ROUND(R38,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T38" s="4">
+        <f>IF(S38&lt;300, 0, MIN(99, IF(S38&lt;500, S38*7%, IF(S38&lt;700, S38*12%, S38*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>RN8-TPU-BK-M</t>
+        </is>
+      </c>
+      <c r="C39" s="7" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D39" s="7" t="inlineStr">
+        <is>
+          <t>Transparent Black</t>
+        </is>
+      </c>
+      <c r="E39" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F39" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H39" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
+        </is>
+      </c>
+      <c r="I39" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8/TPU/sku/RN8-TPU-BK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J39" s="8" t="inlineStr">
+        <is>
+          <t>133.0</t>
+        </is>
+      </c>
+      <c r="K39" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
+      </c>
+      <c r="L39" s="8" t="inlineStr">
+        <is>
+          <t>50.0</t>
+        </is>
+      </c>
+      <c r="M39" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N39" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O39" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P39" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
+      </c>
+      <c r="Q39" s="8">
+        <f>SUM(J39:P39)</f>
+        <v/>
+      </c>
+      <c r="R39" s="8">
+        <f>IF(Q39&lt;300, Q39*1.4, IF(Q39&lt;400, Q39*1.33, Q39*1.25))</f>
+        <v/>
+      </c>
+      <c r="S39" s="9">
+        <f>INT(R39/100)*100 + IF(MOD(ROUND(R39,0),100)&lt;25, 0, IF(MOD(ROUND(R39,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T39" s="8">
+        <f>IF(S39&lt;300, 0, MIN(99, IF(S39&lt;500, S39*7%, IF(S39&lt;700, S39*12%, S39*15%))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: process Honor 600 lite (Silicone) and update inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,13 +476,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T39"/>
+  <dimension ref="A1:T43"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="37" customWidth="1" min="4" max="4"/>
+    <col width="45" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -4215,6 +4215,342 @@
         <v/>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>H600L-SIL-BK-M</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>Built-In Magnetic Suction - Moiré Black</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>Honor 600 lite</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H40" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
+        </is>
+      </c>
+      <c r="I40" s="2" t="inlineStr">
+        <is>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-BK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J40" s="4" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L40" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M40" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O40" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P40" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q40" s="4">
+        <f>SUM(J40:P40)</f>
+        <v/>
+      </c>
+      <c r="R40" s="4">
+        <f>IF(Q40&lt;300, Q40*1.4, IF(Q40&lt;400, Q40*1.33, Q40*1.25))</f>
+        <v/>
+      </c>
+      <c r="S40" s="5">
+        <f>INT(R40/100)*100 + IF(MOD(ROUND(R40,0),100)&lt;25, 0, IF(MOD(ROUND(R40,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T40" s="4">
+        <f>IF(S40&lt;300, 0, MIN(99, IF(S40&lt;500, S40*7%, IF(S40&lt;700, S40*12%, S40*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>H600L-SIL-BL-M</t>
+        </is>
+      </c>
+      <c r="C41" s="7" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="D41" s="7" t="inlineStr">
+        <is>
+          <t>Built-In Magnetic Suction-Gentleman Blue</t>
+        </is>
+      </c>
+      <c r="E41" s="7" t="inlineStr">
+        <is>
+          <t>Honor 600 lite</t>
+        </is>
+      </c>
+      <c r="F41" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H41" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
+        </is>
+      </c>
+      <c r="I41" s="6" t="inlineStr">
+        <is>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-BL-M.jpg</t>
+        </is>
+      </c>
+      <c r="J41" s="8" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K41" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L41" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M41" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N41" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O41" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P41" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q41" s="8">
+        <f>SUM(J41:P41)</f>
+        <v/>
+      </c>
+      <c r="R41" s="8">
+        <f>IF(Q41&lt;300, Q41*1.4, IF(Q41&lt;400, Q41*1.33, Q41*1.25))</f>
+        <v/>
+      </c>
+      <c r="S41" s="9">
+        <f>INT(R41/100)*100 + IF(MOD(ROUND(R41,0),100)&lt;25, 0, IF(MOD(ROUND(R41,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T41" s="8">
+        <f>IF(S41&lt;300, 0, MIN(99, IF(S41&lt;500, S41*7%, IF(S41&lt;700, S41*12%, S41*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>H600L-SIL-GN-M</t>
+        </is>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>Built-In Magnetic Suction-Dark Night Green</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="inlineStr">
+        <is>
+          <t>Honor 600 lite</t>
+        </is>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H42" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
+        </is>
+      </c>
+      <c r="I42" s="2" t="inlineStr">
+        <is>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-GN-M.jpg</t>
+        </is>
+      </c>
+      <c r="J42" s="4" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L42" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M42" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O42" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P42" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q42" s="4">
+        <f>SUM(J42:P42)</f>
+        <v/>
+      </c>
+      <c r="R42" s="4">
+        <f>IF(Q42&lt;300, Q42*1.4, IF(Q42&lt;400, Q42*1.33, Q42*1.25))</f>
+        <v/>
+      </c>
+      <c r="S42" s="5">
+        <f>INT(R42/100)*100 + IF(MOD(ROUND(R42,0),100)&lt;25, 0, IF(MOD(ROUND(R42,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T42" s="4">
+        <f>IF(S42&lt;300, 0, MIN(99, IF(S42&lt;500, S42*7%, IF(S42&lt;700, S42*12%, S42*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>H600L-SIL-RD-M</t>
+        </is>
+      </c>
+      <c r="C43" s="7" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="D43" s="7" t="inlineStr">
+        <is>
+          <t>Built-In Magnetic Suction-Charming Red</t>
+        </is>
+      </c>
+      <c r="E43" s="7" t="inlineStr">
+        <is>
+          <t>Honor 600 lite</t>
+        </is>
+      </c>
+      <c r="F43" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G43" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H43" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
+        </is>
+      </c>
+      <c r="I43" s="6" t="inlineStr">
+        <is>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-RD-M.jpg</t>
+        </is>
+      </c>
+      <c r="J43" s="8" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K43" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L43" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M43" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N43" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O43" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P43" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q43" s="8">
+        <f>SUM(J43:P43)</f>
+        <v/>
+      </c>
+      <c r="R43" s="8">
+        <f>IF(Q43&lt;300, Q43*1.4, IF(Q43&lt;400, Q43*1.33, Q43*1.25))</f>
+        <v/>
+      </c>
+      <c r="S43" s="9">
+        <f>INT(R43/100)*100 + IF(MOD(ROUND(R43,0),100)&lt;25, 0, IF(MOD(ROUND(R43,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T43" s="8">
+        <f>IF(S43&lt;300, 0, MIN(99, IF(S43&lt;500, S43*7%, IF(S43&lt;700, S43*12%, S43*15%))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: refine Honor 600 lite translated badges and update weight-based air shipping in inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -482,7 +482,7 @@
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
-    <col width="45" customWidth="1" min="4" max="4"/>
+    <col width="37" customWidth="1" min="4" max="4"/>
     <col width="27" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
@@ -4233,7 +4233,7 @@
       </c>
       <c r="D40" s="3" t="inlineStr">
         <is>
-          <t>Built-In Magnetic Suction - Moiré Black</t>
+          <t>Moiré Black</t>
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr">
@@ -4261,26 +4261,38 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-BK-M.jpg</t>
         </is>
       </c>
-      <c r="J40" s="4" t="n">
-        <v>186.2</v>
-      </c>
-      <c r="K40" s="4" t="n">
-        <v>10</v>
+      <c r="J40" s="4" t="inlineStr">
+        <is>
+          <t>186.2</t>
+        </is>
+      </c>
+      <c r="K40" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
       </c>
       <c r="L40" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M40" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N40" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O40" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P40" s="4" t="n">
-        <v>0</v>
+        <v>156</v>
+      </c>
+      <c r="M40" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N40" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O40" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P40" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q40" s="4">
         <f>SUM(J40:P40)</f>
@@ -4317,7 +4329,7 @@
       </c>
       <c r="D41" s="7" t="inlineStr">
         <is>
-          <t>Built-In Magnetic Suction-Gentleman Blue</t>
+          <t>Gentleman Blue</t>
         </is>
       </c>
       <c r="E41" s="7" t="inlineStr">
@@ -4345,26 +4357,38 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-BL-M.jpg</t>
         </is>
       </c>
-      <c r="J41" s="8" t="n">
-        <v>186.2</v>
-      </c>
-      <c r="K41" s="8" t="n">
-        <v>10</v>
+      <c r="J41" s="8" t="inlineStr">
+        <is>
+          <t>186.2</t>
+        </is>
+      </c>
+      <c r="K41" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
       </c>
       <c r="L41" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M41" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N41" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O41" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P41" s="8" t="n">
-        <v>0</v>
+        <v>156</v>
+      </c>
+      <c r="M41" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N41" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O41" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P41" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q41" s="8">
         <f>SUM(J41:P41)</f>
@@ -4401,7 +4425,7 @@
       </c>
       <c r="D42" s="3" t="inlineStr">
         <is>
-          <t>Built-In Magnetic Suction-Dark Night Green</t>
+          <t>Dark Night Green</t>
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr">
@@ -4429,26 +4453,38 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-GN-M.jpg</t>
         </is>
       </c>
-      <c r="J42" s="4" t="n">
-        <v>186.2</v>
-      </c>
-      <c r="K42" s="4" t="n">
-        <v>10</v>
+      <c r="J42" s="4" t="inlineStr">
+        <is>
+          <t>186.2</t>
+        </is>
+      </c>
+      <c r="K42" s="4" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
       </c>
       <c r="L42" s="4" t="n">
-        <v>50</v>
-      </c>
-      <c r="M42" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="N42" s="4" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O42" s="4" t="n">
-        <v>20</v>
-      </c>
-      <c r="P42" s="4" t="n">
-        <v>0</v>
+        <v>156</v>
+      </c>
+      <c r="M42" s="4" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N42" s="4" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O42" s="4" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P42" s="4" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q42" s="4">
         <f>SUM(J42:P42)</f>
@@ -4485,7 +4521,7 @@
       </c>
       <c r="D43" s="7" t="inlineStr">
         <is>
-          <t>Built-In Magnetic Suction-Charming Red</t>
+          <t>Charming Red</t>
         </is>
       </c>
       <c r="E43" s="7" t="inlineStr">
@@ -4513,26 +4549,38 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-RD-M.jpg</t>
         </is>
       </c>
-      <c r="J43" s="8" t="n">
-        <v>186.2</v>
-      </c>
-      <c r="K43" s="8" t="n">
-        <v>10</v>
+      <c r="J43" s="8" t="inlineStr">
+        <is>
+          <t>186.2</t>
+        </is>
+      </c>
+      <c r="K43" s="8" t="inlineStr">
+        <is>
+          <t>10.0</t>
+        </is>
       </c>
       <c r="L43" s="8" t="n">
-        <v>50</v>
-      </c>
-      <c r="M43" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N43" s="8" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="O43" s="8" t="n">
-        <v>20</v>
-      </c>
-      <c r="P43" s="8" t="n">
-        <v>0</v>
+        <v>156</v>
+      </c>
+      <c r="M43" s="8" t="inlineStr">
+        <is>
+          <t>5.0</t>
+        </is>
+      </c>
+      <c r="N43" s="8" t="inlineStr">
+        <is>
+          <t>11.5</t>
+        </is>
+      </c>
+      <c r="O43" s="8" t="inlineStr">
+        <is>
+          <t>20.0</t>
+        </is>
+      </c>
+      <c r="P43" s="8" t="inlineStr">
+        <is>
+          <t>0.0</t>
+        </is>
       </c>
       <c r="Q43" s="8">
         <f>SUM(J43:P43)</f>

</xml_diff>

<commit_message>
feat: process Honor x80i, Honor 600lite foreign version (Hard PC) and update inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,14 +476,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T49"/>
+  <dimension ref="A1:T59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
     <col width="17" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
-    <col width="27" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="48" customWidth="1" min="8" max="8"/>
@@ -4523,6 +4523,846 @@
         <v/>
       </c>
     </row>
+    <row r="50">
+      <c r="A50" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>HX80I-PC-GY-M</t>
+        </is>
+      </c>
+      <c r="C50" s="3" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D50" s="3" t="inlineStr">
+        <is>
+          <t>Titanium Gray</t>
+        </is>
+      </c>
+      <c r="E50" s="3" t="inlineStr">
+        <is>
+          <t>Honor x80i</t>
+        </is>
+      </c>
+      <c r="F50" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H50" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I50" s="2" t="inlineStr">
+        <is>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-GY-M.jpg</t>
+        </is>
+      </c>
+      <c r="J50" s="4" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K50" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L50" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M50" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N50" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O50" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P50" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q50" s="4">
+        <f>SUM(J50:P50)</f>
+        <v/>
+      </c>
+      <c r="R50" s="4">
+        <f>IF(Q50&lt;300, Q50*1.4, IF(Q50&lt;400, Q50*1.33, Q50*1.25))</f>
+        <v/>
+      </c>
+      <c r="S50" s="5">
+        <f>INT(R50/100)*100 + IF(MOD(ROUND(R50,0),100)&lt;25, 0, IF(MOD(ROUND(R50,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T50" s="4">
+        <f>IF(S50&lt;300, 0, MIN(99, IF(S50&lt;500, S50*7%, IF(S50&lt;700, S50*12%, S50*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>HX80I-PC-WT-M</t>
+        </is>
+      </c>
+      <c r="C51" s="7" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D51" s="7" t="inlineStr">
+        <is>
+          <t>Silver White</t>
+        </is>
+      </c>
+      <c r="E51" s="7" t="inlineStr">
+        <is>
+          <t>Honor x80i</t>
+        </is>
+      </c>
+      <c r="F51" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H51" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I51" s="6" t="inlineStr">
+        <is>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-WT-M.jpg</t>
+        </is>
+      </c>
+      <c r="J51" s="8" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K51" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L51" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M51" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N51" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O51" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P51" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q51" s="8">
+        <f>SUM(J51:P51)</f>
+        <v/>
+      </c>
+      <c r="R51" s="8">
+        <f>IF(Q51&lt;300, Q51*1.4, IF(Q51&lt;400, Q51*1.33, Q51*1.25))</f>
+        <v/>
+      </c>
+      <c r="S51" s="9">
+        <f>INT(R51/100)*100 + IF(MOD(ROUND(R51,0),100)&lt;25, 0, IF(MOD(ROUND(R51,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T51" s="8">
+        <f>IF(S51&lt;300, 0, MIN(99, IF(S51&lt;500, S51*7%, IF(S51&lt;700, S51*12%, S51*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>HX80I-PC-GN-M</t>
+        </is>
+      </c>
+      <c r="C52" s="3" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D52" s="3" t="inlineStr">
+        <is>
+          <t>Feitianqing</t>
+        </is>
+      </c>
+      <c r="E52" s="3" t="inlineStr">
+        <is>
+          <t>Honor x80i</t>
+        </is>
+      </c>
+      <c r="F52" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H52" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I52" s="2" t="inlineStr">
+        <is>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-GN-M.jpg</t>
+        </is>
+      </c>
+      <c r="J52" s="4" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K52" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L52" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M52" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N52" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O52" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P52" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q52" s="4">
+        <f>SUM(J52:P52)</f>
+        <v/>
+      </c>
+      <c r="R52" s="4">
+        <f>IF(Q52&lt;300, Q52*1.4, IF(Q52&lt;400, Q52*1.33, Q52*1.25))</f>
+        <v/>
+      </c>
+      <c r="S52" s="5">
+        <f>INT(R52/100)*100 + IF(MOD(ROUND(R52,0),100)&lt;25, 0, IF(MOD(ROUND(R52,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T52" s="4">
+        <f>IF(S52&lt;300, 0, MIN(99, IF(S52&lt;500, S52*7%, IF(S52&lt;700, S52*12%, S52*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>HX80I-PC-GD-M</t>
+        </is>
+      </c>
+      <c r="C53" s="7" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D53" s="7" t="inlineStr">
+        <is>
+          <t>Desert Gold</t>
+        </is>
+      </c>
+      <c r="E53" s="7" t="inlineStr">
+        <is>
+          <t>Honor x80i</t>
+        </is>
+      </c>
+      <c r="F53" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H53" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I53" s="6" t="inlineStr">
+        <is>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-GD-M.jpg</t>
+        </is>
+      </c>
+      <c r="J53" s="8" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K53" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L53" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M53" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N53" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O53" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P53" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q53" s="8">
+        <f>SUM(J53:P53)</f>
+        <v/>
+      </c>
+      <c r="R53" s="8">
+        <f>IF(Q53&lt;300, Q53*1.4, IF(Q53&lt;400, Q53*1.33, Q53*1.25))</f>
+        <v/>
+      </c>
+      <c r="S53" s="9">
+        <f>INT(R53/100)*100 + IF(MOD(ROUND(R53,0),100)&lt;25, 0, IF(MOD(ROUND(R53,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T53" s="8">
+        <f>IF(S53&lt;300, 0, MIN(99, IF(S53&lt;500, S53*7%, IF(S53&lt;700, S53*12%, S53*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>HX80I-PC-BK-M</t>
+        </is>
+      </c>
+      <c r="C54" s="3" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D54" s="3" t="inlineStr">
+        <is>
+          <t>Graphite Black</t>
+        </is>
+      </c>
+      <c r="E54" s="3" t="inlineStr">
+        <is>
+          <t>Honor x80i</t>
+        </is>
+      </c>
+      <c r="F54" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H54" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I54" s="2" t="inlineStr">
+        <is>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-BK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J54" s="4" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K54" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L54" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M54" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N54" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O54" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P54" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q54" s="4">
+        <f>SUM(J54:P54)</f>
+        <v/>
+      </c>
+      <c r="R54" s="4">
+        <f>IF(Q54&lt;300, Q54*1.4, IF(Q54&lt;400, Q54*1.33, Q54*1.25))</f>
+        <v/>
+      </c>
+      <c r="S54" s="5">
+        <f>INT(R54/100)*100 + IF(MOD(ROUND(R54,0),100)&lt;25, 0, IF(MOD(ROUND(R54,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T54" s="4">
+        <f>IF(S54&lt;300, 0, MIN(99, IF(S54&lt;500, S54*7%, IF(S54&lt;700, S54*12%, S54*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>H600L-PC-GY-M</t>
+        </is>
+      </c>
+      <c r="C55" s="7" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D55" s="7" t="inlineStr">
+        <is>
+          <t>Titanium Gray</t>
+        </is>
+      </c>
+      <c r="E55" s="7" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version</t>
+        </is>
+      </c>
+      <c r="F55" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G55" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H55" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I55" s="6" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GY-M.jpg</t>
+        </is>
+      </c>
+      <c r="J55" s="8" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K55" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L55" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M55" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N55" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O55" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P55" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q55" s="8">
+        <f>SUM(J55:P55)</f>
+        <v/>
+      </c>
+      <c r="R55" s="8">
+        <f>IF(Q55&lt;300, Q55*1.4, IF(Q55&lt;400, Q55*1.33, Q55*1.25))</f>
+        <v/>
+      </c>
+      <c r="S55" s="9">
+        <f>INT(R55/100)*100 + IF(MOD(ROUND(R55,0),100)&lt;25, 0, IF(MOD(ROUND(R55,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T55" s="8">
+        <f>IF(S55&lt;300, 0, MIN(99, IF(S55&lt;500, S55*7%, IF(S55&lt;700, S55*12%, S55*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>H600L-PC-WT-M</t>
+        </is>
+      </c>
+      <c r="C56" s="3" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D56" s="3" t="inlineStr">
+        <is>
+          <t>Silver White</t>
+        </is>
+      </c>
+      <c r="E56" s="3" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version</t>
+        </is>
+      </c>
+      <c r="F56" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G56" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H56" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I56" s="2" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-WT-M.jpg</t>
+        </is>
+      </c>
+      <c r="J56" s="4" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K56" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L56" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M56" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N56" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O56" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P56" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q56" s="4">
+        <f>SUM(J56:P56)</f>
+        <v/>
+      </c>
+      <c r="R56" s="4">
+        <f>IF(Q56&lt;300, Q56*1.4, IF(Q56&lt;400, Q56*1.33, Q56*1.25))</f>
+        <v/>
+      </c>
+      <c r="S56" s="5">
+        <f>INT(R56/100)*100 + IF(MOD(ROUND(R56,0),100)&lt;25, 0, IF(MOD(ROUND(R56,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T56" s="4">
+        <f>IF(S56&lt;300, 0, MIN(99, IF(S56&lt;500, S56*7%, IF(S56&lt;700, S56*12%, S56*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>H600L-PC-GN-M</t>
+        </is>
+      </c>
+      <c r="C57" s="7" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D57" s="7" t="inlineStr">
+        <is>
+          <t>Feitianqing</t>
+        </is>
+      </c>
+      <c r="E57" s="7" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version</t>
+        </is>
+      </c>
+      <c r="F57" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G57" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H57" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I57" s="6" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GN-M.jpg</t>
+        </is>
+      </c>
+      <c r="J57" s="8" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K57" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L57" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M57" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N57" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O57" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P57" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q57" s="8">
+        <f>SUM(J57:P57)</f>
+        <v/>
+      </c>
+      <c r="R57" s="8">
+        <f>IF(Q57&lt;300, Q57*1.4, IF(Q57&lt;400, Q57*1.33, Q57*1.25))</f>
+        <v/>
+      </c>
+      <c r="S57" s="9">
+        <f>INT(R57/100)*100 + IF(MOD(ROUND(R57,0),100)&lt;25, 0, IF(MOD(ROUND(R57,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T57" s="8">
+        <f>IF(S57&lt;300, 0, MIN(99, IF(S57&lt;500, S57*7%, IF(S57&lt;700, S57*12%, S57*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="2" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>H600L-PC-GD-M</t>
+        </is>
+      </c>
+      <c r="C58" s="3" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D58" s="3" t="inlineStr">
+        <is>
+          <t>Desert Gold</t>
+        </is>
+      </c>
+      <c r="E58" s="3" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version</t>
+        </is>
+      </c>
+      <c r="F58" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G58" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H58" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I58" s="2" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GD-M.jpg</t>
+        </is>
+      </c>
+      <c r="J58" s="4" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K58" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L58" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M58" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N58" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O58" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P58" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q58" s="4">
+        <f>SUM(J58:P58)</f>
+        <v/>
+      </c>
+      <c r="R58" s="4">
+        <f>IF(Q58&lt;300, Q58*1.4, IF(Q58&lt;400, Q58*1.33, Q58*1.25))</f>
+        <v/>
+      </c>
+      <c r="S58" s="5">
+        <f>INT(R58/100)*100 + IF(MOD(ROUND(R58,0),100)&lt;25, 0, IF(MOD(ROUND(R58,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T58" s="4">
+        <f>IF(S58&lt;300, 0, MIN(99, IF(S58&lt;500, S58*7%, IF(S58&lt;700, S58*12%, S58*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>H600L-PC-BK-M</t>
+        </is>
+      </c>
+      <c r="C59" s="7" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D59" s="7" t="inlineStr">
+        <is>
+          <t>Graphite Black</t>
+        </is>
+      </c>
+      <c r="E59" s="7" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version</t>
+        </is>
+      </c>
+      <c r="F59" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G59" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H59" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+        </is>
+      </c>
+      <c r="I59" s="6" t="inlineStr">
+        <is>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-BK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J59" s="8" t="n">
+        <v>478.8</v>
+      </c>
+      <c r="K59" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L59" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M59" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N59" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O59" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P59" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q59" s="8">
+        <f>SUM(J59:P59)</f>
+        <v/>
+      </c>
+      <c r="R59" s="8">
+        <f>IF(Q59&lt;300, Q59*1.4, IF(Q59&lt;400, Q59*1.33, Q59*1.25))</f>
+        <v/>
+      </c>
+      <c r="S59" s="9">
+        <f>INT(R59/100)*100 + IF(MOD(ROUND(R59,0),100)&lt;25, 0, IF(MOD(ROUND(R59,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T59" s="8">
+        <f>IF(S59&lt;300, 0, MIN(99, IF(S59&lt;500, S59*7%, IF(S59&lt;700, S59*12%, S59*15%))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: sync 48 records to inventory.xlsx and remove temp files
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -10,7 +10,7 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1" forceFullCalc="1"/>
 </workbook>
 </file>
 
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T43"/>
+  <dimension ref="A1:T49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="48" customWidth="1" min="1" max="1"/>
@@ -496,9 +496,9 @@
     <col width="12" customWidth="1" min="15" max="15"/>
     <col width="12" customWidth="1" min="16" max="16"/>
     <col width="16" customWidth="1" min="17" max="17"/>
-    <col width="48" customWidth="1" min="18" max="18"/>
-    <col width="48" customWidth="1" min="19" max="19"/>
-    <col width="48" customWidth="1" min="20" max="20"/>
+    <col width="16" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="19" max="19"/>
+    <col width="16" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -645,40 +645,26 @@
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr"/>
-      <c r="J2" s="4" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K2" s="4" t="inlineStr">
-        <is>
-          <t>11.7</t>
-        </is>
-      </c>
-      <c r="L2" s="4" t="inlineStr">
-        <is>
-          <t>54.6</t>
-        </is>
-      </c>
-      <c r="M2" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N2" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O2" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P2" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J2" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K2" s="4" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="L2" s="4" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="M2" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N2" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O2" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P2" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q2" s="4">
         <f>SUM(J2:P2)</f>
@@ -739,40 +725,26 @@
         </is>
       </c>
       <c r="I3" s="6" t="inlineStr"/>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>345.8</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>24.61</t>
-        </is>
-      </c>
-      <c r="L3" s="8" t="inlineStr">
-        <is>
-          <t>35.01</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N3" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J3" s="8" t="n">
+        <v>345.8</v>
+      </c>
+      <c r="K3" s="8" t="n">
+        <v>24.61</v>
+      </c>
+      <c r="L3" s="8" t="n">
+        <v>35.01</v>
+      </c>
+      <c r="M3" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N3" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O3" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P3" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q3" s="8">
         <f>SUM(J3:P3)</f>
@@ -833,40 +805,26 @@
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr"/>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>345.8</t>
-        </is>
-      </c>
-      <c r="K4" s="4" t="inlineStr">
-        <is>
-          <t>24.61</t>
-        </is>
-      </c>
-      <c r="L4" s="4" t="inlineStr">
-        <is>
-          <t>35.01</t>
-        </is>
-      </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N4" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O4" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P4" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J4" s="4" t="n">
+        <v>345.8</v>
+      </c>
+      <c r="K4" s="4" t="n">
+        <v>24.61</v>
+      </c>
+      <c r="L4" s="4" t="n">
+        <v>35.01</v>
+      </c>
+      <c r="M4" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N4" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O4" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P4" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q4" s="4">
         <f>SUM(J4:P4)</f>
@@ -927,40 +885,26 @@
         </is>
       </c>
       <c r="I5" s="6" t="inlineStr"/>
-      <c r="J5" s="8" t="inlineStr">
-        <is>
-          <t>159.6</t>
-        </is>
-      </c>
-      <c r="K5" s="8" t="inlineStr">
-        <is>
-          <t>2.66</t>
-        </is>
-      </c>
-      <c r="L5" s="8" t="inlineStr">
-        <is>
-          <t>51.2</t>
-        </is>
-      </c>
-      <c r="M5" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N5" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O5" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P5" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J5" s="8" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K5" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L5" s="8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M5" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N5" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O5" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P5" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q5" s="8">
         <f>SUM(J5:P5)</f>
@@ -1021,40 +965,26 @@
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr"/>
-      <c r="J6" s="4" t="inlineStr">
-        <is>
-          <t>159.6</t>
-        </is>
-      </c>
-      <c r="K6" s="4" t="inlineStr">
-        <is>
-          <t>2.66</t>
-        </is>
-      </c>
-      <c r="L6" s="4" t="inlineStr">
-        <is>
-          <t>51.2</t>
-        </is>
-      </c>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N6" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O6" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P6" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J6" s="4" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K6" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L6" s="4" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M6" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N6" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O6" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P6" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q6" s="4">
         <f>SUM(J6:P6)</f>
@@ -1115,40 +1045,26 @@
         </is>
       </c>
       <c r="I7" s="6" t="inlineStr"/>
-      <c r="J7" s="8" t="inlineStr">
-        <is>
-          <t>159.6</t>
-        </is>
-      </c>
-      <c r="K7" s="8" t="inlineStr">
-        <is>
-          <t>2.66</t>
-        </is>
-      </c>
-      <c r="L7" s="8" t="inlineStr">
-        <is>
-          <t>51.2</t>
-        </is>
-      </c>
-      <c r="M7" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N7" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O7" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P7" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J7" s="8" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K7" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L7" s="8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M7" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N7" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O7" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P7" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q7" s="8">
         <f>SUM(J7:P7)</f>
@@ -1209,40 +1125,26 @@
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr"/>
-      <c r="J8" s="4" t="inlineStr">
-        <is>
-          <t>159.6</t>
-        </is>
-      </c>
-      <c r="K8" s="4" t="inlineStr">
-        <is>
-          <t>2.66</t>
-        </is>
-      </c>
-      <c r="L8" s="4" t="inlineStr">
-        <is>
-          <t>51.2</t>
-        </is>
-      </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O8" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P8" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J8" s="4" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K8" s="4" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L8" s="4" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M8" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N8" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O8" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P8" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q8" s="4">
         <f>SUM(J8:P8)</f>
@@ -1299,40 +1201,26 @@
         </is>
       </c>
       <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="8" t="inlineStr">
-        <is>
-          <t>159.6</t>
-        </is>
-      </c>
-      <c r="K9" s="8" t="inlineStr">
-        <is>
-          <t>2.66</t>
-        </is>
-      </c>
-      <c r="L9" s="8" t="inlineStr">
-        <is>
-          <t>51.2</t>
-        </is>
-      </c>
-      <c r="M9" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N9" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O9" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P9" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J9" s="8" t="n">
+        <v>159.6</v>
+      </c>
+      <c r="K9" s="8" t="n">
+        <v>2.66</v>
+      </c>
+      <c r="L9" s="8" t="n">
+        <v>51.2</v>
+      </c>
+      <c r="M9" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N9" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O9" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P9" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q9" s="8">
         <f>SUM(J9:P9)</f>
@@ -1393,40 +1281,26 @@
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr"/>
-      <c r="J10" s="4" t="inlineStr">
-        <is>
-          <t>106.4</t>
-        </is>
-      </c>
-      <c r="K10" s="4" t="inlineStr">
-        <is>
-          <t>9.04</t>
-        </is>
-      </c>
-      <c r="L10" s="4" t="inlineStr">
-        <is>
-          <t>54.6</t>
-        </is>
-      </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N10" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O10" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P10" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J10" s="4" t="n">
+        <v>106.4</v>
+      </c>
+      <c r="K10" s="4" t="n">
+        <v>9.039999999999999</v>
+      </c>
+      <c r="L10" s="4" t="n">
+        <v>54.6</v>
+      </c>
+      <c r="M10" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N10" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P10" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q10" s="4">
         <f>SUM(J10:P10)</f>
@@ -1487,40 +1361,26 @@
         </is>
       </c>
       <c r="I11" s="6" t="inlineStr"/>
-      <c r="J11" s="8" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K11" s="8" t="inlineStr">
-        <is>
-          <t>11.44</t>
-        </is>
-      </c>
-      <c r="L11" s="8" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="M11" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N11" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O11" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P11" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J11" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="K11" s="8" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L11" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="M11" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N11" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O11" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P11" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q11" s="8">
         <f>SUM(J11:P11)</f>
@@ -1581,40 +1441,26 @@
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr"/>
-      <c r="J12" s="4" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K12" s="4" t="inlineStr">
-        <is>
-          <t>11.44</t>
-        </is>
-      </c>
-      <c r="L12" s="4" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N12" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O12" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P12" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J12" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K12" s="4" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L12" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="M12" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N12" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O12" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P12" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q12" s="4">
         <f>SUM(J12:P12)</f>
@@ -1675,40 +1521,26 @@
         </is>
       </c>
       <c r="I13" s="6" t="inlineStr"/>
-      <c r="J13" s="8" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>11.44</t>
-        </is>
-      </c>
-      <c r="L13" s="8" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="M13" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N13" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O13" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P13" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J13" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="K13" s="8" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L13" s="8" t="n">
+        <v>56</v>
+      </c>
+      <c r="M13" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N13" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O13" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P13" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q13" s="8">
         <f>SUM(J13:P13)</f>
@@ -1769,40 +1601,26 @@
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr"/>
-      <c r="J14" s="4" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K14" s="4" t="inlineStr">
-        <is>
-          <t>11.44</t>
-        </is>
-      </c>
-      <c r="L14" s="4" t="inlineStr">
-        <is>
-          <t>56.0</t>
-        </is>
-      </c>
-      <c r="M14" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N14" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O14" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P14" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J14" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K14" s="4" t="n">
+        <v>11.44</v>
+      </c>
+      <c r="L14" s="4" t="n">
+        <v>56</v>
+      </c>
+      <c r="M14" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N14" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O14" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P14" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q14" s="4">
         <f>SUM(J14:P14)</f>
@@ -1863,40 +1681,26 @@
         </is>
       </c>
       <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="8" t="inlineStr">
-        <is>
-          <t>146.3</t>
-        </is>
-      </c>
-      <c r="K15" s="8" t="inlineStr">
-        <is>
-          <t>79.8</t>
-        </is>
-      </c>
-      <c r="L15" s="8" t="inlineStr">
-        <is>
-          <t>87.5</t>
-        </is>
-      </c>
-      <c r="M15" s="8" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N15" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O15" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P15" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J15" s="8" t="n">
+        <v>146.3</v>
+      </c>
+      <c r="K15" s="8" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="L15" s="8" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="M15" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N15" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O15" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P15" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q15" s="8">
         <f>SUM(J15:P15)</f>
@@ -1957,40 +1761,26 @@
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr"/>
-      <c r="J16" s="4" t="inlineStr">
-        <is>
-          <t>146.3</t>
-        </is>
-      </c>
-      <c r="K16" s="4" t="inlineStr">
-        <is>
-          <t>79.8</t>
-        </is>
-      </c>
-      <c r="L16" s="4" t="inlineStr">
-        <is>
-          <t>87.5</t>
-        </is>
-      </c>
-      <c r="M16" s="4" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N16" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O16" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P16" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J16" s="4" t="n">
+        <v>146.3</v>
+      </c>
+      <c r="K16" s="4" t="n">
+        <v>79.8</v>
+      </c>
+      <c r="L16" s="4" t="n">
+        <v>87.5</v>
+      </c>
+      <c r="M16" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N16" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O16" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P16" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q16" s="4">
         <f>SUM(J16:P16)</f>
@@ -2051,40 +1841,26 @@
         </is>
       </c>
       <c r="I17" s="6" t="inlineStr"/>
-      <c r="J17" s="8" t="inlineStr">
-        <is>
-          <t>252.7</t>
-        </is>
-      </c>
-      <c r="K17" s="8" t="inlineStr">
-        <is>
-          <t>18.09</t>
-        </is>
-      </c>
-      <c r="L17" s="8" t="inlineStr">
-        <is>
-          <t>35.0</t>
-        </is>
-      </c>
-      <c r="M17" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N17" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O17" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P17" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J17" s="8" t="n">
+        <v>252.7</v>
+      </c>
+      <c r="K17" s="8" t="n">
+        <v>18.09</v>
+      </c>
+      <c r="L17" s="8" t="n">
+        <v>35</v>
+      </c>
+      <c r="M17" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N17" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O17" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P17" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q17" s="8">
         <f>SUM(J17:P17)</f>
@@ -2145,40 +1921,26 @@
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr"/>
-      <c r="J18" s="4" t="inlineStr">
-        <is>
-          <t>252.7</t>
-        </is>
-      </c>
-      <c r="K18" s="4" t="inlineStr">
-        <is>
-          <t>18.09</t>
-        </is>
-      </c>
-      <c r="L18" s="4" t="inlineStr">
-        <is>
-          <t>35.0</t>
-        </is>
-      </c>
-      <c r="M18" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N18" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O18" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P18" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J18" s="4" t="n">
+        <v>252.7</v>
+      </c>
+      <c r="K18" s="4" t="n">
+        <v>18.09</v>
+      </c>
+      <c r="L18" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="M18" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N18" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O18" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P18" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q18" s="4">
         <f>SUM(J18:P18)</f>
@@ -2239,40 +2001,26 @@
         </is>
       </c>
       <c r="I19" s="6" t="inlineStr"/>
-      <c r="J19" s="8" t="inlineStr">
-        <is>
-          <t>265.74</t>
-        </is>
-      </c>
-      <c r="K19" s="8" t="inlineStr">
-        <is>
-          <t>50.2</t>
-        </is>
-      </c>
-      <c r="L19" s="8" t="inlineStr">
-        <is>
-          <t>80.0</t>
-        </is>
-      </c>
-      <c r="M19" s="8" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N19" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O19" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P19" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J19" s="8" t="n">
+        <v>265.74</v>
+      </c>
+      <c r="K19" s="8" t="n">
+        <v>50.2</v>
+      </c>
+      <c r="L19" s="8" t="n">
+        <v>80</v>
+      </c>
+      <c r="M19" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N19" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O19" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P19" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q19" s="8">
         <f>SUM(J19:P19)</f>
@@ -2333,40 +2081,26 @@
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr"/>
-      <c r="J20" s="4" t="inlineStr">
-        <is>
-          <t>87.25</t>
-        </is>
-      </c>
-      <c r="K20" s="4" t="inlineStr">
-        <is>
-          <t>16.55</t>
-        </is>
-      </c>
-      <c r="L20" s="4" t="inlineStr">
-        <is>
-          <t>81.6</t>
-        </is>
-      </c>
-      <c r="M20" s="4" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N20" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O20" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P20" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J20" s="4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K20" s="4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L20" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M20" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N20" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O20" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P20" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q20" s="4">
         <f>SUM(J20:P20)</f>
@@ -2427,40 +2161,26 @@
         </is>
       </c>
       <c r="I21" s="6" t="inlineStr"/>
-      <c r="J21" s="8" t="inlineStr">
-        <is>
-          <t>87.25</t>
-        </is>
-      </c>
-      <c r="K21" s="8" t="inlineStr">
-        <is>
-          <t>16.55</t>
-        </is>
-      </c>
-      <c r="L21" s="8" t="inlineStr">
-        <is>
-          <t>81.6</t>
-        </is>
-      </c>
-      <c r="M21" s="8" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N21" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O21" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P21" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J21" s="8" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K21" s="8" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L21" s="8" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M21" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N21" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O21" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P21" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q21" s="8">
         <f>SUM(J21:P21)</f>
@@ -2521,40 +2241,26 @@
         </is>
       </c>
       <c r="I22" s="2" t="inlineStr"/>
-      <c r="J22" s="4" t="inlineStr">
-        <is>
-          <t>87.25</t>
-        </is>
-      </c>
-      <c r="K22" s="4" t="inlineStr">
-        <is>
-          <t>16.55</t>
-        </is>
-      </c>
-      <c r="L22" s="4" t="inlineStr">
-        <is>
-          <t>81.6</t>
-        </is>
-      </c>
-      <c r="M22" s="4" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N22" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O22" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P22" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J22" s="4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K22" s="4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L22" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M22" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N22" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O22" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P22" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q22" s="4">
         <f>SUM(J22:P22)</f>
@@ -2615,40 +2321,26 @@
         </is>
       </c>
       <c r="I23" s="6" t="inlineStr"/>
-      <c r="J23" s="8" t="inlineStr">
-        <is>
-          <t>87.25</t>
-        </is>
-      </c>
-      <c r="K23" s="8" t="inlineStr">
-        <is>
-          <t>16.55</t>
-        </is>
-      </c>
-      <c r="L23" s="8" t="inlineStr">
-        <is>
-          <t>81.6</t>
-        </is>
-      </c>
-      <c r="M23" s="8" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N23" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O23" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P23" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J23" s="8" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K23" s="8" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L23" s="8" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M23" s="8" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N23" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O23" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P23" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q23" s="8">
         <f>SUM(J23:P23)</f>
@@ -2709,40 +2401,26 @@
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr"/>
-      <c r="J24" s="4" t="inlineStr">
-        <is>
-          <t>87.25</t>
-        </is>
-      </c>
-      <c r="K24" s="4" t="inlineStr">
-        <is>
-          <t>16.55</t>
-        </is>
-      </c>
-      <c r="L24" s="4" t="inlineStr">
-        <is>
-          <t>81.6</t>
-        </is>
-      </c>
-      <c r="M24" s="4" t="inlineStr">
-        <is>
-          <t>5.09</t>
-        </is>
-      </c>
-      <c r="N24" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O24" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P24" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J24" s="4" t="n">
+        <v>87.25</v>
+      </c>
+      <c r="K24" s="4" t="n">
+        <v>16.55</v>
+      </c>
+      <c r="L24" s="4" t="n">
+        <v>81.59999999999999</v>
+      </c>
+      <c r="M24" s="4" t="n">
+        <v>5.09</v>
+      </c>
+      <c r="N24" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O24" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P24" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q24" s="4">
         <f>SUM(J24:P24)</f>
@@ -2803,40 +2481,26 @@
         </is>
       </c>
       <c r="I25" s="6" t="inlineStr"/>
-      <c r="J25" s="8" t="inlineStr">
-        <is>
-          <t>119.7</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr">
-        <is>
-          <t>8.75</t>
-        </is>
-      </c>
-      <c r="L25" s="8" t="inlineStr">
-        <is>
-          <t>38.0</t>
-        </is>
-      </c>
-      <c r="M25" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N25" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O25" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P25" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J25" s="8" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K25" s="8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L25" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="M25" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N25" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O25" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P25" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q25" s="8">
         <f>SUM(J25:P25)</f>
@@ -2897,40 +2561,26 @@
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr"/>
-      <c r="J26" s="4" t="inlineStr">
-        <is>
-          <t>119.7</t>
-        </is>
-      </c>
-      <c r="K26" s="4" t="inlineStr">
-        <is>
-          <t>8.75</t>
-        </is>
-      </c>
-      <c r="L26" s="4" t="inlineStr">
-        <is>
-          <t>38.0</t>
-        </is>
-      </c>
-      <c r="M26" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N26" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O26" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P26" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J26" s="4" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K26" s="4" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L26" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="M26" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N26" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O26" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P26" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q26" s="4">
         <f>SUM(J26:P26)</f>
@@ -2991,40 +2641,26 @@
         </is>
       </c>
       <c r="I27" s="6" t="inlineStr"/>
-      <c r="J27" s="8" t="inlineStr">
-        <is>
-          <t>119.7</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="inlineStr">
-        <is>
-          <t>8.75</t>
-        </is>
-      </c>
-      <c r="L27" s="8" t="inlineStr">
-        <is>
-          <t>38.0</t>
-        </is>
-      </c>
-      <c r="M27" s="8" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N27" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O27" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P27" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J27" s="8" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K27" s="8" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L27" s="8" t="n">
+        <v>38</v>
+      </c>
+      <c r="M27" s="8" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N27" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O27" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P27" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q27" s="8">
         <f>SUM(J27:P27)</f>
@@ -3085,40 +2721,26 @@
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr"/>
-      <c r="J28" s="4" t="inlineStr">
-        <is>
-          <t>119.7</t>
-        </is>
-      </c>
-      <c r="K28" s="4" t="inlineStr">
-        <is>
-          <t>8.75</t>
-        </is>
-      </c>
-      <c r="L28" s="4" t="inlineStr">
-        <is>
-          <t>38.0</t>
-        </is>
-      </c>
-      <c r="M28" s="4" t="inlineStr">
-        <is>
-          <t>2.54</t>
-        </is>
-      </c>
-      <c r="N28" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O28" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P28" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J28" s="4" t="n">
+        <v>119.7</v>
+      </c>
+      <c r="K28" s="4" t="n">
+        <v>8.75</v>
+      </c>
+      <c r="L28" s="4" t="n">
+        <v>38</v>
+      </c>
+      <c r="M28" s="4" t="n">
+        <v>2.54</v>
+      </c>
+      <c r="N28" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O28" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P28" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q28" s="4">
         <f>SUM(J28:P28)</f>
@@ -3183,40 +2805,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S.jpg</t>
         </is>
       </c>
-      <c r="J29" s="8" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K29" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L29" s="8" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M29" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N29" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O29" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P29" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J29" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K29" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L29" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M29" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N29" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O29" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P29" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q29" s="8">
         <f>SUM(J29:P29)</f>
@@ -3281,40 +2889,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
       </c>
-      <c r="J30" s="4" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K30" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L30" s="4" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M30" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N30" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O30" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P30" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J30" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K30" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L30" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M30" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N30" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O30" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P30" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q30" s="4">
         <f>SUM(J30:P30)</f>
@@ -3379,40 +2973,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S.jpg</t>
         </is>
       </c>
-      <c r="J31" s="8" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K31" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L31" s="8" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M31" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N31" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O31" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P31" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J31" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K31" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L31" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M31" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N31" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O31" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P31" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q31" s="8">
         <f>SUM(J31:P31)</f>
@@ -3477,40 +3057,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S.jpg</t>
         </is>
       </c>
-      <c r="J32" s="4" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K32" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L32" s="4" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M32" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N32" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O32" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P32" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J32" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K32" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L32" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M32" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N32" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O32" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P32" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q32" s="4">
         <f>SUM(J32:P32)</f>
@@ -3575,40 +3141,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S.jpg</t>
         </is>
       </c>
-      <c r="J33" s="8" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K33" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L33" s="8" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M33" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N33" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O33" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P33" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J33" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K33" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L33" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M33" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N33" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O33" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P33" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q33" s="8">
         <f>SUM(J33:P33)</f>
@@ -3673,40 +3225,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
       </c>
-      <c r="J34" s="4" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K34" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L34" s="4" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M34" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N34" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O34" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P34" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J34" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K34" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L34" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M34" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N34" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O34" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P34" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q34" s="4">
         <f>SUM(J34:P34)</f>
@@ -3771,40 +3309,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-RD-S.jpg</t>
         </is>
       </c>
-      <c r="J35" s="8" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K35" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L35" s="8" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M35" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N35" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O35" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P35" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J35" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K35" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L35" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M35" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N35" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O35" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P35" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q35" s="8">
         <f>SUM(J35:P35)</f>
@@ -3869,40 +3393,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-TL-S.jpg</t>
         </is>
       </c>
-      <c r="J36" s="4" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K36" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L36" s="4" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M36" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N36" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O36" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P36" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J36" s="4" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K36" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L36" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M36" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N36" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O36" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P36" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q36" s="4">
         <f>SUM(J36:P36)</f>
@@ -3967,40 +3477,26 @@
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-CL-C.jpg</t>
         </is>
       </c>
-      <c r="J37" s="8" t="inlineStr">
-        <is>
-          <t>39.9</t>
-        </is>
-      </c>
-      <c r="K37" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L37" s="8" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M37" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N37" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O37" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P37" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J37" s="8" t="n">
+        <v>39.9</v>
+      </c>
+      <c r="K37" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L37" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M37" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N37" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O37" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P37" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q37" s="8">
         <f>SUM(J37:P37)</f>
@@ -4065,40 +3561,26 @@
           <t>Realme Neo8/TPU/sku/RN8-TPU-WT-M.jpg</t>
         </is>
       </c>
-      <c r="J38" s="4" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K38" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L38" s="4" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M38" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N38" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O38" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P38" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J38" s="4" t="n">
+        <v>133</v>
+      </c>
+      <c r="K38" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L38" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M38" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N38" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O38" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P38" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q38" s="4">
         <f>SUM(J38:P38)</f>
@@ -4163,40 +3645,26 @@
           <t>Realme Neo8/TPU/sku/RN8-TPU-BK-M.jpg</t>
         </is>
       </c>
-      <c r="J39" s="8" t="inlineStr">
-        <is>
-          <t>133.0</t>
-        </is>
-      </c>
-      <c r="K39" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
-      </c>
-      <c r="L39" s="8" t="inlineStr">
-        <is>
-          <t>50.0</t>
-        </is>
-      </c>
-      <c r="M39" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N39" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O39" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P39" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="J39" s="8" t="n">
+        <v>133</v>
+      </c>
+      <c r="K39" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L39" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M39" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N39" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O39" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P39" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q39" s="8">
         <f>SUM(J39:P39)</f>
@@ -4261,38 +3729,26 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-BK-M.jpg</t>
         </is>
       </c>
-      <c r="J40" s="4" t="inlineStr">
-        <is>
-          <t>186.2</t>
-        </is>
-      </c>
-      <c r="K40" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
+      <c r="J40" s="4" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K40" s="4" t="n">
+        <v>10</v>
       </c>
       <c r="L40" s="4" t="n">
         <v>156</v>
       </c>
-      <c r="M40" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N40" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O40" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P40" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="M40" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N40" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O40" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P40" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q40" s="4">
         <f>SUM(J40:P40)</f>
@@ -4357,38 +3813,26 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-BL-M.jpg</t>
         </is>
       </c>
-      <c r="J41" s="8" t="inlineStr">
-        <is>
-          <t>186.2</t>
-        </is>
-      </c>
-      <c r="K41" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
+      <c r="J41" s="8" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K41" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="L41" s="8" t="n">
         <v>156</v>
       </c>
-      <c r="M41" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N41" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O41" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P41" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="M41" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N41" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O41" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P41" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q41" s="8">
         <f>SUM(J41:P41)</f>
@@ -4453,38 +3897,26 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-GN-M.jpg</t>
         </is>
       </c>
-      <c r="J42" s="4" t="inlineStr">
-        <is>
-          <t>186.2</t>
-        </is>
-      </c>
-      <c r="K42" s="4" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
+      <c r="J42" s="4" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K42" s="4" t="n">
+        <v>10</v>
       </c>
       <c r="L42" s="4" t="n">
         <v>156</v>
       </c>
-      <c r="M42" s="4" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N42" s="4" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O42" s="4" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P42" s="4" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="M42" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N42" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O42" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P42" s="4" t="n">
+        <v>0</v>
       </c>
       <c r="Q42" s="4">
         <f>SUM(J42:P42)</f>
@@ -4549,38 +3981,26 @@
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-RD-M.jpg</t>
         </is>
       </c>
-      <c r="J43" s="8" t="inlineStr">
-        <is>
-          <t>186.2</t>
-        </is>
-      </c>
-      <c r="K43" s="8" t="inlineStr">
-        <is>
-          <t>10.0</t>
-        </is>
+      <c r="J43" s="8" t="n">
+        <v>186.2</v>
+      </c>
+      <c r="K43" s="8" t="n">
+        <v>10</v>
       </c>
       <c r="L43" s="8" t="n">
         <v>156</v>
       </c>
-      <c r="M43" s="8" t="inlineStr">
-        <is>
-          <t>5.0</t>
-        </is>
-      </c>
-      <c r="N43" s="8" t="inlineStr">
-        <is>
-          <t>11.5</t>
-        </is>
-      </c>
-      <c r="O43" s="8" t="inlineStr">
-        <is>
-          <t>20.0</t>
-        </is>
-      </c>
-      <c r="P43" s="8" t="inlineStr">
-        <is>
-          <t>0.0</t>
-        </is>
+      <c r="M43" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N43" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O43" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P43" s="8" t="n">
+        <v>0</v>
       </c>
       <c r="Q43" s="8">
         <f>SUM(J43:P43)</f>
@@ -4596,6 +4016,510 @@
       </c>
       <c r="T43" s="8">
         <f>IF(S43&lt;300, 0, MIN(99, IF(S43&lt;500, S43*7%, IF(S43&lt;700, S43*12%, S43*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr">
+        <is>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>HX80I-TPU-SV-E</t>
+        </is>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="inlineStr">
+        <is>
+          <t>Honor X80i</t>
+        </is>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-SV-E.jpg</t>
+        </is>
+      </c>
+      <c r="J44" s="4" t="n">
+        <v>234.08</v>
+      </c>
+      <c r="K44" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L44" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M44" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N44" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O44" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P44" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q44" s="4">
+        <f>SUM(J44:P44)</f>
+        <v/>
+      </c>
+      <c r="R44" s="4">
+        <f>IF(Q44&lt;300, Q44*1.4, IF(Q44&lt;400, Q44*1.33, Q44*1.25))</f>
+        <v/>
+      </c>
+      <c r="S44" s="5">
+        <f>INT(R44/100)*100 + IF(MOD(ROUND(R44,0),100)&lt;25, 0, IF(MOD(ROUND(R44,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T44" s="4">
+        <f>IF(S44&lt;300, 0, MIN(99, IF(S44&lt;500, S44*7%, IF(S44&lt;700, S44*12%, S44*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="6" t="inlineStr">
+        <is>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>HX80I-TPU-BK-E</t>
+        </is>
+      </c>
+      <c r="C45" s="7" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D45" s="7" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="E45" s="7" t="inlineStr">
+        <is>
+          <t>Honor X80i</t>
+        </is>
+      </c>
+      <c r="F45" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H45" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+        </is>
+      </c>
+      <c r="I45" s="6" t="inlineStr">
+        <is>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-BK-E.jpg</t>
+        </is>
+      </c>
+      <c r="J45" s="8" t="n">
+        <v>234.08</v>
+      </c>
+      <c r="K45" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L45" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M45" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N45" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O45" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P45" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q45" s="8">
+        <f>SUM(J45:P45)</f>
+        <v/>
+      </c>
+      <c r="R45" s="8">
+        <f>IF(Q45&lt;300, Q45*1.4, IF(Q45&lt;400, Q45*1.33, Q45*1.25))</f>
+        <v/>
+      </c>
+      <c r="S45" s="9">
+        <f>INT(R45/100)*100 + IF(MOD(ROUND(R45,0),100)&lt;25, 0, IF(MOD(ROUND(R45,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T45" s="8">
+        <f>IF(S45&lt;300, 0, MIN(99, IF(S45&lt;500, S45*7%, IF(S45&lt;700, S45*12%, S45*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="2" t="inlineStr">
+        <is>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>HX80I-TPU-PR-E</t>
+        </is>
+      </c>
+      <c r="C46" s="3" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D46" s="3" t="inlineStr">
+        <is>
+          <t>Purple</t>
+        </is>
+      </c>
+      <c r="E46" s="3" t="inlineStr">
+        <is>
+          <t>Honor X80i</t>
+        </is>
+      </c>
+      <c r="F46" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H46" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+        </is>
+      </c>
+      <c r="I46" s="2" t="inlineStr">
+        <is>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-PR-E.jpg</t>
+        </is>
+      </c>
+      <c r="J46" s="4" t="n">
+        <v>234.08</v>
+      </c>
+      <c r="K46" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L46" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M46" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N46" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O46" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P46" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q46" s="4">
+        <f>SUM(J46:P46)</f>
+        <v/>
+      </c>
+      <c r="R46" s="4">
+        <f>IF(Q46&lt;300, Q46*1.4, IF(Q46&lt;400, Q46*1.33, Q46*1.25))</f>
+        <v/>
+      </c>
+      <c r="S46" s="5">
+        <f>INT(R46/100)*100 + IF(MOD(ROUND(R46,0),100)&lt;25, 0, IF(MOD(ROUND(R46,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T46" s="4">
+        <f>IF(S46&lt;300, 0, MIN(99, IF(S46&lt;500, S46*7%, IF(S46&lt;700, S46*12%, S46*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>HX80I-TPU-BL-E</t>
+        </is>
+      </c>
+      <c r="C47" s="7" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D47" s="7" t="inlineStr">
+        <is>
+          <t>Blue</t>
+        </is>
+      </c>
+      <c r="E47" s="7" t="inlineStr">
+        <is>
+          <t>Honor X80i</t>
+        </is>
+      </c>
+      <c r="F47" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H47" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+        </is>
+      </c>
+      <c r="I47" s="6" t="inlineStr">
+        <is>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-BL-E.jpg</t>
+        </is>
+      </c>
+      <c r="J47" s="8" t="n">
+        <v>234.08</v>
+      </c>
+      <c r="K47" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L47" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M47" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N47" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O47" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P47" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q47" s="8">
+        <f>SUM(J47:P47)</f>
+        <v/>
+      </c>
+      <c r="R47" s="8">
+        <f>IF(Q47&lt;300, Q47*1.4, IF(Q47&lt;400, Q47*1.33, Q47*1.25))</f>
+        <v/>
+      </c>
+      <c r="S47" s="9">
+        <f>INT(R47/100)*100 + IF(MOD(ROUND(R47,0),100)&lt;25, 0, IF(MOD(ROUND(R47,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T47" s="8">
+        <f>IF(S47&lt;300, 0, MIN(99, IF(S47&lt;500, S47*7%, IF(S47&lt;700, S47*12%, S47*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="2" t="inlineStr">
+        <is>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>HX80I-TPU-PK-E</t>
+        </is>
+      </c>
+      <c r="C48" s="3" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D48" s="3" t="inlineStr">
+        <is>
+          <t>Pink</t>
+        </is>
+      </c>
+      <c r="E48" s="3" t="inlineStr">
+        <is>
+          <t>Honor X80i</t>
+        </is>
+      </c>
+      <c r="F48" s="3" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G48" s="3" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H48" s="2" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+        </is>
+      </c>
+      <c r="I48" s="2" t="inlineStr">
+        <is>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-PK-E.jpg</t>
+        </is>
+      </c>
+      <c r="J48" s="4" t="n">
+        <v>234.08</v>
+      </c>
+      <c r="K48" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L48" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="M48" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N48" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O48" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P48" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q48" s="4">
+        <f>SUM(J48:P48)</f>
+        <v/>
+      </c>
+      <c r="R48" s="4">
+        <f>IF(Q48&lt;300, Q48*1.4, IF(Q48&lt;400, Q48*1.33, Q48*1.25))</f>
+        <v/>
+      </c>
+      <c r="S48" s="5">
+        <f>INT(R48/100)*100 + IF(MOD(ROUND(R48,0),100)&lt;25, 0, IF(MOD(ROUND(R48,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T48" s="4">
+        <f>IF(S48&lt;300, 0, MIN(99, IF(S48&lt;500, S48*7%, IF(S48&lt;700, S48*12%, S48*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>HX80I-TPU-GN-E</t>
+        </is>
+      </c>
+      <c r="C49" s="7" t="inlineStr">
+        <is>
+          <t>TPU</t>
+        </is>
+      </c>
+      <c r="D49" s="7" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="E49" s="7" t="inlineStr">
+        <is>
+          <t>Honor X80i</t>
+        </is>
+      </c>
+      <c r="F49" s="7" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" s="7" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H49" s="6" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+        </is>
+      </c>
+      <c r="I49" s="6" t="inlineStr">
+        <is>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-GN-E.jpg</t>
+        </is>
+      </c>
+      <c r="J49" s="8" t="n">
+        <v>234.08</v>
+      </c>
+      <c r="K49" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L49" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="M49" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N49" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O49" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P49" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q49" s="8">
+        <f>SUM(J49:P49)</f>
+        <v/>
+      </c>
+      <c r="R49" s="8">
+        <f>IF(Q49&lt;300, Q49*1.4, IF(Q49&lt;400, Q49*1.33, Q49*1.25))</f>
+        <v/>
+      </c>
+      <c r="S49" s="9">
+        <f>INT(R49/100)*100 + IF(MOD(ROUND(R49,0),100)&lt;25, 0, IF(MOD(ROUND(R49,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T49" s="8">
+        <f>IF(S49&lt;300, 0, MIN(99, IF(S49&lt;500, S49*7%, IF(S49&lt;700, S49*12%, S49*15%))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: make Product Code / SKU Column 1 (A) and Product Name Column 2 (B) in schema
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -88,10 +88,10 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -100,10 +100,10 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="center"/>
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="4" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
@@ -479,8 +479,8 @@
   <dimension ref="A1:T59"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="48" customWidth="1" min="1" max="1"/>
-    <col width="17" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="1" max="1"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="33" customWidth="1" min="3" max="3"/>
     <col width="37" customWidth="1" min="4" max="4"/>
     <col width="32" customWidth="1" min="5" max="5"/>
@@ -504,12 +504,12 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>Product Code</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>Product Name</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Product Code</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
@@ -606,45 +606,45 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>T4P-TG-BP-N</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Protective Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr">
-        <is>
-          <t>T4P-TG-BP-N</t>
-        </is>
-      </c>
-      <c r="C2" s="3" t="inlineStr">
+      <c r="C2" s="2" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D2" s="3" t="inlineStr">
+      <c r="D2" s="2" t="inlineStr">
         <is>
           <t>Black - printed</t>
         </is>
       </c>
-      <c r="E2" s="3" t="inlineStr">
+      <c r="E2" s="2" t="inlineStr">
         <is>
           <t>RedmiTurbo 4 Pro</t>
         </is>
       </c>
-      <c r="F2" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G2" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H2" s="2" t="inlineStr">
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H2" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000TPCI3HYH3-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-independent-station-15spod13t-semi-hosted-civi4/1AD8305263723979</t>
         </is>
       </c>
-      <c r="I2" s="2" t="inlineStr"/>
+      <c r="I2" s="3" t="inlineStr"/>
       <c r="J2" s="4" t="n">
         <v>133</v>
       </c>
@@ -686,45 +686,45 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
+          <t>18PM-TPUM-CR-N</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
           <t>iPhone 18 Pro Max Phone Case, Magnetic, Transparent, with Lens Film</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>18PM-TPUM-CR-N</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="6" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="6" t="inlineStr">
         <is>
           <t>Cherry Red Magnetic Style</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="6" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H3" s="6" t="inlineStr">
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000P47PA9R8D-suitable-for-iphone-18-pro-max-phone-case-magnetic-transparent-with-apple-17-lens-film-full-coverage-and-a-simple-drop-resistant-design/1AD8373708955104</t>
         </is>
       </c>
-      <c r="I3" s="6" t="inlineStr"/>
+      <c r="I3" s="7" t="inlineStr"/>
       <c r="J3" s="8" t="n">
         <v>345.8</v>
       </c>
@@ -766,45 +766,45 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
+          <t>18PM-TPUM-SB-N</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
           <t>iPhone 18 Pro Max Phone Case, Magnetic, Transparent, with Lens Film</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>18PM-TPUM-SB-N</t>
-        </is>
-      </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="D4" s="2" t="inlineStr">
         <is>
           <t>Sky Blue Magnetic Style</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="E4" s="2" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H4" s="2" t="inlineStr">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000P47PA9R8D-suitable-for-iphone-18-pro-max-phone-case-magnetic-transparent-with-apple-17-lens-film-full-coverage-and-a-simple-drop-resistant-design/1AD8373708955104</t>
         </is>
       </c>
-      <c r="I4" s="2" t="inlineStr"/>
+      <c r="I4" s="3" t="inlineStr"/>
       <c r="J4" s="4" t="n">
         <v>345.8</v>
       </c>
@@ -846,45 +846,45 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
+          <t>T4P-AC-BG-N</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
           <t>Redmi Turbo 4 Pro Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>T4P-AC-BG-N</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D5" s="7" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Black -Green</t>
         </is>
       </c>
-      <c r="E5" s="7" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F5" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G5" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H5" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr"/>
+      <c r="I5" s="7" t="inlineStr"/>
       <c r="J5" s="8" t="n">
         <v>159.6</v>
       </c>
@@ -926,45 +926,45 @@
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
+          <t>T4P-AC-BR-N</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
           <t>Redmi Turbo 4 Pro Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
-        <is>
-          <t>T4P-AC-BR-N</t>
-        </is>
-      </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>Black -Red</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G6" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H6" s="2" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H6" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I6" s="2" t="inlineStr"/>
+      <c r="I6" s="3" t="inlineStr"/>
       <c r="J6" s="4" t="n">
         <v>159.6</v>
       </c>
@@ -1006,45 +1006,45 @@
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
+          <t>T4P-AC-BB-N</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
           <t>Redmi  Turbo4 Pro Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>T4P-AC-BB-N</t>
-        </is>
-      </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C7" s="6" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="D7" s="6" t="inlineStr">
         <is>
           <t>Black -Blue</t>
         </is>
       </c>
-      <c r="E7" s="7" t="inlineStr">
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F7" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G7" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H7" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I7" s="6" t="inlineStr"/>
+      <c r="I7" s="7" t="inlineStr"/>
       <c r="J7" s="8" t="n">
         <v>159.6</v>
       </c>
@@ -1086,45 +1086,45 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
+          <t>T4-AC-BR-N</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
           <t>Redmi Turbo  4 Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t>T4-AC-BR-N</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
+      <c r="C8" s="2" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D8" s="3" t="inlineStr">
+      <c r="D8" s="2" t="inlineStr">
         <is>
           <t>Black -Red</t>
         </is>
       </c>
-      <c r="E8" s="3" t="inlineStr">
+      <c r="E8" s="2" t="inlineStr">
         <is>
           <t>Redmi Turbo 4</t>
         </is>
       </c>
-      <c r="F8" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G8" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H8" s="2" t="inlineStr">
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H8" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I8" s="2" t="inlineStr"/>
+      <c r="I8" s="3" t="inlineStr"/>
       <c r="J8" s="4" t="n">
         <v>159.6</v>
       </c>
@@ -1166,41 +1166,41 @@
     <row r="9">
       <c r="A9" s="6" t="inlineStr">
         <is>
+          <t>T4-AC-BB-N</t>
+        </is>
+      </c>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
           <t>Redmi Turbo 4 Mecha style acrylic matte finish case</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr">
-        <is>
-          <t>T4-AC-BB-N</t>
-        </is>
-      </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="D9" s="6" t="inlineStr">
         <is>
           <t>Black -Blue</t>
         </is>
       </c>
-      <c r="E9" s="7" t="inlineStr">
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4</t>
         </is>
       </c>
-      <c r="F9" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G9" s="7" t="inlineStr"/>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000UYR39CZAL-cool-mecha-style-case-suitable-for-redmi-turbo-4-pro-new-mens-mecha-style-turbo-3-phone-case/1AD8366032951156</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
+      <c r="I9" s="7" t="inlineStr"/>
       <c r="J9" s="8" t="n">
         <v>159.6</v>
       </c>
@@ -1242,45 +1242,45 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
+          <t>S26U-SI-BP-N</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
           <t>Samsung Galaxy S26 Series Spider Style Silicone Printed Case</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr">
-        <is>
-          <t>S26U-SI-BP-N</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr">
+      <c r="C10" s="2" t="inlineStr">
         <is>
           <t>Silicone</t>
         </is>
       </c>
-      <c r="D10" s="3" t="inlineStr">
+      <c r="D10" s="2" t="inlineStr">
         <is>
           <t>Black - printed</t>
         </is>
       </c>
-      <c r="E10" s="3" t="inlineStr">
+      <c r="E10" s="2" t="inlineStr">
         <is>
           <t>Galaxy S26 Ultra</t>
         </is>
       </c>
-      <c r="F10" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G10" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H10" s="2" t="inlineStr">
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H10" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000O0R0QIE2O-jit-one-piece-dropshippinggalaxys25-phone-case-semi-managed-s24-fully-managed-s24fe-aliexpress/1AD8304920318534</t>
         </is>
       </c>
-      <c r="I10" s="2" t="inlineStr"/>
+      <c r="I10" s="3" t="inlineStr"/>
       <c r="J10" s="4" t="n">
         <v>106.4</v>
       </c>
@@ -1322,45 +1322,45 @@
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
+          <t>T4P-TG-WP-N</t>
+        </is>
+      </c>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
           <t>RedmiTurbo 4 Pro Tempered Glass Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr">
-        <is>
-          <t>T4P-TG-WP-N</t>
-        </is>
-      </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>White Print</t>
         </is>
       </c>
-      <c r="E11" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F11" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G11" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H11" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr"/>
+      <c r="I11" s="7" t="inlineStr"/>
       <c r="J11" s="8" t="n">
         <v>133</v>
       </c>
@@ -1402,45 +1402,45 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
+          <t>T4P-TG-WP-N</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
           <t>RedmiTurbo 4 Pro Tempered Glass Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
-        <is>
-          <t>T4P-TG-WP-N</t>
-        </is>
-      </c>
-      <c r="C12" s="3" t="inlineStr">
+      <c r="C12" s="2" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D12" s="3" t="inlineStr">
+      <c r="D12" s="2" t="inlineStr">
         <is>
           <t>White Print</t>
         </is>
       </c>
-      <c r="E12" s="3" t="inlineStr">
+      <c r="E12" s="2" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F12" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G12" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H12" s="2" t="inlineStr">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H12" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I12" s="2" t="inlineStr"/>
+      <c r="I12" s="3" t="inlineStr"/>
       <c r="J12" s="4" t="n">
         <v>133</v>
       </c>
@@ -1482,45 +1482,45 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
+          <t>T4P-TG-WP-N</t>
+        </is>
+      </c>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr">
-        <is>
-          <t>T4P-TG-WP-N</t>
-        </is>
-      </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C13" s="6" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D13" s="7" t="inlineStr">
+      <c r="D13" s="6" t="inlineStr">
         <is>
           <t>White Print</t>
         </is>
       </c>
-      <c r="E13" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F13" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G13" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H13" s="6" t="inlineStr">
+      <c r="F13" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G13" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H13" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr"/>
+      <c r="I13" s="7" t="inlineStr"/>
       <c r="J13" s="8" t="n">
         <v>133</v>
       </c>
@@ -1562,45 +1562,45 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
+          <t>T4P-TG-WP-N</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Case – White Glass Shell</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
-        <is>
-          <t>T4P-TG-WP-N</t>
-        </is>
-      </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C14" s="2" t="inlineStr">
         <is>
           <t>Tempered glass</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D14" s="2" t="inlineStr">
         <is>
           <t>White Print</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E14" s="2" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G14" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H14" s="2" t="inlineStr">
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000HHR0RE2BI-jit-one-piece-dropshippingsuitable-for-xiaomi17-phone-case-aliexpress-f7-mercado-libre-turbo4-foreign-trade/1AD8397614601637</t>
         </is>
       </c>
-      <c r="I14" s="2" t="inlineStr"/>
+      <c r="I14" s="3" t="inlineStr"/>
       <c r="J14" s="4" t="n">
         <v>133</v>
       </c>
@@ -1642,45 +1642,45 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
+          <t>H600-SKn-G-N</t>
+        </is>
+      </c>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
           <t>Honor 600 Skin Protective Case</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr">
-        <is>
-          <t>H600-SKn-G-N</t>
-        </is>
-      </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
         <is>
           <t>Skin</t>
         </is>
       </c>
-      <c r="D15" s="7" t="inlineStr">
+      <c r="D15" s="6" t="inlineStr">
         <is>
           <t>Grey</t>
         </is>
       </c>
-      <c r="E15" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>Honor 600</t>
         </is>
       </c>
-      <c r="F15" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G15" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H15" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/000000074X6RUVK3-suitable-for-honor-600-phone-case-honor-600-pro-international-version-carbon-fiber-pattern-leather-protective-cover-back-shell-type/1AD8348014988676</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
+      <c r="I15" s="7" t="inlineStr"/>
       <c r="J15" s="8" t="n">
         <v>146.3</v>
       </c>
@@ -1722,45 +1722,45 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
+          <t>H600P-SKn-G-N</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
           <t>Honor 600 Pro Skin Protective Case</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr">
-        <is>
-          <t>H600P-SKn-G-N</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr">
+      <c r="C16" s="2" t="inlineStr">
         <is>
           <t>Skin</t>
         </is>
       </c>
-      <c r="D16" s="3" t="inlineStr">
+      <c r="D16" s="2" t="inlineStr">
         <is>
           <t>Grey</t>
         </is>
       </c>
-      <c r="E16" s="3" t="inlineStr">
+      <c r="E16" s="2" t="inlineStr">
         <is>
           <t>Honor 600 Pro</t>
         </is>
       </c>
-      <c r="F16" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G16" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H16" s="2" t="inlineStr">
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/000000074X6RUVK3-suitable-for-honor-600-phone-case-honor-600-pro-international-version-carbon-fiber-pattern-leather-protective-cover-back-shell-type/1AD8348014988676</t>
         </is>
       </c>
-      <c r="I16" s="2" t="inlineStr"/>
+      <c r="I16" s="3" t="inlineStr"/>
       <c r="J16" s="4" t="n">
         <v>146.3</v>
       </c>
@@ -1802,45 +1802,45 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
+          <t>S26U-PW-B-N</t>
+        </is>
+      </c>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
           <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
-        <is>
-          <t>S26U-PW-B-N</t>
-        </is>
-      </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D17" s="7" t="inlineStr">
+      <c r="D17" s="6" t="inlineStr">
         <is>
           <t>Poplar Wood Grain</t>
         </is>
       </c>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
-      <c r="F17" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G17" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H17" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr"/>
+      <c r="I17" s="7" t="inlineStr"/>
       <c r="J17" s="8" t="n">
         <v>252.7</v>
       </c>
@@ -1882,45 +1882,45 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
+          <t>S26U-PW-B-N</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
           <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>S26U-PW-B-N</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
+      <c r="C18" s="2" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D18" s="3" t="inlineStr">
+      <c r="D18" s="2" t="inlineStr">
         <is>
           <t>Dark Gray Wood Grain</t>
         </is>
       </c>
-      <c r="E18" s="3" t="inlineStr">
+      <c r="E18" s="2" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
-      <c r="F18" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G18" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H18" s="2" t="inlineStr">
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
         </is>
       </c>
-      <c r="I18" s="2" t="inlineStr"/>
+      <c r="I18" s="3" t="inlineStr"/>
       <c r="J18" s="4" t="n">
         <v>252.7</v>
       </c>
@@ -1962,45 +1962,45 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
+          <t>S26U-MI-B-N</t>
+        </is>
+      </c>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
           <t>Samsung Galaxy S26 Ultra Magnetic Invisible Bracket</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr">
-        <is>
-          <t>S26U-MI-B-N</t>
-        </is>
-      </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C19" s="6" t="inlineStr">
         <is>
           <t>Metal lens frame Acrylic / TPU</t>
         </is>
       </c>
-      <c r="D19" s="7" t="inlineStr">
+      <c r="D19" s="6" t="inlineStr">
         <is>
           <t>Black – Magnetic Invisible Bracket</t>
         </is>
       </c>
-      <c r="E19" s="7" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G19" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H19" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000PWJ01ZSK1-metal-invisible-lens-bracket-suitable-for-samsung-s26ultra-magnetic-phone-case-s25fe-transparent-s24plus-case/1AC5307428543960</t>
         </is>
       </c>
-      <c r="I19" s="6" t="inlineStr"/>
+      <c r="I19" s="7" t="inlineStr"/>
       <c r="J19" s="8" t="n">
         <v>265.74</v>
       </c>
@@ -2042,45 +2042,45 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
+          <t>18P-AC-M-R-N</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
           <t>iPhone 18 Pro Magnetic Acrylic Case</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>18P-AC-M-R-N</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C20" s="2" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D20" s="3" t="inlineStr">
+      <c r="D20" s="2" t="inlineStr">
         <is>
           <t>Wine Red</t>
         </is>
       </c>
-      <c r="E20" s="3" t="inlineStr">
+      <c r="E20" s="2" t="inlineStr">
         <is>
           <t>iPhone 18 Pro</t>
         </is>
       </c>
-      <c r="F20" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G20" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H20" s="2" t="inlineStr">
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I20" s="2" t="inlineStr"/>
+      <c r="I20" s="3" t="inlineStr"/>
       <c r="J20" s="4" t="n">
         <v>87.25</v>
       </c>
@@ -2122,45 +2122,45 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
+          <t>18PM-AC-M-R-N</t>
+        </is>
+      </c>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
           <t>iPhone 18  Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr">
-        <is>
-          <t>18PM-AC-M-R-N</t>
-        </is>
-      </c>
-      <c r="C21" s="7" t="inlineStr">
+      <c r="C21" s="6" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D21" s="7" t="inlineStr">
+      <c r="D21" s="6" t="inlineStr">
         <is>
           <t>Wine Red</t>
         </is>
       </c>
-      <c r="E21" s="7" t="inlineStr">
+      <c r="E21" s="6" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F21" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G21" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H21" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I21" s="6" t="inlineStr"/>
+      <c r="I21" s="7" t="inlineStr"/>
       <c r="J21" s="8" t="n">
         <v>87.25</v>
       </c>
@@ -2202,45 +2202,45 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
+          <t>18PM-AC-M-B-N</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
           <t>iPhone 18  Pro  Magnetic Acrylic Case</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr">
-        <is>
-          <t>18PM-AC-M-B-N</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr">
+      <c r="C22" s="2" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D22" s="3" t="inlineStr">
+      <c r="D22" s="2" t="inlineStr">
         <is>
           <t>Black</t>
         </is>
       </c>
-      <c r="E22" s="3" t="inlineStr">
+      <c r="E22" s="2" t="inlineStr">
         <is>
           <t>iPhone 18 Pro</t>
         </is>
       </c>
-      <c r="F22" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G22" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H22" s="2" t="inlineStr">
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I22" s="2" t="inlineStr"/>
+      <c r="I22" s="3" t="inlineStr"/>
       <c r="J22" s="4" t="n">
         <v>87.25</v>
       </c>
@@ -2282,45 +2282,45 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
+          <t>17PM-AC-M-O-N</t>
+        </is>
+      </c>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
           <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr">
-        <is>
-          <t>17PM-AC-M-O-N</t>
-        </is>
-      </c>
-      <c r="C23" s="7" t="inlineStr">
+      <c r="C23" s="6" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D23" s="7" t="inlineStr">
+      <c r="D23" s="6" t="inlineStr">
         <is>
           <t>Orange</t>
         </is>
       </c>
-      <c r="E23" s="7" t="inlineStr">
+      <c r="E23" s="6" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max</t>
         </is>
       </c>
-      <c r="F23" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G23" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H23" s="6" t="inlineStr">
+      <c r="F23" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G23" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H23" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I23" s="6" t="inlineStr"/>
+      <c r="I23" s="7" t="inlineStr"/>
       <c r="J23" s="8" t="n">
         <v>87.25</v>
       </c>
@@ -2362,45 +2362,45 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
+          <t>17PM-AC-M-PK-N</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
           <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t>17PM-AC-M-PK-N</t>
-        </is>
-      </c>
-      <c r="C24" s="3" t="inlineStr">
+      <c r="C24" s="2" t="inlineStr">
         <is>
           <t>Acrylic</t>
         </is>
       </c>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="2" t="inlineStr">
         <is>
           <t>Pink</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr">
+      <c r="E24" s="2" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max</t>
         </is>
       </c>
-      <c r="F24" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G24" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H24" s="2" t="inlineStr">
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
-      <c r="I24" s="2" t="inlineStr"/>
+      <c r="I24" s="3" t="inlineStr"/>
       <c r="J24" s="4" t="n">
         <v>87.25</v>
       </c>
@@ -2442,45 +2442,45 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
+          <t>18PM-HS-S-N</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
           <t>iPhone 18 Pro Max Hard Shell Case with Lens Film</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr">
-        <is>
-          <t>18PM-HS-S-N</t>
-        </is>
-      </c>
-      <c r="C25" s="7" t="inlineStr">
+      <c r="C25" s="6" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D25" s="7" t="inlineStr">
+      <c r="D25" s="6" t="inlineStr">
         <is>
           <t>Elegant Silver</t>
         </is>
       </c>
-      <c r="E25" s="7" t="inlineStr">
+      <c r="E25" s="6" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max</t>
         </is>
       </c>
-      <c r="F25" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G25" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H25" s="6" t="inlineStr">
+      <c r="F25" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G25" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H25" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I25" s="6" t="inlineStr"/>
+      <c r="I25" s="7" t="inlineStr"/>
       <c r="J25" s="8" t="n">
         <v>119.7</v>
       </c>
@@ -2522,45 +2522,45 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
+          <t>18P-HS-S-N</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
           <t>iPhone 18 Pro Hard Shell Case with Lens Film</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr">
-        <is>
-          <t>18P-HS-S-N</t>
-        </is>
-      </c>
-      <c r="C26" s="3" t="inlineStr">
+      <c r="C26" s="2" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D26" s="3" t="inlineStr">
+      <c r="D26" s="2" t="inlineStr">
         <is>
           <t>Elegant Silver</t>
         </is>
       </c>
-      <c r="E26" s="3" t="inlineStr">
+      <c r="E26" s="2" t="inlineStr">
         <is>
           <t>iPhone 18 Pro</t>
         </is>
       </c>
-      <c r="F26" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G26" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H26" s="2" t="inlineStr">
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I26" s="2" t="inlineStr"/>
+      <c r="I26" s="3" t="inlineStr"/>
       <c r="J26" s="4" t="n">
         <v>119.7</v>
       </c>
@@ -2602,45 +2602,45 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
+          <t>17PM-HS-S-N</t>
+        </is>
+      </c>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
           <t>iPhone 17 Pro Max Hard Shell Case with Lens Film</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr">
-        <is>
-          <t>17PM-HS-S-N</t>
-        </is>
-      </c>
-      <c r="C27" s="7" t="inlineStr">
+      <c r="C27" s="6" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D27" s="7" t="inlineStr">
+      <c r="D27" s="6" t="inlineStr">
         <is>
           <t>Elegant Silver</t>
         </is>
       </c>
-      <c r="E27" s="7" t="inlineStr">
+      <c r="E27" s="6" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max</t>
         </is>
       </c>
-      <c r="F27" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G27" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H27" s="6" t="inlineStr">
+      <c r="F27" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G27" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H27" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I27" s="6" t="inlineStr"/>
+      <c r="I27" s="7" t="inlineStr"/>
       <c r="J27" s="8" t="n">
         <v>119.7</v>
       </c>
@@ -2682,45 +2682,45 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
+          <t>17P-HS-S-N</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
           <t>iPhone 17 Pro Hard Shell Case with Lens Film</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr">
-        <is>
-          <t>17P-HS-S-N</t>
-        </is>
-      </c>
-      <c r="C28" s="3" t="inlineStr">
+      <c r="C28" s="2" t="inlineStr">
         <is>
           <t>PCs</t>
         </is>
       </c>
-      <c r="D28" s="3" t="inlineStr">
+      <c r="D28" s="2" t="inlineStr">
         <is>
           <t>Elegant Silver</t>
         </is>
       </c>
-      <c r="E28" s="3" t="inlineStr">
+      <c r="E28" s="2" t="inlineStr">
         <is>
           <t>iPhone 17 Pro</t>
         </is>
       </c>
-      <c r="F28" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G28" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H28" s="2" t="inlineStr">
+      <c r="F28" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G28" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
-      <c r="I28" s="2" t="inlineStr"/>
+      <c r="I28" s="3" t="inlineStr"/>
       <c r="J28" s="4" t="n">
         <v>119.7</v>
       </c>
@@ -2762,45 +2762,45 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
+          <t>RN8-SIL-WT-S</t>
+        </is>
+      </c>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr">
-        <is>
-          <t>RN8-SIL-WT-S</t>
-        </is>
-      </c>
-      <c r="C29" s="7" t="inlineStr">
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D29" s="7" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Antique White</t>
         </is>
       </c>
-      <c r="E29" s="7" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F29" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G29" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H29" s="6" t="inlineStr">
+      <c r="F29" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G29" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H29" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I29" s="6" t="inlineStr">
+      <c r="I29" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S.jpg</t>
         </is>
@@ -2846,45 +2846,45 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
+          <t>RN8-SIL-PR-S</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr">
-        <is>
-          <t>RN8-SIL-PR-S</t>
-        </is>
-      </c>
-      <c r="C30" s="3" t="inlineStr">
+      <c r="C30" s="2" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D30" s="3" t="inlineStr">
+      <c r="D30" s="2" t="inlineStr">
         <is>
           <t>Grass Purple</t>
         </is>
       </c>
-      <c r="E30" s="3" t="inlineStr">
+      <c r="E30" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F30" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G30" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H30" s="2" t="inlineStr">
+      <c r="F30" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G30" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I30" s="2" t="inlineStr">
+      <c r="I30" s="3" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
@@ -2930,45 +2930,45 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
+          <t>RN8-SIL-GN-S</t>
+        </is>
+      </c>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr">
-        <is>
-          <t>RN8-SIL-GN-S</t>
-        </is>
-      </c>
-      <c r="C31" s="7" t="inlineStr">
+      <c r="C31" s="6" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D31" s="7" t="inlineStr">
+      <c r="D31" s="6" t="inlineStr">
         <is>
           <t>Dark Night Green</t>
         </is>
       </c>
-      <c r="E31" s="7" t="inlineStr">
+      <c r="E31" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F31" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G31" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H31" s="6" t="inlineStr">
+      <c r="F31" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G31" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H31" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I31" s="6" t="inlineStr">
+      <c r="I31" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S.jpg</t>
         </is>
@@ -3014,45 +3014,45 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
+          <t>RN8-SIL-BL-S</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr">
-        <is>
-          <t>RN8-SIL-BL-S</t>
-        </is>
-      </c>
-      <c r="C32" s="3" t="inlineStr">
+      <c r="C32" s="2" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D32" s="3" t="inlineStr">
+      <c r="D32" s="2" t="inlineStr">
         <is>
           <t>Royal Blue</t>
         </is>
       </c>
-      <c r="E32" s="3" t="inlineStr">
+      <c r="E32" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F32" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G32" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H32" s="2" t="inlineStr">
+      <c r="F32" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G32" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I32" s="2" t="inlineStr">
+      <c r="I32" s="3" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S.jpg</t>
         </is>
@@ -3098,45 +3098,45 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
+          <t>RN8-SIL-BK-S</t>
+        </is>
+      </c>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr">
-        <is>
-          <t>RN8-SIL-BK-S</t>
-        </is>
-      </c>
-      <c r="C33" s="7" t="inlineStr">
+      <c r="C33" s="6" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D33" s="7" t="inlineStr">
+      <c r="D33" s="6" t="inlineStr">
         <is>
           <t>Classic Black</t>
         </is>
       </c>
-      <c r="E33" s="7" t="inlineStr">
+      <c r="E33" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F33" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G33" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H33" s="6" t="inlineStr">
+      <c r="F33" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G33" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H33" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I33" s="6" t="inlineStr">
+      <c r="I33" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S.jpg</t>
         </is>
@@ -3182,45 +3182,45 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
+          <t>RN8-SIL-PR-S</t>
+        </is>
+      </c>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr">
-        <is>
-          <t>RN8-SIL-PR-S</t>
-        </is>
-      </c>
-      <c r="C34" s="3" t="inlineStr">
+      <c r="C34" s="2" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D34" s="3" t="inlineStr">
+      <c r="D34" s="2" t="inlineStr">
         <is>
           <t>Lavender Gray</t>
         </is>
       </c>
-      <c r="E34" s="3" t="inlineStr">
+      <c r="E34" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F34" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G34" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H34" s="2" t="inlineStr">
+      <c r="F34" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G34" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I34" s="2" t="inlineStr">
+      <c r="I34" s="3" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
         </is>
@@ -3266,45 +3266,45 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
+          <t>RN8-SIL-RD-S</t>
+        </is>
+      </c>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr">
-        <is>
-          <t>RN8-SIL-RD-S</t>
-        </is>
-      </c>
-      <c r="C35" s="7" t="inlineStr">
+      <c r="C35" s="6" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D35" s="7" t="inlineStr">
+      <c r="D35" s="6" t="inlineStr">
         <is>
           <t>Camellia Red</t>
         </is>
       </c>
-      <c r="E35" s="7" t="inlineStr">
+      <c r="E35" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F35" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G35" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H35" s="6" t="inlineStr">
+      <c r="F35" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G35" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H35" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I35" s="6" t="inlineStr">
+      <c r="I35" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-RD-S.jpg</t>
         </is>
@@ -3350,45 +3350,45 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
+          <t>RN8-SIL-TL-S</t>
+        </is>
+      </c>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr">
-        <is>
-          <t>RN8-SIL-TL-S</t>
-        </is>
-      </c>
-      <c r="C36" s="3" t="inlineStr">
+      <c r="C36" s="2" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D36" s="3" t="inlineStr">
+      <c r="D36" s="2" t="inlineStr">
         <is>
           <t>Light Teal</t>
         </is>
       </c>
-      <c r="E36" s="3" t="inlineStr">
+      <c r="E36" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F36" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G36" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H36" s="2" t="inlineStr">
+      <c r="F36" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G36" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I36" s="2" t="inlineStr">
+      <c r="I36" s="3" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-TL-S.jpg</t>
         </is>
@@ -3434,45 +3434,45 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
+          <t>RN8-SIL-CL-C</t>
+        </is>
+      </c>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr">
-        <is>
-          <t>RN8-SIL-CL-C</t>
-        </is>
-      </c>
-      <c r="C37" s="7" t="inlineStr">
+      <c r="C37" s="6" t="inlineStr">
         <is>
           <t>Liquid Silicone</t>
         </is>
       </c>
-      <c r="D37" s="7" t="inlineStr">
+      <c r="D37" s="6" t="inlineStr">
         <is>
           <t>Transparent</t>
         </is>
       </c>
-      <c r="E37" s="7" t="inlineStr">
+      <c r="E37" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F37" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G37" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H37" s="6" t="inlineStr">
+      <c r="F37" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G37" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H37" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
         </is>
       </c>
-      <c r="I37" s="6" t="inlineStr">
+      <c r="I37" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-CL-C.jpg</t>
         </is>
@@ -3518,45 +3518,45 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
+          <t>RN8-TPU-WT-M</t>
+        </is>
+      </c>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr">
-        <is>
-          <t>RN8-TPU-WT-M</t>
-        </is>
-      </c>
-      <c r="C38" s="3" t="inlineStr">
+      <c r="C38" s="2" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D38" s="3" t="inlineStr">
+      <c r="D38" s="2" t="inlineStr">
         <is>
           <t>Transparent White</t>
         </is>
       </c>
-      <c r="E38" s="3" t="inlineStr">
+      <c r="E38" s="2" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F38" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G38" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H38" s="2" t="inlineStr">
+      <c r="F38" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G38" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
         </is>
       </c>
-      <c r="I38" s="2" t="inlineStr">
+      <c r="I38" s="3" t="inlineStr">
         <is>
           <t>Realme Neo8/TPU/sku/RN8-TPU-WT-M.jpg</t>
         </is>
@@ -3602,45 +3602,45 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
+          <t>RN8-TPU-BK-M</t>
+        </is>
+      </c>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr">
-        <is>
-          <t>RN8-TPU-BK-M</t>
-        </is>
-      </c>
-      <c r="C39" s="7" t="inlineStr">
+      <c r="C39" s="6" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D39" s="7" t="inlineStr">
+      <c r="D39" s="6" t="inlineStr">
         <is>
           <t>Transparent Black</t>
         </is>
       </c>
-      <c r="E39" s="7" t="inlineStr">
+      <c r="E39" s="6" t="inlineStr">
         <is>
           <t>Realme Neo8</t>
         </is>
       </c>
-      <c r="F39" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G39" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H39" s="6" t="inlineStr">
+      <c r="F39" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G39" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H39" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
         </is>
       </c>
-      <c r="I39" s="6" t="inlineStr">
+      <c r="I39" s="7" t="inlineStr">
         <is>
           <t>Realme Neo8/TPU/sku/RN8-TPU-BK-M.jpg</t>
         </is>
@@ -3686,45 +3686,45 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
+          <t>H600L-SIL-BK-M</t>
+        </is>
+      </c>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr">
-        <is>
-          <t>H600L-SIL-BK-M</t>
-        </is>
-      </c>
-      <c r="C40" s="3" t="inlineStr">
+      <c r="C40" s="2" t="inlineStr">
         <is>
           <t>Silicone</t>
         </is>
       </c>
-      <c r="D40" s="3" t="inlineStr">
+      <c r="D40" s="2" t="inlineStr">
         <is>
           <t>Moiré Black</t>
         </is>
       </c>
-      <c r="E40" s="3" t="inlineStr">
+      <c r="E40" s="2" t="inlineStr">
         <is>
           <t>Honor 600 lite</t>
         </is>
       </c>
-      <c r="F40" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G40" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H40" s="2" t="inlineStr">
+      <c r="F40" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G40" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
         </is>
       </c>
-      <c r="I40" s="2" t="inlineStr">
+      <c r="I40" s="3" t="inlineStr">
         <is>
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-BK-M.jpg</t>
         </is>
@@ -3770,45 +3770,45 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
+          <t>H600L-SIL-BL-M</t>
+        </is>
+      </c>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr">
-        <is>
-          <t>H600L-SIL-BL-M</t>
-        </is>
-      </c>
-      <c r="C41" s="7" t="inlineStr">
+      <c r="C41" s="6" t="inlineStr">
         <is>
           <t>Silicone</t>
         </is>
       </c>
-      <c r="D41" s="7" t="inlineStr">
+      <c r="D41" s="6" t="inlineStr">
         <is>
           <t>Gentleman Blue</t>
         </is>
       </c>
-      <c r="E41" s="7" t="inlineStr">
+      <c r="E41" s="6" t="inlineStr">
         <is>
           <t>Honor 600 lite</t>
         </is>
       </c>
-      <c r="F41" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G41" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H41" s="6" t="inlineStr">
+      <c r="F41" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G41" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H41" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
         </is>
       </c>
-      <c r="I41" s="6" t="inlineStr">
+      <c r="I41" s="7" t="inlineStr">
         <is>
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-BL-M.jpg</t>
         </is>
@@ -3854,45 +3854,45 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
+          <t>H600L-SIL-GN-M</t>
+        </is>
+      </c>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr">
-        <is>
-          <t>H600L-SIL-GN-M</t>
-        </is>
-      </c>
-      <c r="C42" s="3" t="inlineStr">
+      <c r="C42" s="2" t="inlineStr">
         <is>
           <t>Silicone</t>
         </is>
       </c>
-      <c r="D42" s="3" t="inlineStr">
+      <c r="D42" s="2" t="inlineStr">
         <is>
           <t>Dark Night Green</t>
         </is>
       </c>
-      <c r="E42" s="3" t="inlineStr">
+      <c r="E42" s="2" t="inlineStr">
         <is>
           <t>Honor 600 lite</t>
         </is>
       </c>
-      <c r="F42" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G42" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H42" s="2" t="inlineStr">
+      <c r="F42" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G42" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
         </is>
       </c>
-      <c r="I42" s="2" t="inlineStr">
+      <c r="I42" s="3" t="inlineStr">
         <is>
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-GN-M.jpg</t>
         </is>
@@ -3938,45 +3938,45 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
+          <t>H600L-SIL-RD-M</t>
+        </is>
+      </c>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr">
-        <is>
-          <t>H600L-SIL-RD-M</t>
-        </is>
-      </c>
-      <c r="C43" s="7" t="inlineStr">
+      <c r="C43" s="6" t="inlineStr">
         <is>
           <t>Silicone</t>
         </is>
       </c>
-      <c r="D43" s="7" t="inlineStr">
+      <c r="D43" s="6" t="inlineStr">
         <is>
           <t>Charming Red</t>
         </is>
       </c>
-      <c r="E43" s="7" t="inlineStr">
+      <c r="E43" s="6" t="inlineStr">
         <is>
           <t>Honor 600 lite</t>
         </is>
       </c>
-      <c r="F43" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G43" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H43" s="6" t="inlineStr">
+      <c r="F43" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G43" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H43" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
         </is>
       </c>
-      <c r="I43" s="6" t="inlineStr">
+      <c r="I43" s="7" t="inlineStr">
         <is>
           <t>Honor 600 lite/Silicone/sku/H600L-SIL-RD-M.jpg</t>
         </is>
@@ -4022,45 +4022,45 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
+          <t>HX80I-TPU-SV-E</t>
+        </is>
+      </c>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr">
-        <is>
-          <t>HX80I-TPU-SV-E</t>
-        </is>
-      </c>
-      <c r="C44" s="3" t="inlineStr">
+      <c r="C44" s="2" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D44" s="3" t="inlineStr">
+      <c r="D44" s="2" t="inlineStr">
         <is>
           <t>Silver</t>
         </is>
       </c>
-      <c r="E44" s="3" t="inlineStr">
+      <c r="E44" s="2" t="inlineStr">
         <is>
           <t>Honor X80i</t>
         </is>
       </c>
-      <c r="F44" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G44" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H44" s="2" t="inlineStr">
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
-      <c r="I44" s="2" t="inlineStr">
+      <c r="I44" s="3" t="inlineStr">
         <is>
           <t>Honor X80i/TPU/sku/HX80I-TPU-SV-E.jpg</t>
         </is>
@@ -4106,45 +4106,45 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
+          <t>HX80I-TPU-BK-E</t>
+        </is>
+      </c>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr">
-        <is>
-          <t>HX80I-TPU-BK-E</t>
-        </is>
-      </c>
-      <c r="C45" s="7" t="inlineStr">
+      <c r="C45" s="6" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D45" s="7" t="inlineStr">
+      <c r="D45" s="6" t="inlineStr">
         <is>
           <t>Black</t>
         </is>
       </c>
-      <c r="E45" s="7" t="inlineStr">
+      <c r="E45" s="6" t="inlineStr">
         <is>
           <t>Honor X80i</t>
         </is>
       </c>
-      <c r="F45" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G45" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H45" s="6" t="inlineStr">
+      <c r="F45" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G45" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H45" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
-      <c r="I45" s="6" t="inlineStr">
+      <c r="I45" s="7" t="inlineStr">
         <is>
           <t>Honor X80i/TPU/sku/HX80I-TPU-BK-E.jpg</t>
         </is>
@@ -4190,45 +4190,45 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
+          <t>HX80I-TPU-PR-E</t>
+        </is>
+      </c>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr">
-        <is>
-          <t>HX80I-TPU-PR-E</t>
-        </is>
-      </c>
-      <c r="C46" s="3" t="inlineStr">
+      <c r="C46" s="2" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D46" s="3" t="inlineStr">
+      <c r="D46" s="2" t="inlineStr">
         <is>
           <t>Purple</t>
         </is>
       </c>
-      <c r="E46" s="3" t="inlineStr">
+      <c r="E46" s="2" t="inlineStr">
         <is>
           <t>Honor X80i</t>
         </is>
       </c>
-      <c r="F46" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G46" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H46" s="2" t="inlineStr">
+      <c r="F46" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G46" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
-      <c r="I46" s="2" t="inlineStr">
+      <c r="I46" s="3" t="inlineStr">
         <is>
           <t>Honor X80i/TPU/sku/HX80I-TPU-PR-E.jpg</t>
         </is>
@@ -4274,45 +4274,45 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
+          <t>HX80I-TPU-BL-E</t>
+        </is>
+      </c>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr">
-        <is>
-          <t>HX80I-TPU-BL-E</t>
-        </is>
-      </c>
-      <c r="C47" s="7" t="inlineStr">
+      <c r="C47" s="6" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D47" s="7" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>Blue</t>
         </is>
       </c>
-      <c r="E47" s="7" t="inlineStr">
+      <c r="E47" s="6" t="inlineStr">
         <is>
           <t>Honor X80i</t>
         </is>
       </c>
-      <c r="F47" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G47" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H47" s="6" t="inlineStr">
+      <c r="F47" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G47" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H47" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
-      <c r="I47" s="6" t="inlineStr">
+      <c r="I47" s="7" t="inlineStr">
         <is>
           <t>Honor X80i/TPU/sku/HX80I-TPU-BL-E.jpg</t>
         </is>
@@ -4358,45 +4358,45 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
+          <t>HX80I-TPU-PK-E</t>
+        </is>
+      </c>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr">
-        <is>
-          <t>HX80I-TPU-PK-E</t>
-        </is>
-      </c>
-      <c r="C48" s="3" t="inlineStr">
+      <c r="C48" s="2" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D48" s="3" t="inlineStr">
+      <c r="D48" s="2" t="inlineStr">
         <is>
           <t>Pink</t>
         </is>
       </c>
-      <c r="E48" s="3" t="inlineStr">
+      <c r="E48" s="2" t="inlineStr">
         <is>
           <t>Honor X80i</t>
         </is>
       </c>
-      <c r="F48" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G48" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H48" s="2" t="inlineStr">
+      <c r="F48" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G48" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H48" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
-      <c r="I48" s="2" t="inlineStr">
+      <c r="I48" s="3" t="inlineStr">
         <is>
           <t>Honor X80i/TPU/sku/HX80I-TPU-PK-E.jpg</t>
         </is>
@@ -4442,45 +4442,45 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
+          <t>HX80I-TPU-GN-E</t>
+        </is>
+      </c>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr">
-        <is>
-          <t>HX80I-TPU-GN-E</t>
-        </is>
-      </c>
-      <c r="C49" s="7" t="inlineStr">
+      <c r="C49" s="6" t="inlineStr">
         <is>
           <t>TPU</t>
         </is>
       </c>
-      <c r="D49" s="7" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>Green</t>
         </is>
       </c>
-      <c r="E49" s="7" t="inlineStr">
+      <c r="E49" s="6" t="inlineStr">
         <is>
           <t>Honor X80i</t>
         </is>
       </c>
-      <c r="F49" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G49" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H49" s="6" t="inlineStr">
+      <c r="F49" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G49" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H49" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
-      <c r="I49" s="6" t="inlineStr">
+      <c r="I49" s="7" t="inlineStr">
         <is>
           <t>Honor X80i/TPU/sku/HX80I-TPU-GN-E.jpg</t>
         </is>
@@ -4526,45 +4526,45 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
+          <t>HX80I-PC-GY-M</t>
+        </is>
+      </c>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr">
-        <is>
-          <t>HX80I-PC-GY-M</t>
-        </is>
-      </c>
-      <c r="C50" s="3" t="inlineStr">
+      <c r="C50" s="2" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D50" s="3" t="inlineStr">
+      <c r="D50" s="2" t="inlineStr">
         <is>
           <t>Titanium Gray</t>
         </is>
       </c>
-      <c r="E50" s="3" t="inlineStr">
+      <c r="E50" s="2" t="inlineStr">
         <is>
           <t>Honor x80i</t>
         </is>
       </c>
-      <c r="F50" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G50" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H50" s="2" t="inlineStr">
+      <c r="F50" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G50" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H50" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I50" s="2" t="inlineStr">
+      <c r="I50" s="3" t="inlineStr">
         <is>
           <t>Honor x80i/Hard PC/sku/HX80I-PC-GY-M.jpg</t>
         </is>
@@ -4610,45 +4610,45 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
+          <t>HX80I-PC-WT-M</t>
+        </is>
+      </c>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr">
-        <is>
-          <t>HX80I-PC-WT-M</t>
-        </is>
-      </c>
-      <c r="C51" s="7" t="inlineStr">
+      <c r="C51" s="6" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D51" s="7" t="inlineStr">
+      <c r="D51" s="6" t="inlineStr">
         <is>
           <t>Silver White</t>
         </is>
       </c>
-      <c r="E51" s="7" t="inlineStr">
+      <c r="E51" s="6" t="inlineStr">
         <is>
           <t>Honor x80i</t>
         </is>
       </c>
-      <c r="F51" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G51" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H51" s="6" t="inlineStr">
+      <c r="F51" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G51" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H51" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I51" s="6" t="inlineStr">
+      <c r="I51" s="7" t="inlineStr">
         <is>
           <t>Honor x80i/Hard PC/sku/HX80I-PC-WT-M.jpg</t>
         </is>
@@ -4694,45 +4694,45 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
+          <t>HX80I-PC-GN-M</t>
+        </is>
+      </c>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr">
-        <is>
-          <t>HX80I-PC-GN-M</t>
-        </is>
-      </c>
-      <c r="C52" s="3" t="inlineStr">
+      <c r="C52" s="2" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D52" s="3" t="inlineStr">
+      <c r="D52" s="2" t="inlineStr">
         <is>
           <t>Feitianqing</t>
         </is>
       </c>
-      <c r="E52" s="3" t="inlineStr">
+      <c r="E52" s="2" t="inlineStr">
         <is>
           <t>Honor x80i</t>
         </is>
       </c>
-      <c r="F52" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G52" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H52" s="2" t="inlineStr">
+      <c r="F52" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G52" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H52" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I52" s="2" t="inlineStr">
+      <c r="I52" s="3" t="inlineStr">
         <is>
           <t>Honor x80i/Hard PC/sku/HX80I-PC-GN-M.jpg</t>
         </is>
@@ -4778,45 +4778,45 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
+          <t>HX80I-PC-GD-M</t>
+        </is>
+      </c>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr">
-        <is>
-          <t>HX80I-PC-GD-M</t>
-        </is>
-      </c>
-      <c r="C53" s="7" t="inlineStr">
+      <c r="C53" s="6" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D53" s="7" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>Desert Gold</t>
         </is>
       </c>
-      <c r="E53" s="7" t="inlineStr">
+      <c r="E53" s="6" t="inlineStr">
         <is>
           <t>Honor x80i</t>
         </is>
       </c>
-      <c r="F53" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G53" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H53" s="6" t="inlineStr">
+      <c r="F53" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G53" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H53" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I53" s="6" t="inlineStr">
+      <c r="I53" s="7" t="inlineStr">
         <is>
           <t>Honor x80i/Hard PC/sku/HX80I-PC-GD-M.jpg</t>
         </is>
@@ -4862,45 +4862,45 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
+          <t>HX80I-PC-BK-M</t>
+        </is>
+      </c>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr">
-        <is>
-          <t>HX80I-PC-BK-M</t>
-        </is>
-      </c>
-      <c r="C54" s="3" t="inlineStr">
+      <c r="C54" s="2" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D54" s="3" t="inlineStr">
+      <c r="D54" s="2" t="inlineStr">
         <is>
           <t>Graphite Black</t>
         </is>
       </c>
-      <c r="E54" s="3" t="inlineStr">
+      <c r="E54" s="2" t="inlineStr">
         <is>
           <t>Honor x80i</t>
         </is>
       </c>
-      <c r="F54" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G54" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H54" s="2" t="inlineStr">
+      <c r="F54" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G54" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H54" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I54" s="2" t="inlineStr">
+      <c r="I54" s="3" t="inlineStr">
         <is>
           <t>Honor x80i/Hard PC/sku/HX80I-PC-BK-M.jpg</t>
         </is>
@@ -4946,45 +4946,45 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
+          <t>H600L-PC-GY-M</t>
+        </is>
+      </c>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr">
-        <is>
-          <t>H600L-PC-GY-M</t>
-        </is>
-      </c>
-      <c r="C55" s="7" t="inlineStr">
+      <c r="C55" s="6" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D55" s="7" t="inlineStr">
+      <c r="D55" s="6" t="inlineStr">
         <is>
           <t>Titanium Gray</t>
         </is>
       </c>
-      <c r="E55" s="7" t="inlineStr">
+      <c r="E55" s="6" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version</t>
         </is>
       </c>
-      <c r="F55" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G55" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H55" s="6" t="inlineStr">
+      <c r="F55" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G55" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H55" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I55" s="6" t="inlineStr">
+      <c r="I55" s="7" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GY-M.jpg</t>
         </is>
@@ -5030,45 +5030,45 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
+          <t>H600L-PC-WT-M</t>
+        </is>
+      </c>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr">
-        <is>
-          <t>H600L-PC-WT-M</t>
-        </is>
-      </c>
-      <c r="C56" s="3" t="inlineStr">
+      <c r="C56" s="2" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D56" s="3" t="inlineStr">
+      <c r="D56" s="2" t="inlineStr">
         <is>
           <t>Silver White</t>
         </is>
       </c>
-      <c r="E56" s="3" t="inlineStr">
+      <c r="E56" s="2" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version</t>
         </is>
       </c>
-      <c r="F56" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G56" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H56" s="2" t="inlineStr">
+      <c r="F56" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G56" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H56" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I56" s="2" t="inlineStr">
+      <c r="I56" s="3" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-WT-M.jpg</t>
         </is>
@@ -5114,45 +5114,45 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
+          <t>H600L-PC-GN-M</t>
+        </is>
+      </c>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr">
-        <is>
-          <t>H600L-PC-GN-M</t>
-        </is>
-      </c>
-      <c r="C57" s="7" t="inlineStr">
+      <c r="C57" s="6" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D57" s="7" t="inlineStr">
+      <c r="D57" s="6" t="inlineStr">
         <is>
           <t>Feitianqing</t>
         </is>
       </c>
-      <c r="E57" s="7" t="inlineStr">
+      <c r="E57" s="6" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version</t>
         </is>
       </c>
-      <c r="F57" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G57" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H57" s="6" t="inlineStr">
+      <c r="F57" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G57" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H57" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I57" s="6" t="inlineStr">
+      <c r="I57" s="7" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GN-M.jpg</t>
         </is>
@@ -5198,45 +5198,45 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
+          <t>H600L-PC-GD-M</t>
+        </is>
+      </c>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr">
-        <is>
-          <t>H600L-PC-GD-M</t>
-        </is>
-      </c>
-      <c r="C58" s="3" t="inlineStr">
+      <c r="C58" s="2" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D58" s="3" t="inlineStr">
+      <c r="D58" s="2" t="inlineStr">
         <is>
           <t>Desert Gold</t>
         </is>
       </c>
-      <c r="E58" s="3" t="inlineStr">
+      <c r="E58" s="2" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version</t>
         </is>
       </c>
-      <c r="F58" s="3" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G58" s="3" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H58" s="2" t="inlineStr">
+      <c r="F58" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G58" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H58" s="3" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I58" s="2" t="inlineStr">
+      <c r="I58" s="3" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GD-M.jpg</t>
         </is>
@@ -5282,45 +5282,45 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
+          <t>H600L-PC-BK-M</t>
+        </is>
+      </c>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr">
-        <is>
-          <t>H600L-PC-BK-M</t>
-        </is>
-      </c>
-      <c r="C59" s="7" t="inlineStr">
+      <c r="C59" s="6" t="inlineStr">
         <is>
           <t>Hard PC</t>
         </is>
       </c>
-      <c r="D59" s="7" t="inlineStr">
+      <c r="D59" s="6" t="inlineStr">
         <is>
           <t>Graphite Black</t>
         </is>
       </c>
-      <c r="E59" s="7" t="inlineStr">
+      <c r="E59" s="6" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version</t>
         </is>
       </c>
-      <c r="F59" s="7" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="G59" s="7" t="inlineStr">
-        <is>
-          <t>Link</t>
-        </is>
-      </c>
-      <c r="H59" s="6" t="inlineStr">
+      <c r="F59" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G59" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H59" s="7" t="inlineStr">
         <is>
           <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
-      <c r="I59" s="6" t="inlineStr">
+      <c r="I59" s="7" t="inlineStr">
         <is>
           <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-BK-M.jpg</t>
         </is>

</xml_diff>

<commit_message>
feat: process Realme Neo8 (Hard PC) and update inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:T59"/>
+  <dimension ref="A1:T67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -5363,6 +5363,678 @@
         <v/>
       </c>
     </row>
+    <row r="60">
+      <c r="A60" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-RK-M</t>
+        </is>
+      </c>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C60" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D60" s="2" t="inlineStr">
+        <is>
+          <t>Peak Rock Color</t>
+        </is>
+      </c>
+      <c r="E60" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F60" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G60" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H60" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I60" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-RK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J60" s="4" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K60" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L60" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M60" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N60" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O60" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P60" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q60" s="4">
+        <f>SUM(J60:P60)</f>
+        <v/>
+      </c>
+      <c r="R60" s="4">
+        <f>IF(Q60&lt;300, Q60*1.4, IF(Q60&lt;400, Q60*1.33, Q60*1.25))</f>
+        <v/>
+      </c>
+      <c r="S60" s="5">
+        <f>INT(R60/100)*100 + IF(MOD(ROUND(R60,0),100)&lt;25, 0, IF(MOD(ROUND(R60,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T60" s="4">
+        <f>IF(S60&lt;300, 0, MIN(99, IF(S60&lt;500, S60*7%, IF(S60&lt;700, S60*12%, S60*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-GD-M</t>
+        </is>
+      </c>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C61" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>Desert Gold</t>
+        </is>
+      </c>
+      <c r="E61" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F61" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G61" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H61" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I61" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-GD-M.jpg</t>
+        </is>
+      </c>
+      <c r="J61" s="8" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K61" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L61" s="8" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M61" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N61" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O61" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P61" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q61" s="8">
+        <f>SUM(J61:P61)</f>
+        <v/>
+      </c>
+      <c r="R61" s="8">
+        <f>IF(Q61&lt;300, Q61*1.4, IF(Q61&lt;400, Q61*1.33, Q61*1.25))</f>
+        <v/>
+      </c>
+      <c r="S61" s="9">
+        <f>INT(R61/100)*100 + IF(MOD(ROUND(R61,0),100)&lt;25, 0, IF(MOD(ROUND(R61,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T61" s="8">
+        <f>IF(S61&lt;300, 0, MIN(99, IF(S61&lt;500, S61*7%, IF(S61&lt;700, S61*12%, S61*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-BL-M</t>
+        </is>
+      </c>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C62" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D62" s="2" t="inlineStr">
+        <is>
+          <t>Wave Blue</t>
+        </is>
+      </c>
+      <c r="E62" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F62" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G62" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H62" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I62" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-BL-M.jpg</t>
+        </is>
+      </c>
+      <c r="J62" s="4" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K62" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L62" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M62" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N62" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O62" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P62" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q62" s="4">
+        <f>SUM(J62:P62)</f>
+        <v/>
+      </c>
+      <c r="R62" s="4">
+        <f>IF(Q62&lt;300, Q62*1.4, IF(Q62&lt;400, Q62*1.33, Q62*1.25))</f>
+        <v/>
+      </c>
+      <c r="S62" s="5">
+        <f>INT(R62/100)*100 + IF(MOD(ROUND(R62,0),100)&lt;25, 0, IF(MOD(ROUND(R62,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T62" s="4">
+        <f>IF(S62&lt;300, 0, MIN(99, IF(S62&lt;500, S62*7%, IF(S62&lt;700, S62*12%, S62*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-PK-M</t>
+        </is>
+      </c>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C63" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D63" s="6" t="inlineStr">
+        <is>
+          <t>Sakura Pink</t>
+        </is>
+      </c>
+      <c r="E63" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F63" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G63" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H63" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I63" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-PK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J63" s="8" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K63" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L63" s="8" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M63" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N63" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O63" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P63" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q63" s="8">
+        <f>SUM(J63:P63)</f>
+        <v/>
+      </c>
+      <c r="R63" s="8">
+        <f>IF(Q63&lt;300, Q63*1.4, IF(Q63&lt;400, Q63*1.33, Q63*1.25))</f>
+        <v/>
+      </c>
+      <c r="S63" s="9">
+        <f>INT(R63/100)*100 + IF(MOD(ROUND(R63,0),100)&lt;25, 0, IF(MOD(ROUND(R63,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T63" s="8">
+        <f>IF(S63&lt;300, 0, MIN(99, IF(S63&lt;500, S63*7%, IF(S63&lt;700, S63*12%, S63*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-CG-M</t>
+        </is>
+      </c>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C64" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D64" s="2" t="inlineStr">
+        <is>
+          <t>Carbon Gray</t>
+        </is>
+      </c>
+      <c r="E64" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F64" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G64" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H64" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I64" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-CG-M.jpg</t>
+        </is>
+      </c>
+      <c r="J64" s="4" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K64" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L64" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M64" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N64" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O64" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P64" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q64" s="4">
+        <f>SUM(J64:P64)</f>
+        <v/>
+      </c>
+      <c r="R64" s="4">
+        <f>IF(Q64&lt;300, Q64*1.4, IF(Q64&lt;400, Q64*1.33, Q64*1.25))</f>
+        <v/>
+      </c>
+      <c r="S64" s="5">
+        <f>INT(R64/100)*100 + IF(MOD(ROUND(R64,0),100)&lt;25, 0, IF(MOD(ROUND(R64,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T64" s="4">
+        <f>IF(S64&lt;300, 0, MIN(99, IF(S64&lt;500, S64*7%, IF(S64&lt;700, S64*12%, S64*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-PR-M</t>
+        </is>
+      </c>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C65" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D65" s="6" t="inlineStr">
+        <is>
+          <t>Sunset Purple</t>
+        </is>
+      </c>
+      <c r="E65" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F65" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G65" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H65" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I65" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-PR-M.jpg</t>
+        </is>
+      </c>
+      <c r="J65" s="8" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K65" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L65" s="8" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M65" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N65" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O65" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P65" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q65" s="8">
+        <f>SUM(J65:P65)</f>
+        <v/>
+      </c>
+      <c r="R65" s="8">
+        <f>IF(Q65&lt;300, Q65*1.4, IF(Q65&lt;400, Q65*1.33, Q65*1.25))</f>
+        <v/>
+      </c>
+      <c r="S65" s="9">
+        <f>INT(R65/100)*100 + IF(MOD(ROUND(R65,0),100)&lt;25, 0, IF(MOD(ROUND(R65,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T65" s="8">
+        <f>IF(S65&lt;300, 0, MIN(99, IF(S65&lt;500, S65*7%, IF(S65&lt;700, S65*12%, S65*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-TG-M</t>
+        </is>
+      </c>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C66" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D66" s="2" t="inlineStr">
+        <is>
+          <t>Titanium Gray</t>
+        </is>
+      </c>
+      <c r="E66" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F66" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G66" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H66" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I66" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-TG-M.jpg</t>
+        </is>
+      </c>
+      <c r="J66" s="4" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K66" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="L66" s="4" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M66" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="N66" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O66" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="P66" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q66" s="4">
+        <f>SUM(J66:P66)</f>
+        <v/>
+      </c>
+      <c r="R66" s="4">
+        <f>IF(Q66&lt;300, Q66*1.4, IF(Q66&lt;400, Q66*1.33, Q66*1.25))</f>
+        <v/>
+      </c>
+      <c r="S66" s="5">
+        <f>INT(R66/100)*100 + IF(MOD(ROUND(R66,0),100)&lt;25, 0, IF(MOD(ROUND(R66,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T66" s="4">
+        <f>IF(S66&lt;300, 0, MIN(99, IF(S66&lt;500, S66*7%, IF(S66&lt;700, S66*12%, S66*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-BK-M</t>
+        </is>
+      </c>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+        </is>
+      </c>
+      <c r="C67" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="D67" s="6" t="inlineStr">
+        <is>
+          <t>Classic Black</t>
+        </is>
+      </c>
+      <c r="E67" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="F67" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="G67" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="H67" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+        </is>
+      </c>
+      <c r="I67" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-BK-M.jpg</t>
+        </is>
+      </c>
+      <c r="J67" s="8" t="n">
+        <v>367.08</v>
+      </c>
+      <c r="K67" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="L67" s="8" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="M67" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="N67" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="O67" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="P67" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q67" s="8">
+        <f>SUM(J67:P67)</f>
+        <v/>
+      </c>
+      <c r="R67" s="8">
+        <f>IF(Q67&lt;300, Q67*1.4, IF(Q67&lt;400, Q67*1.33, Q67*1.25))</f>
+        <v/>
+      </c>
+      <c r="S67" s="9">
+        <f>INT(R67/100)*100 + IF(MOD(ROUND(R67,0),100)&lt;25, 0, IF(MOD(ROUND(R67,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="T67" s="8">
+        <f>IF(S67&lt;300, 0, MIN(99, IF(S67&lt;500, S67*7%, IF(S67&lt;700, S67*12%, S67*15%))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
docs: add customer-attracting product description templates and copywriting guide
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -480,7 +480,7 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="2" max="2"/>
     <col width="48" customWidth="1" min="3" max="3"/>
     <col width="33" customWidth="1" min="4" max="4"/>
     <col width="37" customWidth="1" min="5" max="5"/>
@@ -615,7 +615,11 @@
           <t>T4P-TG-BP-N</t>
         </is>
       </c>
-      <c r="B2" s="3" t="inlineStr"/>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Luxury 9H Tempered Glass Back Cover for RedmiTurbo 4 Pro – Glossy Anti-Scratch Armor Protective Case</t>
+        </is>
+      </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Protective Case – White Glass Shell</t>
@@ -674,19 +678,19 @@
         <v>0</v>
       </c>
       <c r="R2" s="4">
-        <f>SUM(J2:P2)</f>
+        <f>SUM(K2:Q2)</f>
         <v/>
       </c>
       <c r="S2" s="4">
-        <f>IF(Q2&lt;300, Q2*1.4, IF(Q2&lt;400, Q2*1.33, Q2*1.25))</f>
+        <f>IF(R2&lt;300, R2*1.4, IF(R2&lt;400, R2*1.33, R2*1.25))</f>
         <v/>
       </c>
       <c r="T2" s="5">
-        <f>INT(R2/100)*100 + IF(MOD(ROUND(R2,0),100)&lt;25, 0, IF(MOD(ROUND(R2,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S2/100)*100 + IF(MOD(ROUND(S2,0),100)&lt;25, 0, IF(MOD(ROUND(S2,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U2" s="4">
-        <f>IF(S2&lt;300, 0, MIN(99, IF(S2&lt;500, S2*7%, IF(S2&lt;700, S2*12%, S2*15%))))</f>
+        <f>IF(T2&lt;300, 0, MIN(99, IF(T2&lt;500, T2*7%, IF(T2&lt;700, T2*12%, T2*15%))))</f>
         <v/>
       </c>
     </row>
@@ -696,7 +700,11 @@
           <t>18PM-TPUM-CR-N</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr"/>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Clear Shockproof TPU Case with Lens Film for iPhone 18 Pro Max – Full Protection Slim Soft Cover</t>
+        </is>
+      </c>
       <c r="C3" s="7" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max Phone Case, Magnetic, Transparent, with Lens Film</t>
@@ -755,19 +763,19 @@
         <v>0</v>
       </c>
       <c r="R3" s="8">
-        <f>SUM(J3:P3)</f>
+        <f>SUM(K3:Q3)</f>
         <v/>
       </c>
       <c r="S3" s="8">
-        <f>IF(Q3&lt;300, Q3*1.4, IF(Q3&lt;400, Q3*1.33, Q3*1.25))</f>
+        <f>IF(R3&lt;300, R3*1.4, IF(R3&lt;400, R3*1.33, R3*1.25))</f>
         <v/>
       </c>
       <c r="T3" s="9">
-        <f>INT(R3/100)*100 + IF(MOD(ROUND(R3,0),100)&lt;25, 0, IF(MOD(ROUND(R3,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S3/100)*100 + IF(MOD(ROUND(S3,0),100)&lt;25, 0, IF(MOD(ROUND(S3,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U3" s="8">
-        <f>IF(S3&lt;300, 0, MIN(99, IF(S3&lt;500, S3*7%, IF(S3&lt;700, S3*12%, S3*15%))))</f>
+        <f>IF(T3&lt;300, 0, MIN(99, IF(T3&lt;500, T3*7%, IF(T3&lt;700, T3*12%, T3*15%))))</f>
         <v/>
       </c>
     </row>
@@ -777,7 +785,11 @@
           <t>18PM-TPUM-SB-N</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr"/>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Clear Shockproof TPU Case with Lens Film for iPhone 18 Pro Max – Full Protection Slim Soft Cover</t>
+        </is>
+      </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max Phone Case, Magnetic, Transparent, with Lens Film</t>
@@ -836,19 +848,19 @@
         <v>0</v>
       </c>
       <c r="R4" s="4">
-        <f>SUM(J4:P4)</f>
+        <f>SUM(K4:Q4)</f>
         <v/>
       </c>
       <c r="S4" s="4">
-        <f>IF(Q4&lt;300, Q4*1.4, IF(Q4&lt;400, Q4*1.33, Q4*1.25))</f>
+        <f>IF(R4&lt;300, R4*1.4, IF(R4&lt;400, R4*1.33, R4*1.25))</f>
         <v/>
       </c>
       <c r="T4" s="5">
-        <f>INT(R4/100)*100 + IF(MOD(ROUND(R4,0),100)&lt;25, 0, IF(MOD(ROUND(R4,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S4/100)*100 + IF(MOD(ROUND(S4,0),100)&lt;25, 0, IF(MOD(ROUND(S4,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U4" s="4">
-        <f>IF(S4&lt;300, 0, MIN(99, IF(S4&lt;500, S4*7%, IF(S4&lt;700, S4*12%, S4*15%))))</f>
+        <f>IF(T4&lt;300, 0, MIN(99, IF(T4&lt;500, T4*7%, IF(T4&lt;700, T4*12%, T4*15%))))</f>
         <v/>
       </c>
     </row>
@@ -858,7 +870,11 @@
           <t>T4P-AC-BG-N</t>
         </is>
       </c>
-      <c r="B5" s="7" t="inlineStr"/>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Mecha Armor Shockproof Matte Case for Redmi Turbo 4 Pro – Heavy Duty Acrylic Bumper Back Cover</t>
+        </is>
+      </c>
       <c r="C5" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Mecha style acrylic matte finish case</t>
@@ -917,19 +933,19 @@
         <v>0</v>
       </c>
       <c r="R5" s="8">
-        <f>SUM(J5:P5)</f>
+        <f>SUM(K5:Q5)</f>
         <v/>
       </c>
       <c r="S5" s="8">
-        <f>IF(Q5&lt;300, Q5*1.4, IF(Q5&lt;400, Q5*1.33, Q5*1.25))</f>
+        <f>IF(R5&lt;300, R5*1.4, IF(R5&lt;400, R5*1.33, R5*1.25))</f>
         <v/>
       </c>
       <c r="T5" s="9">
-        <f>INT(R5/100)*100 + IF(MOD(ROUND(R5,0),100)&lt;25, 0, IF(MOD(ROUND(R5,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S5/100)*100 + IF(MOD(ROUND(S5,0),100)&lt;25, 0, IF(MOD(ROUND(S5,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U5" s="8">
-        <f>IF(S5&lt;300, 0, MIN(99, IF(S5&lt;500, S5*7%, IF(S5&lt;700, S5*12%, S5*15%))))</f>
+        <f>IF(T5&lt;300, 0, MIN(99, IF(T5&lt;500, T5*7%, IF(T5&lt;700, T5*12%, T5*15%))))</f>
         <v/>
       </c>
     </row>
@@ -939,7 +955,11 @@
           <t>T4P-AC-BR-N</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr"/>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Mecha Armor Shockproof Matte Case for Redmi Turbo 4 Pro – Heavy Duty Acrylic Bumper Back Cover</t>
+        </is>
+      </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Mecha style acrylic matte finish case</t>
@@ -998,19 +1018,19 @@
         <v>0</v>
       </c>
       <c r="R6" s="4">
-        <f>SUM(J6:P6)</f>
+        <f>SUM(K6:Q6)</f>
         <v/>
       </c>
       <c r="S6" s="4">
-        <f>IF(Q6&lt;300, Q6*1.4, IF(Q6&lt;400, Q6*1.33, Q6*1.25))</f>
+        <f>IF(R6&lt;300, R6*1.4, IF(R6&lt;400, R6*1.33, R6*1.25))</f>
         <v/>
       </c>
       <c r="T6" s="5">
-        <f>INT(R6/100)*100 + IF(MOD(ROUND(R6,0),100)&lt;25, 0, IF(MOD(ROUND(R6,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S6/100)*100 + IF(MOD(ROUND(S6,0),100)&lt;25, 0, IF(MOD(ROUND(S6,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U6" s="4">
-        <f>IF(S6&lt;300, 0, MIN(99, IF(S6&lt;500, S6*7%, IF(S6&lt;700, S6*12%, S6*15%))))</f>
+        <f>IF(T6&lt;300, 0, MIN(99, IF(T6&lt;500, T6*7%, IF(T6&lt;700, T6*12%, T6*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1020,7 +1040,11 @@
           <t>T4P-AC-BB-N</t>
         </is>
       </c>
-      <c r="B7" s="7" t="inlineStr"/>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>Mecha Armor Shockproof Matte Case for Redmi Turbo 4 Pro – Heavy Duty Acrylic Bumper Back Cover</t>
+        </is>
+      </c>
       <c r="C7" s="7" t="inlineStr">
         <is>
           <t>Redmi  Turbo4 Pro Mecha style acrylic matte finish case</t>
@@ -1079,19 +1103,19 @@
         <v>0</v>
       </c>
       <c r="R7" s="8">
-        <f>SUM(J7:P7)</f>
+        <f>SUM(K7:Q7)</f>
         <v/>
       </c>
       <c r="S7" s="8">
-        <f>IF(Q7&lt;300, Q7*1.4, IF(Q7&lt;400, Q7*1.33, Q7*1.25))</f>
+        <f>IF(R7&lt;300, R7*1.4, IF(R7&lt;400, R7*1.33, R7*1.25))</f>
         <v/>
       </c>
       <c r="T7" s="9">
-        <f>INT(R7/100)*100 + IF(MOD(ROUND(R7,0),100)&lt;25, 0, IF(MOD(ROUND(R7,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S7/100)*100 + IF(MOD(ROUND(S7,0),100)&lt;25, 0, IF(MOD(ROUND(S7,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U7" s="8">
-        <f>IF(S7&lt;300, 0, MIN(99, IF(S7&lt;500, S7*7%, IF(S7&lt;700, S7*12%, S7*15%))))</f>
+        <f>IF(T7&lt;300, 0, MIN(99, IF(T7&lt;500, T7*7%, IF(T7&lt;700, T7*12%, T7*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1101,7 +1125,11 @@
           <t>T4-AC-BR-N</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr"/>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Mecha Armor Shockproof Matte Case for Redmi Turbo 4 – Heavy Duty Acrylic Bumper Back Cover</t>
+        </is>
+      </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
           <t>Redmi Turbo  4 Mecha style acrylic matte finish case</t>
@@ -1160,19 +1188,19 @@
         <v>0</v>
       </c>
       <c r="R8" s="4">
-        <f>SUM(J8:P8)</f>
+        <f>SUM(K8:Q8)</f>
         <v/>
       </c>
       <c r="S8" s="4">
-        <f>IF(Q8&lt;300, Q8*1.4, IF(Q8&lt;400, Q8*1.33, Q8*1.25))</f>
+        <f>IF(R8&lt;300, R8*1.4, IF(R8&lt;400, R8*1.33, R8*1.25))</f>
         <v/>
       </c>
       <c r="T8" s="5">
-        <f>INT(R8/100)*100 + IF(MOD(ROUND(R8,0),100)&lt;25, 0, IF(MOD(ROUND(R8,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S8/100)*100 + IF(MOD(ROUND(S8,0),100)&lt;25, 0, IF(MOD(ROUND(S8,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U8" s="4">
-        <f>IF(S8&lt;300, 0, MIN(99, IF(S8&lt;500, S8*7%, IF(S8&lt;700, S8*12%, S8*15%))))</f>
+        <f>IF(T8&lt;300, 0, MIN(99, IF(T8&lt;500, T8*7%, IF(T8&lt;700, T8*12%, T8*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1182,7 +1210,11 @@
           <t>T4-AC-BB-N</t>
         </is>
       </c>
-      <c r="B9" s="7" t="inlineStr"/>
+      <c r="B9" s="7" t="inlineStr">
+        <is>
+          <t>Mecha Armor Shockproof Matte Case for Redmi Turbo 4 – Heavy Duty Acrylic Bumper Back Cover</t>
+        </is>
+      </c>
       <c r="C9" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Mecha style acrylic matte finish case</t>
@@ -1237,19 +1269,19 @@
         <v>0</v>
       </c>
       <c r="R9" s="8">
-        <f>SUM(J9:P9)</f>
+        <f>SUM(K9:Q9)</f>
         <v/>
       </c>
       <c r="S9" s="8">
-        <f>IF(Q9&lt;300, Q9*1.4, IF(Q9&lt;400, Q9*1.33, Q9*1.25))</f>
+        <f>IF(R9&lt;300, R9*1.4, IF(R9&lt;400, R9*1.33, R9*1.25))</f>
         <v/>
       </c>
       <c r="T9" s="9">
-        <f>INT(R9/100)*100 + IF(MOD(ROUND(R9,0),100)&lt;25, 0, IF(MOD(ROUND(R9,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S9/100)*100 + IF(MOD(ROUND(S9,0),100)&lt;25, 0, IF(MOD(ROUND(S9,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U9" s="8">
-        <f>IF(S9&lt;300, 0, MIN(99, IF(S9&lt;500, S9*7%, IF(S9&lt;700, S9*12%, S9*15%))))</f>
+        <f>IF(T9&lt;300, 0, MIN(99, IF(T9&lt;500, T9*7%, IF(T9&lt;700, T9*12%, T9*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1259,7 +1291,11 @@
           <t>S26U-SI-BP-N</t>
         </is>
       </c>
-      <c r="B10" s="3" t="inlineStr"/>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>3D Spider Style Shockproof Silicone Case for Galaxy S26 Ultra – Printed Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Series Spider Style Silicone Printed Case</t>
@@ -1318,19 +1354,19 @@
         <v>0</v>
       </c>
       <c r="R10" s="4">
-        <f>SUM(J10:P10)</f>
+        <f>SUM(K10:Q10)</f>
         <v/>
       </c>
       <c r="S10" s="4">
-        <f>IF(Q10&lt;300, Q10*1.4, IF(Q10&lt;400, Q10*1.33, Q10*1.25))</f>
+        <f>IF(R10&lt;300, R10*1.4, IF(R10&lt;400, R10*1.33, R10*1.25))</f>
         <v/>
       </c>
       <c r="T10" s="5">
-        <f>INT(R10/100)*100 + IF(MOD(ROUND(R10,0),100)&lt;25, 0, IF(MOD(ROUND(R10,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S10/100)*100 + IF(MOD(ROUND(S10,0),100)&lt;25, 0, IF(MOD(ROUND(S10,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U10" s="4">
-        <f>IF(S10&lt;300, 0, MIN(99, IF(S10&lt;500, S10*7%, IF(S10&lt;700, S10*12%, S10*15%))))</f>
+        <f>IF(T10&lt;300, 0, MIN(99, IF(T10&lt;500, T10*7%, IF(T10&lt;700, T10*12%, T10*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1340,7 +1376,11 @@
           <t>T4P-TG-WP-N</t>
         </is>
       </c>
-      <c r="B11" s="7" t="inlineStr"/>
+      <c r="B11" s="7" t="inlineStr">
+        <is>
+          <t>Luxury 9H Tempered Glass Back Cover for Redmi Turbo 4 Pro – Glossy Anti-Scratch Armor Protective Case</t>
+        </is>
+      </c>
       <c r="C11" s="7" t="inlineStr">
         <is>
           <t>RedmiTurbo 4 Pro Tempered Glass Case – White Glass Shell</t>
@@ -1399,19 +1439,19 @@
         <v>0</v>
       </c>
       <c r="R11" s="8">
-        <f>SUM(J11:P11)</f>
+        <f>SUM(K11:Q11)</f>
         <v/>
       </c>
       <c r="S11" s="8">
-        <f>IF(Q11&lt;300, Q11*1.4, IF(Q11&lt;400, Q11*1.33, Q11*1.25))</f>
+        <f>IF(R11&lt;300, R11*1.4, IF(R11&lt;400, R11*1.33, R11*1.25))</f>
         <v/>
       </c>
       <c r="T11" s="9">
-        <f>INT(R11/100)*100 + IF(MOD(ROUND(R11,0),100)&lt;25, 0, IF(MOD(ROUND(R11,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S11/100)*100 + IF(MOD(ROUND(S11,0),100)&lt;25, 0, IF(MOD(ROUND(S11,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U11" s="8">
-        <f>IF(S11&lt;300, 0, MIN(99, IF(S11&lt;500, S11*7%, IF(S11&lt;700, S11*12%, S11*15%))))</f>
+        <f>IF(T11&lt;300, 0, MIN(99, IF(T11&lt;500, T11*7%, IF(T11&lt;700, T11*12%, T11*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1421,7 +1461,11 @@
           <t>T4P-TG-WP-N</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr"/>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Luxury 9H Tempered Glass Back Cover for Redmi Turbo 4 Pro – Glossy Anti-Scratch Armor Protective Case</t>
+        </is>
+      </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
           <t>RedmiTurbo 4 Pro Tempered Glass Case – White Glass Shell</t>
@@ -1480,19 +1524,19 @@
         <v>0</v>
       </c>
       <c r="R12" s="4">
-        <f>SUM(J12:P12)</f>
+        <f>SUM(K12:Q12)</f>
         <v/>
       </c>
       <c r="S12" s="4">
-        <f>IF(Q12&lt;300, Q12*1.4, IF(Q12&lt;400, Q12*1.33, Q12*1.25))</f>
+        <f>IF(R12&lt;300, R12*1.4, IF(R12&lt;400, R12*1.33, R12*1.25))</f>
         <v/>
       </c>
       <c r="T12" s="5">
-        <f>INT(R12/100)*100 + IF(MOD(ROUND(R12,0),100)&lt;25, 0, IF(MOD(ROUND(R12,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S12/100)*100 + IF(MOD(ROUND(S12,0),100)&lt;25, 0, IF(MOD(ROUND(S12,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U12" s="4">
-        <f>IF(S12&lt;300, 0, MIN(99, IF(S12&lt;500, S12*7%, IF(S12&lt;700, S12*12%, S12*15%))))</f>
+        <f>IF(T12&lt;300, 0, MIN(99, IF(T12&lt;500, T12*7%, IF(T12&lt;700, T12*12%, T12*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1502,7 +1546,11 @@
           <t>T4P-TG-WP-N</t>
         </is>
       </c>
-      <c r="B13" s="7" t="inlineStr"/>
+      <c r="B13" s="7" t="inlineStr">
+        <is>
+          <t>Luxury 9H Tempered Glass Back Cover for Redmi Turbo 4 Pro – Glossy Anti-Scratch Armor Protective Case</t>
+        </is>
+      </c>
       <c r="C13" s="7" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Case – White Glass Shell</t>
@@ -1561,19 +1609,19 @@
         <v>0</v>
       </c>
       <c r="R13" s="8">
-        <f>SUM(J13:P13)</f>
+        <f>SUM(K13:Q13)</f>
         <v/>
       </c>
       <c r="S13" s="8">
-        <f>IF(Q13&lt;300, Q13*1.4, IF(Q13&lt;400, Q13*1.33, Q13*1.25))</f>
+        <f>IF(R13&lt;300, R13*1.4, IF(R13&lt;400, R13*1.33, R13*1.25))</f>
         <v/>
       </c>
       <c r="T13" s="9">
-        <f>INT(R13/100)*100 + IF(MOD(ROUND(R13,0),100)&lt;25, 0, IF(MOD(ROUND(R13,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S13/100)*100 + IF(MOD(ROUND(S13,0),100)&lt;25, 0, IF(MOD(ROUND(S13,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U13" s="8">
-        <f>IF(S13&lt;300, 0, MIN(99, IF(S13&lt;500, S13*7%, IF(S13&lt;700, S13*12%, S13*15%))))</f>
+        <f>IF(T13&lt;300, 0, MIN(99, IF(T13&lt;500, T13*7%, IF(T13&lt;700, T13*12%, T13*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1583,7 +1631,11 @@
           <t>T4P-TG-WP-N</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Luxury 9H Tempered Glass Back Cover for Redmi Turbo 4 Pro – Glossy Anti-Scratch Armor Protective Case</t>
+        </is>
+      </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
           <t>Redmi Turbo 4 Pro Tempered Glass Case – White Glass Shell</t>
@@ -1642,19 +1694,19 @@
         <v>0</v>
       </c>
       <c r="R14" s="4">
-        <f>SUM(J14:P14)</f>
+        <f>SUM(K14:Q14)</f>
         <v/>
       </c>
       <c r="S14" s="4">
-        <f>IF(Q14&lt;300, Q14*1.4, IF(Q14&lt;400, Q14*1.33, Q14*1.25))</f>
+        <f>IF(R14&lt;300, R14*1.4, IF(R14&lt;400, R14*1.33, R14*1.25))</f>
         <v/>
       </c>
       <c r="T14" s="5">
-        <f>INT(R14/100)*100 + IF(MOD(ROUND(R14,0),100)&lt;25, 0, IF(MOD(ROUND(R14,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S14/100)*100 + IF(MOD(ROUND(S14,0),100)&lt;25, 0, IF(MOD(ROUND(S14,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U14" s="4">
-        <f>IF(S14&lt;300, 0, MIN(99, IF(S14&lt;500, S14*7%, IF(S14&lt;700, S14*12%, S14*15%))))</f>
+        <f>IF(T14&lt;300, 0, MIN(99, IF(T14&lt;500, T14*7%, IF(T14&lt;700, T14*12%, T14*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1664,7 +1716,11 @@
           <t>H600-SKn-G-N</t>
         </is>
       </c>
-      <c r="B15" s="7" t="inlineStr"/>
+      <c r="B15" s="7" t="inlineStr">
+        <is>
+          <t>Ultra-Thin Matte Skin Protective Case for Honor 600 – Lightweight Anti-Fingerprint Back Cover</t>
+        </is>
+      </c>
       <c r="C15" s="7" t="inlineStr">
         <is>
           <t>Honor 600 Skin Protective Case</t>
@@ -1723,19 +1779,19 @@
         <v>0</v>
       </c>
       <c r="R15" s="8">
-        <f>SUM(J15:P15)</f>
+        <f>SUM(K15:Q15)</f>
         <v/>
       </c>
       <c r="S15" s="8">
-        <f>IF(Q15&lt;300, Q15*1.4, IF(Q15&lt;400, Q15*1.33, Q15*1.25))</f>
+        <f>IF(R15&lt;300, R15*1.4, IF(R15&lt;400, R15*1.33, R15*1.25))</f>
         <v/>
       </c>
       <c r="T15" s="9">
-        <f>INT(R15/100)*100 + IF(MOD(ROUND(R15,0),100)&lt;25, 0, IF(MOD(ROUND(R15,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S15/100)*100 + IF(MOD(ROUND(S15,0),100)&lt;25, 0, IF(MOD(ROUND(S15,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U15" s="8">
-        <f>IF(S15&lt;300, 0, MIN(99, IF(S15&lt;500, S15*7%, IF(S15&lt;700, S15*12%, S15*15%))))</f>
+        <f>IF(T15&lt;300, 0, MIN(99, IF(T15&lt;500, T15*7%, IF(T15&lt;700, T15*12%, T15*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1745,7 +1801,11 @@
           <t>H600P-SKn-G-N</t>
         </is>
       </c>
-      <c r="B16" s="3" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Ultra-Thin Matte Skin Protective Case for Honor 600 Pro – Lightweight Anti-Fingerprint Back Cover</t>
+        </is>
+      </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
           <t>Honor 600 Pro Skin Protective Case</t>
@@ -1804,19 +1864,19 @@
         <v>0</v>
       </c>
       <c r="R16" s="4">
-        <f>SUM(J16:P16)</f>
+        <f>SUM(K16:Q16)</f>
         <v/>
       </c>
       <c r="S16" s="4">
-        <f>IF(Q16&lt;300, Q16*1.4, IF(Q16&lt;400, Q16*1.33, Q16*1.25))</f>
+        <f>IF(R16&lt;300, R16*1.4, IF(R16&lt;400, R16*1.33, R16*1.25))</f>
         <v/>
       </c>
       <c r="T16" s="5">
-        <f>INT(R16/100)*100 + IF(MOD(ROUND(R16,0),100)&lt;25, 0, IF(MOD(ROUND(R16,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S16/100)*100 + IF(MOD(ROUND(S16,0),100)&lt;25, 0, IF(MOD(ROUND(S16,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U16" s="4">
-        <f>IF(S16&lt;300, 0, MIN(99, IF(S16&lt;500, S16*7%, IF(S16&lt;700, S16*12%, S16*15%))))</f>
+        <f>IF(T16&lt;300, 0, MIN(99, IF(T16&lt;500, T16*7%, IF(T16&lt;700, T16*12%, T16*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1826,7 +1886,11 @@
           <t>S26U-PW-B-N</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr"/>
+      <c r="B17" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Wood Grain Magnetic Case for Samsung Galaxy S26 Ultra – Slim Shockproof Hard Back Cover</t>
+        </is>
+      </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
@@ -1885,19 +1949,19 @@
         <v>0</v>
       </c>
       <c r="R17" s="8">
-        <f>SUM(J17:P17)</f>
+        <f>SUM(K17:Q17)</f>
         <v/>
       </c>
       <c r="S17" s="8">
-        <f>IF(Q17&lt;300, Q17*1.4, IF(Q17&lt;400, Q17*1.33, Q17*1.25))</f>
+        <f>IF(R17&lt;300, R17*1.4, IF(R17&lt;400, R17*1.33, R17*1.25))</f>
         <v/>
       </c>
       <c r="T17" s="9">
-        <f>INT(R17/100)*100 + IF(MOD(ROUND(R17,0),100)&lt;25, 0, IF(MOD(ROUND(R17,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S17/100)*100 + IF(MOD(ROUND(S17,0),100)&lt;25, 0, IF(MOD(ROUND(S17,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U17" s="8">
-        <f>IF(S17&lt;300, 0, MIN(99, IF(S17&lt;500, S17*7%, IF(S17&lt;700, S17*12%, S17*15%))))</f>
+        <f>IF(T17&lt;300, 0, MIN(99, IF(T17&lt;500, T17*7%, IF(T17&lt;700, T17*12%, T17*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1907,7 +1971,11 @@
           <t>S26U-PW-B-N</t>
         </is>
       </c>
-      <c r="B18" s="3" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Wood Grain Magnetic Case for Samsung Galaxy S26 Ultra – Slim Shockproof Hard Back Cover</t>
+        </is>
+      </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
@@ -1966,19 +2034,19 @@
         <v>0</v>
       </c>
       <c r="R18" s="4">
-        <f>SUM(J18:P18)</f>
+        <f>SUM(K18:Q18)</f>
         <v/>
       </c>
       <c r="S18" s="4">
-        <f>IF(Q18&lt;300, Q18*1.4, IF(Q18&lt;400, Q18*1.33, Q18*1.25))</f>
+        <f>IF(R18&lt;300, R18*1.4, IF(R18&lt;400, R18*1.33, R18*1.25))</f>
         <v/>
       </c>
       <c r="T18" s="5">
-        <f>INT(R18/100)*100 + IF(MOD(ROUND(R18,0),100)&lt;25, 0, IF(MOD(ROUND(R18,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S18/100)*100 + IF(MOD(ROUND(S18,0),100)&lt;25, 0, IF(MOD(ROUND(S18,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U18" s="4">
-        <f>IF(S18&lt;300, 0, MIN(99, IF(S18&lt;500, S18*7%, IF(S18&lt;700, S18*12%, S18*15%))))</f>
+        <f>IF(T18&lt;300, 0, MIN(99, IF(T18&lt;500, T18*7%, IF(T18&lt;700, T18*12%, T18*15%))))</f>
         <v/>
       </c>
     </row>
@@ -1988,7 +2056,11 @@
           <t>S26U-MI-B-N</t>
         </is>
       </c>
-      <c r="B19" s="7" t="inlineStr"/>
+      <c r="B19" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Invisible Stand Armor Case for Samsung Galaxy S26 Ultra – Heavy Duty Metal Lens Frame Hybrid Back Cover</t>
+        </is>
+      </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
           <t>Samsung Galaxy S26 Ultra Magnetic Invisible Bracket</t>
@@ -2047,19 +2119,19 @@
         <v>0</v>
       </c>
       <c r="R19" s="8">
-        <f>SUM(J19:P19)</f>
+        <f>SUM(K19:Q19)</f>
         <v/>
       </c>
       <c r="S19" s="8">
-        <f>IF(Q19&lt;300, Q19*1.4, IF(Q19&lt;400, Q19*1.33, Q19*1.25))</f>
+        <f>IF(R19&lt;300, R19*1.4, IF(R19&lt;400, R19*1.33, R19*1.25))</f>
         <v/>
       </c>
       <c r="T19" s="9">
-        <f>INT(R19/100)*100 + IF(MOD(ROUND(R19,0),100)&lt;25, 0, IF(MOD(ROUND(R19,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S19/100)*100 + IF(MOD(ROUND(S19,0),100)&lt;25, 0, IF(MOD(ROUND(S19,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U19" s="8">
-        <f>IF(S19&lt;300, 0, MIN(99, IF(S19&lt;500, S19*7%, IF(S19&lt;700, S19*12%, S19*15%))))</f>
+        <f>IF(T19&lt;300, 0, MIN(99, IF(T19&lt;500, T19*7%, IF(T19&lt;700, T19*12%, T19*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2069,7 +2141,11 @@
           <t>18P-AC-M-R-N</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+        </is>
+      </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Magnetic Acrylic Case</t>
@@ -2128,19 +2204,19 @@
         <v>0</v>
       </c>
       <c r="R20" s="4">
-        <f>SUM(J20:P20)</f>
+        <f>SUM(K20:Q20)</f>
         <v/>
       </c>
       <c r="S20" s="4">
-        <f>IF(Q20&lt;300, Q20*1.4, IF(Q20&lt;400, Q20*1.33, Q20*1.25))</f>
+        <f>IF(R20&lt;300, R20*1.4, IF(R20&lt;400, R20*1.33, R20*1.25))</f>
         <v/>
       </c>
       <c r="T20" s="5">
-        <f>INT(R20/100)*100 + IF(MOD(ROUND(R20,0),100)&lt;25, 0, IF(MOD(ROUND(R20,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S20/100)*100 + IF(MOD(ROUND(S20,0),100)&lt;25, 0, IF(MOD(ROUND(S20,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U20" s="4">
-        <f>IF(S20&lt;300, 0, MIN(99, IF(S20&lt;500, S20*7%, IF(S20&lt;700, S20*12%, S20*15%))))</f>
+        <f>IF(T20&lt;300, 0, MIN(99, IF(T20&lt;500, T20*7%, IF(T20&lt;700, T20*12%, T20*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2150,7 +2226,11 @@
           <t>18PM-AC-M-R-N</t>
         </is>
       </c>
-      <c r="B21" s="7" t="inlineStr"/>
+      <c r="B21" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+        </is>
+      </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
           <t>iPhone 18  Pro Max Magnetic Acrylic Case</t>
@@ -2209,19 +2289,19 @@
         <v>0</v>
       </c>
       <c r="R21" s="8">
-        <f>SUM(J21:P21)</f>
+        <f>SUM(K21:Q21)</f>
         <v/>
       </c>
       <c r="S21" s="8">
-        <f>IF(Q21&lt;300, Q21*1.4, IF(Q21&lt;400, Q21*1.33, Q21*1.25))</f>
+        <f>IF(R21&lt;300, R21*1.4, IF(R21&lt;400, R21*1.33, R21*1.25))</f>
         <v/>
       </c>
       <c r="T21" s="9">
-        <f>INT(R21/100)*100 + IF(MOD(ROUND(R21,0),100)&lt;25, 0, IF(MOD(ROUND(R21,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S21/100)*100 + IF(MOD(ROUND(S21,0),100)&lt;25, 0, IF(MOD(ROUND(S21,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U21" s="8">
-        <f>IF(S21&lt;300, 0, MIN(99, IF(S21&lt;500, S21*7%, IF(S21&lt;700, S21*12%, S21*15%))))</f>
+        <f>IF(T21&lt;300, 0, MIN(99, IF(T21&lt;500, T21*7%, IF(T21&lt;700, T21*12%, T21*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2231,7 +2311,11 @@
           <t>18PM-AC-M-B-N</t>
         </is>
       </c>
-      <c r="B22" s="3" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+        </is>
+      </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
           <t>iPhone 18  Pro  Magnetic Acrylic Case</t>
@@ -2290,19 +2374,19 @@
         <v>0</v>
       </c>
       <c r="R22" s="4">
-        <f>SUM(J22:P22)</f>
+        <f>SUM(K22:Q22)</f>
         <v/>
       </c>
       <c r="S22" s="4">
-        <f>IF(Q22&lt;300, Q22*1.4, IF(Q22&lt;400, Q22*1.33, Q22*1.25))</f>
+        <f>IF(R22&lt;300, R22*1.4, IF(R22&lt;400, R22*1.33, R22*1.25))</f>
         <v/>
       </c>
       <c r="T22" s="5">
-        <f>INT(R22/100)*100 + IF(MOD(ROUND(R22,0),100)&lt;25, 0, IF(MOD(ROUND(R22,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S22/100)*100 + IF(MOD(ROUND(S22,0),100)&lt;25, 0, IF(MOD(ROUND(S22,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U22" s="4">
-        <f>IF(S22&lt;300, 0, MIN(99, IF(S22&lt;500, S22*7%, IF(S22&lt;700, S22*12%, S22*15%))))</f>
+        <f>IF(T22&lt;300, 0, MIN(99, IF(T22&lt;500, T22*7%, IF(T22&lt;700, T22*12%, T22*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2312,7 +2396,11 @@
           <t>17PM-AC-M-O-N</t>
         </is>
       </c>
-      <c r="B23" s="7" t="inlineStr"/>
+      <c r="B23" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 17 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+        </is>
+      </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
@@ -2371,19 +2459,19 @@
         <v>0</v>
       </c>
       <c r="R23" s="8">
-        <f>SUM(J23:P23)</f>
+        <f>SUM(K23:Q23)</f>
         <v/>
       </c>
       <c r="S23" s="8">
-        <f>IF(Q23&lt;300, Q23*1.4, IF(Q23&lt;400, Q23*1.33, Q23*1.25))</f>
+        <f>IF(R23&lt;300, R23*1.4, IF(R23&lt;400, R23*1.33, R23*1.25))</f>
         <v/>
       </c>
       <c r="T23" s="9">
-        <f>INT(R23/100)*100 + IF(MOD(ROUND(R23,0),100)&lt;25, 0, IF(MOD(ROUND(R23,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S23/100)*100 + IF(MOD(ROUND(S23,0),100)&lt;25, 0, IF(MOD(ROUND(S23,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U23" s="8">
-        <f>IF(S23&lt;300, 0, MIN(99, IF(S23&lt;500, S23*7%, IF(S23&lt;700, S23*12%, S23*15%))))</f>
+        <f>IF(T23&lt;300, 0, MIN(99, IF(T23&lt;500, T23*7%, IF(T23&lt;700, T23*12%, T23*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2393,7 +2481,11 @@
           <t>17PM-AC-M-PK-N</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 17 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+        </is>
+      </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
@@ -2452,19 +2544,19 @@
         <v>0</v>
       </c>
       <c r="R24" s="4">
-        <f>SUM(J24:P24)</f>
+        <f>SUM(K24:Q24)</f>
         <v/>
       </c>
       <c r="S24" s="4">
-        <f>IF(Q24&lt;300, Q24*1.4, IF(Q24&lt;400, Q24*1.33, Q24*1.25))</f>
+        <f>IF(R24&lt;300, R24*1.4, IF(R24&lt;400, R24*1.33, R24*1.25))</f>
         <v/>
       </c>
       <c r="T24" s="5">
-        <f>INT(R24/100)*100 + IF(MOD(ROUND(R24,0),100)&lt;25, 0, IF(MOD(ROUND(R24,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S24/100)*100 + IF(MOD(ROUND(S24,0),100)&lt;25, 0, IF(MOD(ROUND(S24,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U24" s="4">
-        <f>IF(S24&lt;300, 0, MIN(99, IF(S24&lt;500, S24*7%, IF(S24&lt;700, S24*12%, S24*15%))))</f>
+        <f>IF(T24&lt;300, 0, MIN(99, IF(T24&lt;500, T24*7%, IF(T24&lt;700, T24*12%, T24*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2474,7 +2566,11 @@
           <t>18PM-HS-S-N</t>
         </is>
       </c>
-      <c r="B25" s="7" t="inlineStr"/>
+      <c r="B25" s="7" t="inlineStr">
+        <is>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 18 Pro Max – Luxury Anti-Scratch Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Max Hard Shell Case with Lens Film</t>
@@ -2533,19 +2629,19 @@
         <v>0</v>
       </c>
       <c r="R25" s="8">
-        <f>SUM(J25:P25)</f>
+        <f>SUM(K25:Q25)</f>
         <v/>
       </c>
       <c r="S25" s="8">
-        <f>IF(Q25&lt;300, Q25*1.4, IF(Q25&lt;400, Q25*1.33, Q25*1.25))</f>
+        <f>IF(R25&lt;300, R25*1.4, IF(R25&lt;400, R25*1.33, R25*1.25))</f>
         <v/>
       </c>
       <c r="T25" s="9">
-        <f>INT(R25/100)*100 + IF(MOD(ROUND(R25,0),100)&lt;25, 0, IF(MOD(ROUND(R25,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S25/100)*100 + IF(MOD(ROUND(S25,0),100)&lt;25, 0, IF(MOD(ROUND(S25,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U25" s="8">
-        <f>IF(S25&lt;300, 0, MIN(99, IF(S25&lt;500, S25*7%, IF(S25&lt;700, S25*12%, S25*15%))))</f>
+        <f>IF(T25&lt;300, 0, MIN(99, IF(T25&lt;500, T25*7%, IF(T25&lt;700, T25*12%, T25*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2555,7 +2651,11 @@
           <t>18P-HS-S-N</t>
         </is>
       </c>
-      <c r="B26" s="3" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 18 Pro – Luxury Anti-Scratch Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
           <t>iPhone 18 Pro Hard Shell Case with Lens Film</t>
@@ -2614,19 +2714,19 @@
         <v>0</v>
       </c>
       <c r="R26" s="4">
-        <f>SUM(J26:P26)</f>
+        <f>SUM(K26:Q26)</f>
         <v/>
       </c>
       <c r="S26" s="4">
-        <f>IF(Q26&lt;300, Q26*1.4, IF(Q26&lt;400, Q26*1.33, Q26*1.25))</f>
+        <f>IF(R26&lt;300, R26*1.4, IF(R26&lt;400, R26*1.33, R26*1.25))</f>
         <v/>
       </c>
       <c r="T26" s="5">
-        <f>INT(R26/100)*100 + IF(MOD(ROUND(R26,0),100)&lt;25, 0, IF(MOD(ROUND(R26,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S26/100)*100 + IF(MOD(ROUND(S26,0),100)&lt;25, 0, IF(MOD(ROUND(S26,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U26" s="4">
-        <f>IF(S26&lt;300, 0, MIN(99, IF(S26&lt;500, S26*7%, IF(S26&lt;700, S26*12%, S26*15%))))</f>
+        <f>IF(T26&lt;300, 0, MIN(99, IF(T26&lt;500, T26*7%, IF(T26&lt;700, T26*12%, T26*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2636,7 +2736,11 @@
           <t>17PM-HS-S-N</t>
         </is>
       </c>
-      <c r="B27" s="7" t="inlineStr"/>
+      <c r="B27" s="7" t="inlineStr">
+        <is>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 17 Pro Max – Luxury Anti-Scratch Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Max Hard Shell Case with Lens Film</t>
@@ -2695,19 +2799,19 @@
         <v>0</v>
       </c>
       <c r="R27" s="8">
-        <f>SUM(J27:P27)</f>
+        <f>SUM(K27:Q27)</f>
         <v/>
       </c>
       <c r="S27" s="8">
-        <f>IF(Q27&lt;300, Q27*1.4, IF(Q27&lt;400, Q27*1.33, Q27*1.25))</f>
+        <f>IF(R27&lt;300, R27*1.4, IF(R27&lt;400, R27*1.33, R27*1.25))</f>
         <v/>
       </c>
       <c r="T27" s="9">
-        <f>INT(R27/100)*100 + IF(MOD(ROUND(R27,0),100)&lt;25, 0, IF(MOD(ROUND(R27,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S27/100)*100 + IF(MOD(ROUND(S27,0),100)&lt;25, 0, IF(MOD(ROUND(S27,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U27" s="8">
-        <f>IF(S27&lt;300, 0, MIN(99, IF(S27&lt;500, S27*7%, IF(S27&lt;700, S27*12%, S27*15%))))</f>
+        <f>IF(T27&lt;300, 0, MIN(99, IF(T27&lt;500, T27*7%, IF(T27&lt;700, T27*12%, T27*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2717,7 +2821,11 @@
           <t>17P-HS-S-N</t>
         </is>
       </c>
-      <c r="B28" s="3" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 17 Pro – Luxury Anti-Scratch Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
           <t>iPhone 17 Pro Hard Shell Case with Lens Film</t>
@@ -2776,19 +2884,19 @@
         <v>0</v>
       </c>
       <c r="R28" s="4">
-        <f>SUM(J28:P28)</f>
+        <f>SUM(K28:Q28)</f>
         <v/>
       </c>
       <c r="S28" s="4">
-        <f>IF(Q28&lt;300, Q28*1.4, IF(Q28&lt;400, Q28*1.33, Q28*1.25))</f>
+        <f>IF(R28&lt;300, R28*1.4, IF(R28&lt;400, R28*1.33, R28*1.25))</f>
         <v/>
       </c>
       <c r="T28" s="5">
-        <f>INT(R28/100)*100 + IF(MOD(ROUND(R28,0),100)&lt;25, 0, IF(MOD(ROUND(R28,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S28/100)*100 + IF(MOD(ROUND(S28,0),100)&lt;25, 0, IF(MOD(ROUND(S28,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U28" s="4">
-        <f>IF(S28&lt;300, 0, MIN(99, IF(S28&lt;500, S28*7%, IF(S28&lt;700, S28*12%, S28*15%))))</f>
+        <f>IF(T28&lt;300, 0, MIN(99, IF(T28&lt;500, T28*7%, IF(T28&lt;700, T28*12%, T28*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2798,7 +2906,11 @@
           <t>RN8-SIL-WT-S</t>
         </is>
       </c>
-      <c r="B29" s="7" t="inlineStr"/>
+      <c r="B29" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C29" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -2861,19 +2973,19 @@
         <v>0</v>
       </c>
       <c r="R29" s="8">
-        <f>SUM(J29:P29)</f>
+        <f>SUM(K29:Q29)</f>
         <v/>
       </c>
       <c r="S29" s="8">
-        <f>IF(Q29&lt;300, Q29*1.4, IF(Q29&lt;400, Q29*1.33, Q29*1.25))</f>
+        <f>IF(R29&lt;300, R29*1.4, IF(R29&lt;400, R29*1.33, R29*1.25))</f>
         <v/>
       </c>
       <c r="T29" s="9">
-        <f>INT(R29/100)*100 + IF(MOD(ROUND(R29,0),100)&lt;25, 0, IF(MOD(ROUND(R29,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S29/100)*100 + IF(MOD(ROUND(S29,0),100)&lt;25, 0, IF(MOD(ROUND(S29,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U29" s="8">
-        <f>IF(S29&lt;300, 0, MIN(99, IF(S29&lt;500, S29*7%, IF(S29&lt;700, S29*12%, S29*15%))))</f>
+        <f>IF(T29&lt;300, 0, MIN(99, IF(T29&lt;500, T29*7%, IF(T29&lt;700, T29*12%, T29*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2883,7 +2995,11 @@
           <t>RN8-SIL-PR-S</t>
         </is>
       </c>
-      <c r="B30" s="3" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C30" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -2946,19 +3062,19 @@
         <v>0</v>
       </c>
       <c r="R30" s="4">
-        <f>SUM(J30:P30)</f>
+        <f>SUM(K30:Q30)</f>
         <v/>
       </c>
       <c r="S30" s="4">
-        <f>IF(Q30&lt;300, Q30*1.4, IF(Q30&lt;400, Q30*1.33, Q30*1.25))</f>
+        <f>IF(R30&lt;300, R30*1.4, IF(R30&lt;400, R30*1.33, R30*1.25))</f>
         <v/>
       </c>
       <c r="T30" s="5">
-        <f>INT(R30/100)*100 + IF(MOD(ROUND(R30,0),100)&lt;25, 0, IF(MOD(ROUND(R30,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S30/100)*100 + IF(MOD(ROUND(S30,0),100)&lt;25, 0, IF(MOD(ROUND(S30,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U30" s="4">
-        <f>IF(S30&lt;300, 0, MIN(99, IF(S30&lt;500, S30*7%, IF(S30&lt;700, S30*12%, S30*15%))))</f>
+        <f>IF(T30&lt;300, 0, MIN(99, IF(T30&lt;500, T30*7%, IF(T30&lt;700, T30*12%, T30*15%))))</f>
         <v/>
       </c>
     </row>
@@ -2968,7 +3084,11 @@
           <t>RN8-SIL-GN-S</t>
         </is>
       </c>
-      <c r="B31" s="7" t="inlineStr"/>
+      <c r="B31" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C31" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3031,19 +3151,19 @@
         <v>0</v>
       </c>
       <c r="R31" s="8">
-        <f>SUM(J31:P31)</f>
+        <f>SUM(K31:Q31)</f>
         <v/>
       </c>
       <c r="S31" s="8">
-        <f>IF(Q31&lt;300, Q31*1.4, IF(Q31&lt;400, Q31*1.33, Q31*1.25))</f>
+        <f>IF(R31&lt;300, R31*1.4, IF(R31&lt;400, R31*1.33, R31*1.25))</f>
         <v/>
       </c>
       <c r="T31" s="9">
-        <f>INT(R31/100)*100 + IF(MOD(ROUND(R31,0),100)&lt;25, 0, IF(MOD(ROUND(R31,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S31/100)*100 + IF(MOD(ROUND(S31,0),100)&lt;25, 0, IF(MOD(ROUND(S31,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U31" s="8">
-        <f>IF(S31&lt;300, 0, MIN(99, IF(S31&lt;500, S31*7%, IF(S31&lt;700, S31*12%, S31*15%))))</f>
+        <f>IF(T31&lt;300, 0, MIN(99, IF(T31&lt;500, T31*7%, IF(T31&lt;700, T31*12%, T31*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3053,7 +3173,11 @@
           <t>RN8-SIL-BL-S</t>
         </is>
       </c>
-      <c r="B32" s="3" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C32" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3116,19 +3240,19 @@
         <v>0</v>
       </c>
       <c r="R32" s="4">
-        <f>SUM(J32:P32)</f>
+        <f>SUM(K32:Q32)</f>
         <v/>
       </c>
       <c r="S32" s="4">
-        <f>IF(Q32&lt;300, Q32*1.4, IF(Q32&lt;400, Q32*1.33, Q32*1.25))</f>
+        <f>IF(R32&lt;300, R32*1.4, IF(R32&lt;400, R32*1.33, R32*1.25))</f>
         <v/>
       </c>
       <c r="T32" s="5">
-        <f>INT(R32/100)*100 + IF(MOD(ROUND(R32,0),100)&lt;25, 0, IF(MOD(ROUND(R32,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S32/100)*100 + IF(MOD(ROUND(S32,0),100)&lt;25, 0, IF(MOD(ROUND(S32,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U32" s="4">
-        <f>IF(S32&lt;300, 0, MIN(99, IF(S32&lt;500, S32*7%, IF(S32&lt;700, S32*12%, S32*15%))))</f>
+        <f>IF(T32&lt;300, 0, MIN(99, IF(T32&lt;500, T32*7%, IF(T32&lt;700, T32*12%, T32*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3138,7 +3262,11 @@
           <t>RN8-SIL-BK-S</t>
         </is>
       </c>
-      <c r="B33" s="7" t="inlineStr"/>
+      <c r="B33" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C33" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3201,19 +3329,19 @@
         <v>0</v>
       </c>
       <c r="R33" s="8">
-        <f>SUM(J33:P33)</f>
+        <f>SUM(K33:Q33)</f>
         <v/>
       </c>
       <c r="S33" s="8">
-        <f>IF(Q33&lt;300, Q33*1.4, IF(Q33&lt;400, Q33*1.33, Q33*1.25))</f>
+        <f>IF(R33&lt;300, R33*1.4, IF(R33&lt;400, R33*1.33, R33*1.25))</f>
         <v/>
       </c>
       <c r="T33" s="9">
-        <f>INT(R33/100)*100 + IF(MOD(ROUND(R33,0),100)&lt;25, 0, IF(MOD(ROUND(R33,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S33/100)*100 + IF(MOD(ROUND(S33,0),100)&lt;25, 0, IF(MOD(ROUND(S33,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U33" s="8">
-        <f>IF(S33&lt;300, 0, MIN(99, IF(S33&lt;500, S33*7%, IF(S33&lt;700, S33*12%, S33*15%))))</f>
+        <f>IF(T33&lt;300, 0, MIN(99, IF(T33&lt;500, T33*7%, IF(T33&lt;700, T33*12%, T33*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3223,7 +3351,11 @@
           <t>RN8-SIL-PR-S</t>
         </is>
       </c>
-      <c r="B34" s="3" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C34" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3286,19 +3418,19 @@
         <v>0</v>
       </c>
       <c r="R34" s="4">
-        <f>SUM(J34:P34)</f>
+        <f>SUM(K34:Q34)</f>
         <v/>
       </c>
       <c r="S34" s="4">
-        <f>IF(Q34&lt;300, Q34*1.4, IF(Q34&lt;400, Q34*1.33, Q34*1.25))</f>
+        <f>IF(R34&lt;300, R34*1.4, IF(R34&lt;400, R34*1.33, R34*1.25))</f>
         <v/>
       </c>
       <c r="T34" s="5">
-        <f>INT(R34/100)*100 + IF(MOD(ROUND(R34,0),100)&lt;25, 0, IF(MOD(ROUND(R34,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S34/100)*100 + IF(MOD(ROUND(S34,0),100)&lt;25, 0, IF(MOD(ROUND(S34,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U34" s="4">
-        <f>IF(S34&lt;300, 0, MIN(99, IF(S34&lt;500, S34*7%, IF(S34&lt;700, S34*12%, S34*15%))))</f>
+        <f>IF(T34&lt;300, 0, MIN(99, IF(T34&lt;500, T34*7%, IF(T34&lt;700, T34*12%, T34*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3308,7 +3440,11 @@
           <t>RN8-SIL-RD-S</t>
         </is>
       </c>
-      <c r="B35" s="7" t="inlineStr"/>
+      <c r="B35" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C35" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3371,19 +3507,19 @@
         <v>0</v>
       </c>
       <c r="R35" s="8">
-        <f>SUM(J35:P35)</f>
+        <f>SUM(K35:Q35)</f>
         <v/>
       </c>
       <c r="S35" s="8">
-        <f>IF(Q35&lt;300, Q35*1.4, IF(Q35&lt;400, Q35*1.33, Q35*1.25))</f>
+        <f>IF(R35&lt;300, R35*1.4, IF(R35&lt;400, R35*1.33, R35*1.25))</f>
         <v/>
       </c>
       <c r="T35" s="9">
-        <f>INT(R35/100)*100 + IF(MOD(ROUND(R35,0),100)&lt;25, 0, IF(MOD(ROUND(R35,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S35/100)*100 + IF(MOD(ROUND(S35,0),100)&lt;25, 0, IF(MOD(ROUND(S35,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U35" s="8">
-        <f>IF(S35&lt;300, 0, MIN(99, IF(S35&lt;500, S35*7%, IF(S35&lt;700, S35*12%, S35*15%))))</f>
+        <f>IF(T35&lt;300, 0, MIN(99, IF(T35&lt;500, T35*7%, IF(T35&lt;700, T35*12%, T35*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3393,7 +3529,11 @@
           <t>RN8-SIL-TL-S</t>
         </is>
       </c>
-      <c r="B36" s="3" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3456,19 +3596,19 @@
         <v>0</v>
       </c>
       <c r="R36" s="4">
-        <f>SUM(J36:P36)</f>
+        <f>SUM(K36:Q36)</f>
         <v/>
       </c>
       <c r="S36" s="4">
-        <f>IF(Q36&lt;300, Q36*1.4, IF(Q36&lt;400, Q36*1.33, Q36*1.25))</f>
+        <f>IF(R36&lt;300, R36*1.4, IF(R36&lt;400, R36*1.33, R36*1.25))</f>
         <v/>
       </c>
       <c r="T36" s="5">
-        <f>INT(R36/100)*100 + IF(MOD(ROUND(R36,0),100)&lt;25, 0, IF(MOD(ROUND(R36,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S36/100)*100 + IF(MOD(ROUND(S36,0),100)&lt;25, 0, IF(MOD(ROUND(S36,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U36" s="4">
-        <f>IF(S36&lt;300, 0, MIN(99, IF(S36&lt;500, S36*7%, IF(S36&lt;700, S36*12%, S36*15%))))</f>
+        <f>IF(T36&lt;300, 0, MIN(99, IF(T36&lt;500, T36*7%, IF(T36&lt;700, T36*12%, T36*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3478,7 +3618,11 @@
           <t>RN8-SIL-CL-C</t>
         </is>
       </c>
-      <c r="B37" s="7" t="inlineStr"/>
+      <c r="B37" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
@@ -3541,19 +3685,19 @@
         <v>0</v>
       </c>
       <c r="R37" s="8">
-        <f>SUM(J37:P37)</f>
+        <f>SUM(K37:Q37)</f>
         <v/>
       </c>
       <c r="S37" s="8">
-        <f>IF(Q37&lt;300, Q37*1.4, IF(Q37&lt;400, Q37*1.33, Q37*1.25))</f>
+        <f>IF(R37&lt;300, R37*1.4, IF(R37&lt;400, R37*1.33, R37*1.25))</f>
         <v/>
       </c>
       <c r="T37" s="9">
-        <f>INT(R37/100)*100 + IF(MOD(ROUND(R37,0),100)&lt;25, 0, IF(MOD(ROUND(R37,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S37/100)*100 + IF(MOD(ROUND(S37,0),100)&lt;25, 0, IF(MOD(ROUND(S37,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U37" s="8">
-        <f>IF(S37&lt;300, 0, MIN(99, IF(S37&lt;500, S37*7%, IF(S37&lt;700, S37*12%, S37*15%))))</f>
+        <f>IF(T37&lt;300, 0, MIN(99, IF(T37&lt;500, T37*7%, IF(T37&lt;700, T37*12%, T37*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3563,7 +3707,11 @@
           <t>RN8-TPU-WT-M</t>
         </is>
       </c>
-      <c r="B38" s="3" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Ultra-Thin Shockproof Case for Realme GT Neo 8 – Slim Soft TPU Full Protection Back Cover</t>
+        </is>
+      </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
@@ -3626,19 +3774,19 @@
         <v>0</v>
       </c>
       <c r="R38" s="4">
-        <f>SUM(J38:P38)</f>
+        <f>SUM(K38:Q38)</f>
         <v/>
       </c>
       <c r="S38" s="4">
-        <f>IF(Q38&lt;300, Q38*1.4, IF(Q38&lt;400, Q38*1.33, Q38*1.25))</f>
+        <f>IF(R38&lt;300, R38*1.4, IF(R38&lt;400, R38*1.33, R38*1.25))</f>
         <v/>
       </c>
       <c r="T38" s="5">
-        <f>INT(R38/100)*100 + IF(MOD(ROUND(R38,0),100)&lt;25, 0, IF(MOD(ROUND(R38,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S38/100)*100 + IF(MOD(ROUND(S38,0),100)&lt;25, 0, IF(MOD(ROUND(S38,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U38" s="4">
-        <f>IF(S38&lt;300, 0, MIN(99, IF(S38&lt;500, S38*7%, IF(S38&lt;700, S38*12%, S38*15%))))</f>
+        <f>IF(T38&lt;300, 0, MIN(99, IF(T38&lt;500, T38*7%, IF(T38&lt;700, T38*12%, T38*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3648,7 +3796,11 @@
           <t>RN8-TPU-BK-M</t>
         </is>
       </c>
-      <c r="B39" s="7" t="inlineStr"/>
+      <c r="B39" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Ultra-Thin Shockproof Case for Realme GT Neo 8 – Slim Soft TPU Full Protection Back Cover</t>
+        </is>
+      </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
@@ -3711,19 +3863,19 @@
         <v>0</v>
       </c>
       <c r="R39" s="8">
-        <f>SUM(J39:P39)</f>
+        <f>SUM(K39:Q39)</f>
         <v/>
       </c>
       <c r="S39" s="8">
-        <f>IF(Q39&lt;300, Q39*1.4, IF(Q39&lt;400, Q39*1.33, Q39*1.25))</f>
+        <f>IF(R39&lt;300, R39*1.4, IF(R39&lt;400, R39*1.33, R39*1.25))</f>
         <v/>
       </c>
       <c r="T39" s="9">
-        <f>INT(R39/100)*100 + IF(MOD(ROUND(R39,0),100)&lt;25, 0, IF(MOD(ROUND(R39,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S39/100)*100 + IF(MOD(ROUND(S39,0),100)&lt;25, 0, IF(MOD(ROUND(S39,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U39" s="8">
-        <f>IF(S39&lt;300, 0, MIN(99, IF(S39&lt;500, S39*7%, IF(S39&lt;700, S39*12%, S39*15%))))</f>
+        <f>IF(T39&lt;300, 0, MIN(99, IF(T39&lt;500, T39*7%, IF(T39&lt;700, T39*12%, T39*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3733,7 +3885,11 @@
           <t>H600L-SIL-BK-M</t>
         </is>
       </c>
-      <c r="B40" s="3" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C40" s="3" t="inlineStr">
         <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
@@ -3796,19 +3952,19 @@
         <v>0</v>
       </c>
       <c r="R40" s="4">
-        <f>SUM(J40:P40)</f>
+        <f>SUM(K40:Q40)</f>
         <v/>
       </c>
       <c r="S40" s="4">
-        <f>IF(Q40&lt;300, Q40*1.4, IF(Q40&lt;400, Q40*1.33, Q40*1.25))</f>
+        <f>IF(R40&lt;300, R40*1.4, IF(R40&lt;400, R40*1.33, R40*1.25))</f>
         <v/>
       </c>
       <c r="T40" s="5">
-        <f>INT(R40/100)*100 + IF(MOD(ROUND(R40,0),100)&lt;25, 0, IF(MOD(ROUND(R40,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S40/100)*100 + IF(MOD(ROUND(S40,0),100)&lt;25, 0, IF(MOD(ROUND(S40,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U40" s="4">
-        <f>IF(S40&lt;300, 0, MIN(99, IF(S40&lt;500, S40*7%, IF(S40&lt;700, S40*12%, S40*15%))))</f>
+        <f>IF(T40&lt;300, 0, MIN(99, IF(T40&lt;500, T40*7%, IF(T40&lt;700, T40*12%, T40*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3818,7 +3974,11 @@
           <t>H600L-SIL-BL-M</t>
         </is>
       </c>
-      <c r="B41" s="7" t="inlineStr"/>
+      <c r="B41" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C41" s="7" t="inlineStr">
         <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
@@ -3881,19 +4041,19 @@
         <v>0</v>
       </c>
       <c r="R41" s="8">
-        <f>SUM(J41:P41)</f>
+        <f>SUM(K41:Q41)</f>
         <v/>
       </c>
       <c r="S41" s="8">
-        <f>IF(Q41&lt;300, Q41*1.4, IF(Q41&lt;400, Q41*1.33, Q41*1.25))</f>
+        <f>IF(R41&lt;300, R41*1.4, IF(R41&lt;400, R41*1.33, R41*1.25))</f>
         <v/>
       </c>
       <c r="T41" s="9">
-        <f>INT(R41/100)*100 + IF(MOD(ROUND(R41,0),100)&lt;25, 0, IF(MOD(ROUND(R41,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S41/100)*100 + IF(MOD(ROUND(S41,0),100)&lt;25, 0, IF(MOD(ROUND(S41,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U41" s="8">
-        <f>IF(S41&lt;300, 0, MIN(99, IF(S41&lt;500, S41*7%, IF(S41&lt;700, S41*12%, S41*15%))))</f>
+        <f>IF(T41&lt;300, 0, MIN(99, IF(T41&lt;500, T41*7%, IF(T41&lt;700, T41*12%, T41*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3903,7 +4063,11 @@
           <t>H600L-SIL-GN-M</t>
         </is>
       </c>
-      <c r="B42" s="3" t="inlineStr"/>
+      <c r="B42" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
@@ -3966,19 +4130,19 @@
         <v>0</v>
       </c>
       <c r="R42" s="4">
-        <f>SUM(J42:P42)</f>
+        <f>SUM(K42:Q42)</f>
         <v/>
       </c>
       <c r="S42" s="4">
-        <f>IF(Q42&lt;300, Q42*1.4, IF(Q42&lt;400, Q42*1.33, Q42*1.25))</f>
+        <f>IF(R42&lt;300, R42*1.4, IF(R42&lt;400, R42*1.33, R42*1.25))</f>
         <v/>
       </c>
       <c r="T42" s="5">
-        <f>INT(R42/100)*100 + IF(MOD(ROUND(R42,0),100)&lt;25, 0, IF(MOD(ROUND(R42,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S42/100)*100 + IF(MOD(ROUND(S42,0),100)&lt;25, 0, IF(MOD(ROUND(S42,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U42" s="4">
-        <f>IF(S42&lt;300, 0, MIN(99, IF(S42&lt;500, S42*7%, IF(S42&lt;700, S42*12%, S42*15%))))</f>
+        <f>IF(T42&lt;300, 0, MIN(99, IF(T42&lt;500, T42*7%, IF(T42&lt;700, T42*12%, T42*15%))))</f>
         <v/>
       </c>
     </row>
@@ -3988,7 +4152,11 @@
           <t>H600L-SIL-RD-M</t>
         </is>
       </c>
-      <c r="B43" s="7" t="inlineStr"/>
+      <c r="B43" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
           <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
@@ -4051,19 +4219,19 @@
         <v>0</v>
       </c>
       <c r="R43" s="8">
-        <f>SUM(J43:P43)</f>
+        <f>SUM(K43:Q43)</f>
         <v/>
       </c>
       <c r="S43" s="8">
-        <f>IF(Q43&lt;300, Q43*1.4, IF(Q43&lt;400, Q43*1.33, Q43*1.25))</f>
+        <f>IF(R43&lt;300, R43*1.4, IF(R43&lt;400, R43*1.33, R43*1.25))</f>
         <v/>
       </c>
       <c r="T43" s="9">
-        <f>INT(R43/100)*100 + IF(MOD(ROUND(R43,0),100)&lt;25, 0, IF(MOD(ROUND(R43,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S43/100)*100 + IF(MOD(ROUND(S43,0),100)&lt;25, 0, IF(MOD(ROUND(S43,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U43" s="8">
-        <f>IF(S43&lt;300, 0, MIN(99, IF(S43&lt;500, S43*7%, IF(S43&lt;700, S43*12%, S43*15%))))</f>
+        <f>IF(T43&lt;300, 0, MIN(99, IF(T43&lt;500, T43*7%, IF(T43&lt;700, T43*12%, T43*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4073,7 +4241,11 @@
           <t>HX80I-TPU-SV-E</t>
         </is>
       </c>
-      <c r="B44" s="3" t="inlineStr"/>
+      <c r="B44" s="3" t="inlineStr">
+        <is>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C44" s="3" t="inlineStr">
         <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
@@ -4136,19 +4308,19 @@
         <v>0</v>
       </c>
       <c r="R44" s="4">
-        <f>SUM(J44:P44)</f>
+        <f>SUM(K44:Q44)</f>
         <v/>
       </c>
       <c r="S44" s="4">
-        <f>IF(Q44&lt;300, Q44*1.4, IF(Q44&lt;400, Q44*1.33, Q44*1.25))</f>
+        <f>IF(R44&lt;300, R44*1.4, IF(R44&lt;400, R44*1.33, R44*1.25))</f>
         <v/>
       </c>
       <c r="T44" s="5">
-        <f>INT(R44/100)*100 + IF(MOD(ROUND(R44,0),100)&lt;25, 0, IF(MOD(ROUND(R44,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S44/100)*100 + IF(MOD(ROUND(S44,0),100)&lt;25, 0, IF(MOD(ROUND(S44,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U44" s="4">
-        <f>IF(S44&lt;300, 0, MIN(99, IF(S44&lt;500, S44*7%, IF(S44&lt;700, S44*12%, S44*15%))))</f>
+        <f>IF(T44&lt;300, 0, MIN(99, IF(T44&lt;500, T44*7%, IF(T44&lt;700, T44*12%, T44*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4158,7 +4330,11 @@
           <t>HX80I-TPU-BK-E</t>
         </is>
       </c>
-      <c r="B45" s="7" t="inlineStr"/>
+      <c r="B45" s="7" t="inlineStr">
+        <is>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C45" s="7" t="inlineStr">
         <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
@@ -4221,19 +4397,19 @@
         <v>0</v>
       </c>
       <c r="R45" s="8">
-        <f>SUM(J45:P45)</f>
+        <f>SUM(K45:Q45)</f>
         <v/>
       </c>
       <c r="S45" s="8">
-        <f>IF(Q45&lt;300, Q45*1.4, IF(Q45&lt;400, Q45*1.33, Q45*1.25))</f>
+        <f>IF(R45&lt;300, R45*1.4, IF(R45&lt;400, R45*1.33, R45*1.25))</f>
         <v/>
       </c>
       <c r="T45" s="9">
-        <f>INT(R45/100)*100 + IF(MOD(ROUND(R45,0),100)&lt;25, 0, IF(MOD(ROUND(R45,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S45/100)*100 + IF(MOD(ROUND(S45,0),100)&lt;25, 0, IF(MOD(ROUND(S45,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U45" s="8">
-        <f>IF(S45&lt;300, 0, MIN(99, IF(S45&lt;500, S45*7%, IF(S45&lt;700, S45*12%, S45*15%))))</f>
+        <f>IF(T45&lt;300, 0, MIN(99, IF(T45&lt;500, T45*7%, IF(T45&lt;700, T45*12%, T45*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4243,7 +4419,11 @@
           <t>HX80I-TPU-PR-E</t>
         </is>
       </c>
-      <c r="B46" s="3" t="inlineStr"/>
+      <c r="B46" s="3" t="inlineStr">
+        <is>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C46" s="3" t="inlineStr">
         <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
@@ -4306,19 +4486,19 @@
         <v>0</v>
       </c>
       <c r="R46" s="4">
-        <f>SUM(J46:P46)</f>
+        <f>SUM(K46:Q46)</f>
         <v/>
       </c>
       <c r="S46" s="4">
-        <f>IF(Q46&lt;300, Q46*1.4, IF(Q46&lt;400, Q46*1.33, Q46*1.25))</f>
+        <f>IF(R46&lt;300, R46*1.4, IF(R46&lt;400, R46*1.33, R46*1.25))</f>
         <v/>
       </c>
       <c r="T46" s="5">
-        <f>INT(R46/100)*100 + IF(MOD(ROUND(R46,0),100)&lt;25, 0, IF(MOD(ROUND(R46,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S46/100)*100 + IF(MOD(ROUND(S46,0),100)&lt;25, 0, IF(MOD(ROUND(S46,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U46" s="4">
-        <f>IF(S46&lt;300, 0, MIN(99, IF(S46&lt;500, S46*7%, IF(S46&lt;700, S46*12%, S46*15%))))</f>
+        <f>IF(T46&lt;300, 0, MIN(99, IF(T46&lt;500, T46*7%, IF(T46&lt;700, T46*12%, T46*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4328,7 +4508,11 @@
           <t>HX80I-TPU-BL-E</t>
         </is>
       </c>
-      <c r="B47" s="7" t="inlineStr"/>
+      <c r="B47" s="7" t="inlineStr">
+        <is>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C47" s="7" t="inlineStr">
         <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
@@ -4391,19 +4575,19 @@
         <v>0</v>
       </c>
       <c r="R47" s="8">
-        <f>SUM(J47:P47)</f>
+        <f>SUM(K47:Q47)</f>
         <v/>
       </c>
       <c r="S47" s="8">
-        <f>IF(Q47&lt;300, Q47*1.4, IF(Q47&lt;400, Q47*1.33, Q47*1.25))</f>
+        <f>IF(R47&lt;300, R47*1.4, IF(R47&lt;400, R47*1.33, R47*1.25))</f>
         <v/>
       </c>
       <c r="T47" s="9">
-        <f>INT(R47/100)*100 + IF(MOD(ROUND(R47,0),100)&lt;25, 0, IF(MOD(ROUND(R47,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S47/100)*100 + IF(MOD(ROUND(S47,0),100)&lt;25, 0, IF(MOD(ROUND(S47,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U47" s="8">
-        <f>IF(S47&lt;300, 0, MIN(99, IF(S47&lt;500, S47*7%, IF(S47&lt;700, S47*12%, S47*15%))))</f>
+        <f>IF(T47&lt;300, 0, MIN(99, IF(T47&lt;500, T47*7%, IF(T47&lt;700, T47*12%, T47*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4413,7 +4597,11 @@
           <t>HX80I-TPU-PK-E</t>
         </is>
       </c>
-      <c r="B48" s="3" t="inlineStr"/>
+      <c r="B48" s="3" t="inlineStr">
+        <is>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
@@ -4476,19 +4664,19 @@
         <v>0</v>
       </c>
       <c r="R48" s="4">
-        <f>SUM(J48:P48)</f>
+        <f>SUM(K48:Q48)</f>
         <v/>
       </c>
       <c r="S48" s="4">
-        <f>IF(Q48&lt;300, Q48*1.4, IF(Q48&lt;400, Q48*1.33, Q48*1.25))</f>
+        <f>IF(R48&lt;300, R48*1.4, IF(R48&lt;400, R48*1.33, R48*1.25))</f>
         <v/>
       </c>
       <c r="T48" s="5">
-        <f>INT(R48/100)*100 + IF(MOD(ROUND(R48,0),100)&lt;25, 0, IF(MOD(ROUND(R48,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S48/100)*100 + IF(MOD(ROUND(S48,0),100)&lt;25, 0, IF(MOD(ROUND(S48,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U48" s="4">
-        <f>IF(S48&lt;300, 0, MIN(99, IF(S48&lt;500, S48*7%, IF(S48&lt;700, S48*12%, S48*15%))))</f>
+        <f>IF(T48&lt;300, 0, MIN(99, IF(T48&lt;500, T48*7%, IF(T48&lt;700, T48*12%, T48*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4498,7 +4686,11 @@
           <t>HX80I-TPU-GN-E</t>
         </is>
       </c>
-      <c r="B49" s="7" t="inlineStr"/>
+      <c r="B49" s="7" t="inlineStr">
+        <is>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
           <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
@@ -4561,19 +4753,19 @@
         <v>0</v>
       </c>
       <c r="R49" s="8">
-        <f>SUM(J49:P49)</f>
+        <f>SUM(K49:Q49)</f>
         <v/>
       </c>
       <c r="S49" s="8">
-        <f>IF(Q49&lt;300, Q49*1.4, IF(Q49&lt;400, Q49*1.33, Q49*1.25))</f>
+        <f>IF(R49&lt;300, R49*1.4, IF(R49&lt;400, R49*1.33, R49*1.25))</f>
         <v/>
       </c>
       <c r="T49" s="9">
-        <f>INT(R49/100)*100 + IF(MOD(ROUND(R49,0),100)&lt;25, 0, IF(MOD(ROUND(R49,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S49/100)*100 + IF(MOD(ROUND(S49,0),100)&lt;25, 0, IF(MOD(ROUND(S49,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U49" s="8">
-        <f>IF(S49&lt;300, 0, MIN(99, IF(S49&lt;500, S49*7%, IF(S49&lt;700, S49*12%, S49*15%))))</f>
+        <f>IF(T49&lt;300, 0, MIN(99, IF(T49&lt;500, T49*7%, IF(T49&lt;700, T49*12%, T49*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4583,7 +4775,11 @@
           <t>HX80I-PC-GY-M</t>
         </is>
       </c>
-      <c r="B50" s="3" t="inlineStr"/>
+      <c r="B50" s="3" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C50" s="3" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -4646,19 +4842,19 @@
         <v>0</v>
       </c>
       <c r="R50" s="4">
-        <f>SUM(J50:P50)</f>
+        <f>SUM(K50:Q50)</f>
         <v/>
       </c>
       <c r="S50" s="4">
-        <f>IF(Q50&lt;300, Q50*1.4, IF(Q50&lt;400, Q50*1.33, Q50*1.25))</f>
+        <f>IF(R50&lt;300, R50*1.4, IF(R50&lt;400, R50*1.33, R50*1.25))</f>
         <v/>
       </c>
       <c r="T50" s="5">
-        <f>INT(R50/100)*100 + IF(MOD(ROUND(R50,0),100)&lt;25, 0, IF(MOD(ROUND(R50,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S50/100)*100 + IF(MOD(ROUND(S50,0),100)&lt;25, 0, IF(MOD(ROUND(S50,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U50" s="4">
-        <f>IF(S50&lt;300, 0, MIN(99, IF(S50&lt;500, S50*7%, IF(S50&lt;700, S50*12%, S50*15%))))</f>
+        <f>IF(T50&lt;300, 0, MIN(99, IF(T50&lt;500, T50*7%, IF(T50&lt;700, T50*12%, T50*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4668,7 +4864,11 @@
           <t>HX80I-PC-WT-M</t>
         </is>
       </c>
-      <c r="B51" s="7" t="inlineStr"/>
+      <c r="B51" s="7" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C51" s="7" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -4731,19 +4931,19 @@
         <v>0</v>
       </c>
       <c r="R51" s="8">
-        <f>SUM(J51:P51)</f>
+        <f>SUM(K51:Q51)</f>
         <v/>
       </c>
       <c r="S51" s="8">
-        <f>IF(Q51&lt;300, Q51*1.4, IF(Q51&lt;400, Q51*1.33, Q51*1.25))</f>
+        <f>IF(R51&lt;300, R51*1.4, IF(R51&lt;400, R51*1.33, R51*1.25))</f>
         <v/>
       </c>
       <c r="T51" s="9">
-        <f>INT(R51/100)*100 + IF(MOD(ROUND(R51,0),100)&lt;25, 0, IF(MOD(ROUND(R51,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S51/100)*100 + IF(MOD(ROUND(S51,0),100)&lt;25, 0, IF(MOD(ROUND(S51,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U51" s="8">
-        <f>IF(S51&lt;300, 0, MIN(99, IF(S51&lt;500, S51*7%, IF(S51&lt;700, S51*12%, S51*15%))))</f>
+        <f>IF(T51&lt;300, 0, MIN(99, IF(T51&lt;500, T51*7%, IF(T51&lt;700, T51*12%, T51*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4753,7 +4953,11 @@
           <t>HX80I-PC-GN-M</t>
         </is>
       </c>
-      <c r="B52" s="3" t="inlineStr"/>
+      <c r="B52" s="3" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C52" s="3" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -4816,19 +5020,19 @@
         <v>0</v>
       </c>
       <c r="R52" s="4">
-        <f>SUM(J52:P52)</f>
+        <f>SUM(K52:Q52)</f>
         <v/>
       </c>
       <c r="S52" s="4">
-        <f>IF(Q52&lt;300, Q52*1.4, IF(Q52&lt;400, Q52*1.33, Q52*1.25))</f>
+        <f>IF(R52&lt;300, R52*1.4, IF(R52&lt;400, R52*1.33, R52*1.25))</f>
         <v/>
       </c>
       <c r="T52" s="5">
-        <f>INT(R52/100)*100 + IF(MOD(ROUND(R52,0),100)&lt;25, 0, IF(MOD(ROUND(R52,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S52/100)*100 + IF(MOD(ROUND(S52,0),100)&lt;25, 0, IF(MOD(ROUND(S52,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U52" s="4">
-        <f>IF(S52&lt;300, 0, MIN(99, IF(S52&lt;500, S52*7%, IF(S52&lt;700, S52*12%, S52*15%))))</f>
+        <f>IF(T52&lt;300, 0, MIN(99, IF(T52&lt;500, T52*7%, IF(T52&lt;700, T52*12%, T52*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4838,7 +5042,11 @@
           <t>HX80I-PC-GD-M</t>
         </is>
       </c>
-      <c r="B53" s="7" t="inlineStr"/>
+      <c r="B53" s="7" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C53" s="7" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -4901,19 +5109,19 @@
         <v>0</v>
       </c>
       <c r="R53" s="8">
-        <f>SUM(J53:P53)</f>
+        <f>SUM(K53:Q53)</f>
         <v/>
       </c>
       <c r="S53" s="8">
-        <f>IF(Q53&lt;300, Q53*1.4, IF(Q53&lt;400, Q53*1.33, Q53*1.25))</f>
+        <f>IF(R53&lt;300, R53*1.4, IF(R53&lt;400, R53*1.33, R53*1.25))</f>
         <v/>
       </c>
       <c r="T53" s="9">
-        <f>INT(R53/100)*100 + IF(MOD(ROUND(R53,0),100)&lt;25, 0, IF(MOD(ROUND(R53,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S53/100)*100 + IF(MOD(ROUND(S53,0),100)&lt;25, 0, IF(MOD(ROUND(S53,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U53" s="8">
-        <f>IF(S53&lt;300, 0, MIN(99, IF(S53&lt;500, S53*7%, IF(S53&lt;700, S53*12%, S53*15%))))</f>
+        <f>IF(T53&lt;300, 0, MIN(99, IF(T53&lt;500, T53*7%, IF(T53&lt;700, T53*12%, T53*15%))))</f>
         <v/>
       </c>
     </row>
@@ -4923,7 +5131,11 @@
           <t>HX80I-PC-BK-M</t>
         </is>
       </c>
-      <c r="B54" s="3" t="inlineStr"/>
+      <c r="B54" s="3" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C54" s="3" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -4986,19 +5198,19 @@
         <v>0</v>
       </c>
       <c r="R54" s="4">
-        <f>SUM(J54:P54)</f>
+        <f>SUM(K54:Q54)</f>
         <v/>
       </c>
       <c r="S54" s="4">
-        <f>IF(Q54&lt;300, Q54*1.4, IF(Q54&lt;400, Q54*1.33, Q54*1.25))</f>
+        <f>IF(R54&lt;300, R54*1.4, IF(R54&lt;400, R54*1.33, R54*1.25))</f>
         <v/>
       </c>
       <c r="T54" s="5">
-        <f>INT(R54/100)*100 + IF(MOD(ROUND(R54,0),100)&lt;25, 0, IF(MOD(ROUND(R54,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S54/100)*100 + IF(MOD(ROUND(S54,0),100)&lt;25, 0, IF(MOD(ROUND(S54,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U54" s="4">
-        <f>IF(S54&lt;300, 0, MIN(99, IF(S54&lt;500, S54*7%, IF(S54&lt;700, S54*12%, S54*15%))))</f>
+        <f>IF(T54&lt;300, 0, MIN(99, IF(T54&lt;500, T54*7%, IF(T54&lt;700, T54*12%, T54*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5008,7 +5220,11 @@
           <t>H600L-PC-GY-M</t>
         </is>
       </c>
-      <c r="B55" s="7" t="inlineStr"/>
+      <c r="B55" s="7" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C55" s="7" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -5071,19 +5287,19 @@
         <v>0</v>
       </c>
       <c r="R55" s="8">
-        <f>SUM(J55:P55)</f>
+        <f>SUM(K55:Q55)</f>
         <v/>
       </c>
       <c r="S55" s="8">
-        <f>IF(Q55&lt;300, Q55*1.4, IF(Q55&lt;400, Q55*1.33, Q55*1.25))</f>
+        <f>IF(R55&lt;300, R55*1.4, IF(R55&lt;400, R55*1.33, R55*1.25))</f>
         <v/>
       </c>
       <c r="T55" s="9">
-        <f>INT(R55/100)*100 + IF(MOD(ROUND(R55,0),100)&lt;25, 0, IF(MOD(ROUND(R55,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S55/100)*100 + IF(MOD(ROUND(S55,0),100)&lt;25, 0, IF(MOD(ROUND(S55,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U55" s="8">
-        <f>IF(S55&lt;300, 0, MIN(99, IF(S55&lt;500, S55*7%, IF(S55&lt;700, S55*12%, S55*15%))))</f>
+        <f>IF(T55&lt;300, 0, MIN(99, IF(T55&lt;500, T55*7%, IF(T55&lt;700, T55*12%, T55*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5093,7 +5309,11 @@
           <t>H600L-PC-WT-M</t>
         </is>
       </c>
-      <c r="B56" s="3" t="inlineStr"/>
+      <c r="B56" s="3" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C56" s="3" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -5156,19 +5376,19 @@
         <v>0</v>
       </c>
       <c r="R56" s="4">
-        <f>SUM(J56:P56)</f>
+        <f>SUM(K56:Q56)</f>
         <v/>
       </c>
       <c r="S56" s="4">
-        <f>IF(Q56&lt;300, Q56*1.4, IF(Q56&lt;400, Q56*1.33, Q56*1.25))</f>
+        <f>IF(R56&lt;300, R56*1.4, IF(R56&lt;400, R56*1.33, R56*1.25))</f>
         <v/>
       </c>
       <c r="T56" s="5">
-        <f>INT(R56/100)*100 + IF(MOD(ROUND(R56,0),100)&lt;25, 0, IF(MOD(ROUND(R56,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S56/100)*100 + IF(MOD(ROUND(S56,0),100)&lt;25, 0, IF(MOD(ROUND(S56,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U56" s="4">
-        <f>IF(S56&lt;300, 0, MIN(99, IF(S56&lt;500, S56*7%, IF(S56&lt;700, S56*12%, S56*15%))))</f>
+        <f>IF(T56&lt;300, 0, MIN(99, IF(T56&lt;500, T56*7%, IF(T56&lt;700, T56*12%, T56*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5178,7 +5398,11 @@
           <t>H600L-PC-GN-M</t>
         </is>
       </c>
-      <c r="B57" s="7" t="inlineStr"/>
+      <c r="B57" s="7" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C57" s="7" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -5241,19 +5465,19 @@
         <v>0</v>
       </c>
       <c r="R57" s="8">
-        <f>SUM(J57:P57)</f>
+        <f>SUM(K57:Q57)</f>
         <v/>
       </c>
       <c r="S57" s="8">
-        <f>IF(Q57&lt;300, Q57*1.4, IF(Q57&lt;400, Q57*1.33, Q57*1.25))</f>
+        <f>IF(R57&lt;300, R57*1.4, IF(R57&lt;400, R57*1.33, R57*1.25))</f>
         <v/>
       </c>
       <c r="T57" s="9">
-        <f>INT(R57/100)*100 + IF(MOD(ROUND(R57,0),100)&lt;25, 0, IF(MOD(ROUND(R57,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S57/100)*100 + IF(MOD(ROUND(S57,0),100)&lt;25, 0, IF(MOD(ROUND(S57,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U57" s="8">
-        <f>IF(S57&lt;300, 0, MIN(99, IF(S57&lt;500, S57*7%, IF(S57&lt;700, S57*12%, S57*15%))))</f>
+        <f>IF(T57&lt;300, 0, MIN(99, IF(T57&lt;500, T57*7%, IF(T57&lt;700, T57*12%, T57*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5263,7 +5487,11 @@
           <t>H600L-PC-GD-M</t>
         </is>
       </c>
-      <c r="B58" s="3" t="inlineStr"/>
+      <c r="B58" s="3" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -5326,19 +5554,19 @@
         <v>0</v>
       </c>
       <c r="R58" s="4">
-        <f>SUM(J58:P58)</f>
+        <f>SUM(K58:Q58)</f>
         <v/>
       </c>
       <c r="S58" s="4">
-        <f>IF(Q58&lt;300, Q58*1.4, IF(Q58&lt;400, Q58*1.33, Q58*1.25))</f>
+        <f>IF(R58&lt;300, R58*1.4, IF(R58&lt;400, R58*1.33, R58*1.25))</f>
         <v/>
       </c>
       <c r="T58" s="5">
-        <f>INT(R58/100)*100 + IF(MOD(ROUND(R58,0),100)&lt;25, 0, IF(MOD(ROUND(R58,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S58/100)*100 + IF(MOD(ROUND(S58,0),100)&lt;25, 0, IF(MOD(ROUND(S58,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U58" s="4">
-        <f>IF(S58&lt;300, 0, MIN(99, IF(S58&lt;500, S58*7%, IF(S58&lt;700, S58*12%, S58*15%))))</f>
+        <f>IF(T58&lt;300, 0, MIN(99, IF(T58&lt;500, T58*7%, IF(T58&lt;700, T58*12%, T58*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5348,7 +5576,11 @@
           <t>H600L-PC-BK-M</t>
         </is>
       </c>
-      <c r="B59" s="7" t="inlineStr"/>
+      <c r="B59" s="7" t="inlineStr">
+        <is>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+        </is>
+      </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
           <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
@@ -5411,19 +5643,19 @@
         <v>0</v>
       </c>
       <c r="R59" s="8">
-        <f>SUM(J59:P59)</f>
+        <f>SUM(K59:Q59)</f>
         <v/>
       </c>
       <c r="S59" s="8">
-        <f>IF(Q59&lt;300, Q59*1.4, IF(Q59&lt;400, Q59*1.33, Q59*1.25))</f>
+        <f>IF(R59&lt;300, R59*1.4, IF(R59&lt;400, R59*1.33, R59*1.25))</f>
         <v/>
       </c>
       <c r="T59" s="9">
-        <f>INT(R59/100)*100 + IF(MOD(ROUND(R59,0),100)&lt;25, 0, IF(MOD(ROUND(R59,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S59/100)*100 + IF(MOD(ROUND(S59,0),100)&lt;25, 0, IF(MOD(ROUND(S59,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U59" s="8">
-        <f>IF(S59&lt;300, 0, MIN(99, IF(S59&lt;500, S59*7%, IF(S59&lt;700, S59*12%, S59*15%))))</f>
+        <f>IF(T59&lt;300, 0, MIN(99, IF(T59&lt;500, T59*7%, IF(T59&lt;700, T59*12%, T59*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5433,7 +5665,11 @@
           <t>RN8-PC-RK-M</t>
         </is>
       </c>
-      <c r="B60" s="3" t="inlineStr"/>
+      <c r="B60" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C60" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -5496,19 +5732,19 @@
         <v>0</v>
       </c>
       <c r="R60" s="4">
-        <f>SUM(J60:P60)</f>
+        <f>SUM(K60:Q60)</f>
         <v/>
       </c>
       <c r="S60" s="4">
-        <f>IF(Q60&lt;300, Q60*1.4, IF(Q60&lt;400, Q60*1.33, Q60*1.25))</f>
+        <f>IF(R60&lt;300, R60*1.4, IF(R60&lt;400, R60*1.33, R60*1.25))</f>
         <v/>
       </c>
       <c r="T60" s="5">
-        <f>INT(R60/100)*100 + IF(MOD(ROUND(R60,0),100)&lt;25, 0, IF(MOD(ROUND(R60,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S60/100)*100 + IF(MOD(ROUND(S60,0),100)&lt;25, 0, IF(MOD(ROUND(S60,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U60" s="4">
-        <f>IF(S60&lt;300, 0, MIN(99, IF(S60&lt;500, S60*7%, IF(S60&lt;700, S60*12%, S60*15%))))</f>
+        <f>IF(T60&lt;300, 0, MIN(99, IF(T60&lt;500, T60*7%, IF(T60&lt;700, T60*12%, T60*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5518,7 +5754,11 @@
           <t>RN8-PC-GD-M</t>
         </is>
       </c>
-      <c r="B61" s="7" t="inlineStr"/>
+      <c r="B61" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C61" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -5581,19 +5821,19 @@
         <v>0</v>
       </c>
       <c r="R61" s="8">
-        <f>SUM(J61:P61)</f>
+        <f>SUM(K61:Q61)</f>
         <v/>
       </c>
       <c r="S61" s="8">
-        <f>IF(Q61&lt;300, Q61*1.4, IF(Q61&lt;400, Q61*1.33, Q61*1.25))</f>
+        <f>IF(R61&lt;300, R61*1.4, IF(R61&lt;400, R61*1.33, R61*1.25))</f>
         <v/>
       </c>
       <c r="T61" s="9">
-        <f>INT(R61/100)*100 + IF(MOD(ROUND(R61,0),100)&lt;25, 0, IF(MOD(ROUND(R61,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S61/100)*100 + IF(MOD(ROUND(S61,0),100)&lt;25, 0, IF(MOD(ROUND(S61,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U61" s="8">
-        <f>IF(S61&lt;300, 0, MIN(99, IF(S61&lt;500, S61*7%, IF(S61&lt;700, S61*12%, S61*15%))))</f>
+        <f>IF(T61&lt;300, 0, MIN(99, IF(T61&lt;500, T61*7%, IF(T61&lt;700, T61*12%, T61*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5603,7 +5843,11 @@
           <t>RN8-PC-BL-M</t>
         </is>
       </c>
-      <c r="B62" s="3" t="inlineStr"/>
+      <c r="B62" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C62" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -5666,19 +5910,19 @@
         <v>0</v>
       </c>
       <c r="R62" s="4">
-        <f>SUM(J62:P62)</f>
+        <f>SUM(K62:Q62)</f>
         <v/>
       </c>
       <c r="S62" s="4">
-        <f>IF(Q62&lt;300, Q62*1.4, IF(Q62&lt;400, Q62*1.33, Q62*1.25))</f>
+        <f>IF(R62&lt;300, R62*1.4, IF(R62&lt;400, R62*1.33, R62*1.25))</f>
         <v/>
       </c>
       <c r="T62" s="5">
-        <f>INT(R62/100)*100 + IF(MOD(ROUND(R62,0),100)&lt;25, 0, IF(MOD(ROUND(R62,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S62/100)*100 + IF(MOD(ROUND(S62,0),100)&lt;25, 0, IF(MOD(ROUND(S62,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U62" s="4">
-        <f>IF(S62&lt;300, 0, MIN(99, IF(S62&lt;500, S62*7%, IF(S62&lt;700, S62*12%, S62*15%))))</f>
+        <f>IF(T62&lt;300, 0, MIN(99, IF(T62&lt;500, T62*7%, IF(T62&lt;700, T62*12%, T62*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5688,7 +5932,11 @@
           <t>RN8-PC-PK-M</t>
         </is>
       </c>
-      <c r="B63" s="7" t="inlineStr"/>
+      <c r="B63" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C63" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -5751,19 +5999,19 @@
         <v>0</v>
       </c>
       <c r="R63" s="8">
-        <f>SUM(J63:P63)</f>
+        <f>SUM(K63:Q63)</f>
         <v/>
       </c>
       <c r="S63" s="8">
-        <f>IF(Q63&lt;300, Q63*1.4, IF(Q63&lt;400, Q63*1.33, Q63*1.25))</f>
+        <f>IF(R63&lt;300, R63*1.4, IF(R63&lt;400, R63*1.33, R63*1.25))</f>
         <v/>
       </c>
       <c r="T63" s="9">
-        <f>INT(R63/100)*100 + IF(MOD(ROUND(R63,0),100)&lt;25, 0, IF(MOD(ROUND(R63,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S63/100)*100 + IF(MOD(ROUND(S63,0),100)&lt;25, 0, IF(MOD(ROUND(S63,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U63" s="8">
-        <f>IF(S63&lt;300, 0, MIN(99, IF(S63&lt;500, S63*7%, IF(S63&lt;700, S63*12%, S63*15%))))</f>
+        <f>IF(T63&lt;300, 0, MIN(99, IF(T63&lt;500, T63*7%, IF(T63&lt;700, T63*12%, T63*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5773,7 +6021,11 @@
           <t>RN8-PC-CG-M</t>
         </is>
       </c>
-      <c r="B64" s="3" t="inlineStr"/>
+      <c r="B64" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C64" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -5836,19 +6088,19 @@
         <v>0</v>
       </c>
       <c r="R64" s="4">
-        <f>SUM(J64:P64)</f>
+        <f>SUM(K64:Q64)</f>
         <v/>
       </c>
       <c r="S64" s="4">
-        <f>IF(Q64&lt;300, Q64*1.4, IF(Q64&lt;400, Q64*1.33, Q64*1.25))</f>
+        <f>IF(R64&lt;300, R64*1.4, IF(R64&lt;400, R64*1.33, R64*1.25))</f>
         <v/>
       </c>
       <c r="T64" s="5">
-        <f>INT(R64/100)*100 + IF(MOD(ROUND(R64,0),100)&lt;25, 0, IF(MOD(ROUND(R64,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S64/100)*100 + IF(MOD(ROUND(S64,0),100)&lt;25, 0, IF(MOD(ROUND(S64,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U64" s="4">
-        <f>IF(S64&lt;300, 0, MIN(99, IF(S64&lt;500, S64*7%, IF(S64&lt;700, S64*12%, S64*15%))))</f>
+        <f>IF(T64&lt;300, 0, MIN(99, IF(T64&lt;500, T64*7%, IF(T64&lt;700, T64*12%, T64*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5858,7 +6110,11 @@
           <t>RN8-PC-PR-M</t>
         </is>
       </c>
-      <c r="B65" s="7" t="inlineStr"/>
+      <c r="B65" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C65" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -5921,19 +6177,19 @@
         <v>0</v>
       </c>
       <c r="R65" s="8">
-        <f>SUM(J65:P65)</f>
+        <f>SUM(K65:Q65)</f>
         <v/>
       </c>
       <c r="S65" s="8">
-        <f>IF(Q65&lt;300, Q65*1.4, IF(Q65&lt;400, Q65*1.33, Q65*1.25))</f>
+        <f>IF(R65&lt;300, R65*1.4, IF(R65&lt;400, R65*1.33, R65*1.25))</f>
         <v/>
       </c>
       <c r="T65" s="9">
-        <f>INT(R65/100)*100 + IF(MOD(ROUND(R65,0),100)&lt;25, 0, IF(MOD(ROUND(R65,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S65/100)*100 + IF(MOD(ROUND(S65,0),100)&lt;25, 0, IF(MOD(ROUND(S65,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U65" s="8">
-        <f>IF(S65&lt;300, 0, MIN(99, IF(S65&lt;500, S65*7%, IF(S65&lt;700, S65*12%, S65*15%))))</f>
+        <f>IF(T65&lt;300, 0, MIN(99, IF(T65&lt;500, T65*7%, IF(T65&lt;700, T65*12%, T65*15%))))</f>
         <v/>
       </c>
     </row>
@@ -5943,7 +6199,11 @@
           <t>RN8-PC-TG-M</t>
         </is>
       </c>
-      <c r="B66" s="3" t="inlineStr"/>
+      <c r="B66" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -6006,19 +6266,19 @@
         <v>0</v>
       </c>
       <c r="R66" s="4">
-        <f>SUM(J66:P66)</f>
+        <f>SUM(K66:Q66)</f>
         <v/>
       </c>
       <c r="S66" s="4">
-        <f>IF(Q66&lt;300, Q66*1.4, IF(Q66&lt;400, Q66*1.33, Q66*1.25))</f>
+        <f>IF(R66&lt;300, R66*1.4, IF(R66&lt;400, R66*1.33, R66*1.25))</f>
         <v/>
       </c>
       <c r="T66" s="5">
-        <f>INT(R66/100)*100 + IF(MOD(ROUND(R66,0),100)&lt;25, 0, IF(MOD(ROUND(R66,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S66/100)*100 + IF(MOD(ROUND(S66,0),100)&lt;25, 0, IF(MOD(ROUND(S66,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U66" s="4">
-        <f>IF(S66&lt;300, 0, MIN(99, IF(S66&lt;500, S66*7%, IF(S66&lt;700, S66*12%, S66*15%))))</f>
+        <f>IF(T66&lt;300, 0, MIN(99, IF(T66&lt;500, T66*7%, IF(T66&lt;700, T66*12%, T66*15%))))</f>
         <v/>
       </c>
     </row>
@@ -6028,7 +6288,11 @@
           <t>RN8-PC-BK-M</t>
         </is>
       </c>
-      <c r="B67" s="7" t="inlineStr"/>
+      <c r="B67" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+        </is>
+      </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
           <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
@@ -6091,19 +6355,19 @@
         <v>0</v>
       </c>
       <c r="R67" s="8">
-        <f>SUM(J67:P67)</f>
+        <f>SUM(K67:Q67)</f>
         <v/>
       </c>
       <c r="S67" s="8">
-        <f>IF(Q67&lt;300, Q67*1.4, IF(Q67&lt;400, Q67*1.33, Q67*1.25))</f>
+        <f>IF(R67&lt;300, R67*1.4, IF(R67&lt;400, R67*1.33, R67*1.25))</f>
         <v/>
       </c>
       <c r="T67" s="9">
-        <f>INT(R67/100)*100 + IF(MOD(ROUND(R67,0),100)&lt;25, 0, IF(MOD(ROUND(R67,0),100)&lt;=74, 49, 99))</f>
+        <f>INT(S67/100)*100 + IF(MOD(ROUND(S67,0),100)&lt;25, 0, IF(MOD(ROUND(S67,0),100)&lt;=74, 49, 99))</f>
         <v/>
       </c>
       <c r="U67" s="8">
-        <f>IF(S67&lt;300, 0, MIN(99, IF(S67&lt;500, S67*7%, IF(S67&lt;700, S67*12%, S67*15%))))</f>
+        <f>IF(T67&lt;300, 0, MIN(99, IF(T67&lt;500, T67*7%, IF(T67&lt;700, T67*12%, T67*15%))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: process Realme Neo8 Graphene Cooling Silicone case and update inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U67"/>
+  <dimension ref="A1:U70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -6371,6 +6371,273 @@
         <v/>
       </c>
     </row>
+    <row r="68">
+      <c r="A68" s="2" t="inlineStr">
+        <is>
+          <t>RN8-SIL-BK-M</t>
+        </is>
+      </c>
+      <c r="B68" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
+        </is>
+      </c>
+      <c r="C68" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
+        </is>
+      </c>
+      <c r="D68" s="2" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="E68" s="2" t="inlineStr">
+        <is>
+          <t>Obsidian Black</t>
+        </is>
+      </c>
+      <c r="F68" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G68" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H68" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I68" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
+        </is>
+      </c>
+      <c r="J68" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Silicone/sku/RN8-SIL-BK-M.jpg</t>
+        </is>
+      </c>
+      <c r="K68" s="4" t="n">
+        <v>425.6</v>
+      </c>
+      <c r="L68" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M68" s="4" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="N68" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O68" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P68" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q68" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R68" s="4">
+        <f>SUM(K68:Q68)</f>
+        <v/>
+      </c>
+      <c r="S68" s="4">
+        <f>IF(R68&lt;300, R68*1.4, IF(R68&lt;400, R68*1.33, R68*1.25))</f>
+        <v/>
+      </c>
+      <c r="T68" s="5">
+        <f>INT(S68/100)*100 + IF(MOD(ROUND(S68,0),100)&lt;25, 0, IF(MOD(ROUND(S68,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U68" s="4">
+        <f>IF(T68&lt;300, 0, MIN(99, IF(T68&lt;500, T68*7%, IF(T68&lt;700, T68*12%, T68*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="6" t="inlineStr">
+        <is>
+          <t>RN8-SIL-GY-M</t>
+        </is>
+      </c>
+      <c r="B69" s="7" t="inlineStr">
+        <is>
+          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
+        </is>
+      </c>
+      <c r="C69" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
+        </is>
+      </c>
+      <c r="D69" s="6" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="E69" s="6" t="inlineStr">
+        <is>
+          <t>Matte Gray</t>
+        </is>
+      </c>
+      <c r="F69" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G69" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H69" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I69" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
+        </is>
+      </c>
+      <c r="J69" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Silicone/sku/RN8-SIL-GY-M.jpg</t>
+        </is>
+      </c>
+      <c r="K69" s="8" t="n">
+        <v>425.6</v>
+      </c>
+      <c r="L69" s="8" t="n">
+        <v>10</v>
+      </c>
+      <c r="M69" s="8" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="N69" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O69" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P69" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q69" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R69" s="8">
+        <f>SUM(K69:Q69)</f>
+        <v/>
+      </c>
+      <c r="S69" s="8">
+        <f>IF(R69&lt;300, R69*1.4, IF(R69&lt;400, R69*1.33, R69*1.25))</f>
+        <v/>
+      </c>
+      <c r="T69" s="9">
+        <f>INT(S69/100)*100 + IF(MOD(ROUND(S69,0),100)&lt;25, 0, IF(MOD(ROUND(S69,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U69" s="8">
+        <f>IF(T69&lt;300, 0, MIN(99, IF(T69&lt;500, T69*7%, IF(T69&lt;700, T69*12%, T69*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="2" t="inlineStr">
+        <is>
+          <t>RN8-SIL-OR-M</t>
+        </is>
+      </c>
+      <c r="B70" s="3" t="inlineStr">
+        <is>
+          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
+        </is>
+      </c>
+      <c r="C70" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
+        </is>
+      </c>
+      <c r="D70" s="2" t="inlineStr">
+        <is>
+          <t>Silicone</t>
+        </is>
+      </c>
+      <c r="E70" s="2" t="inlineStr">
+        <is>
+          <t>Terracotta Orange</t>
+        </is>
+      </c>
+      <c r="F70" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G70" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H70" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I70" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
+        </is>
+      </c>
+      <c r="J70" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Silicone/sku/RN8-SIL-OR-M.jpg</t>
+        </is>
+      </c>
+      <c r="K70" s="4" t="n">
+        <v>425.6</v>
+      </c>
+      <c r="L70" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="M70" s="4" t="n">
+        <v>1.56</v>
+      </c>
+      <c r="N70" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O70" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P70" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q70" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R70" s="4">
+        <f>SUM(K70:Q70)</f>
+        <v/>
+      </c>
+      <c r="S70" s="4">
+        <f>IF(R70&lt;300, R70*1.4, IF(R70&lt;400, R70*1.33, R70*1.25))</f>
+        <v/>
+      </c>
+      <c r="T70" s="5">
+        <f>INT(S70/100)*100 + IF(MOD(ROUND(S70,0),100)&lt;25, 0, IF(MOD(ROUND(S70,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U70" s="4">
+        <f>IF(T70&lt;300, 0, MIN(99, IF(T70&lt;500, T70*7%, IF(T70&lt;700, T70*12%, T70*15%))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
fix: remove 1.1703 multiplier as MoveOn prices are already in BDT, and redo last link
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -6423,7 +6423,7 @@
         </is>
       </c>
       <c r="K68" s="4" t="n">
-        <v>425.6</v>
+        <v>363.66</v>
       </c>
       <c r="L68" s="4" t="n">
         <v>10</v>
@@ -6512,7 +6512,7 @@
         </is>
       </c>
       <c r="K69" s="8" t="n">
-        <v>425.6</v>
+        <v>363.66</v>
       </c>
       <c r="L69" s="8" t="n">
         <v>10</v>
@@ -6601,7 +6601,7 @@
         </is>
       </c>
       <c r="K70" s="4" t="n">
-        <v>425.6</v>
+        <v>363.66</v>
       </c>
       <c r="L70" s="4" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
fix: enforce 50-80 BDT floor for fake supplier weights and update inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -6429,7 +6429,7 @@
         <v>10</v>
       </c>
       <c r="M68" s="4" t="n">
-        <v>1.56</v>
+        <v>50</v>
       </c>
       <c r="N68" s="4" t="n">
         <v>5</v>
@@ -6518,7 +6518,7 @@
         <v>10</v>
       </c>
       <c r="M69" s="8" t="n">
-        <v>1.56</v>
+        <v>50</v>
       </c>
       <c r="N69" s="8" t="n">
         <v>5</v>
@@ -6607,7 +6607,7 @@
         <v>10</v>
       </c>
       <c r="M70" s="4" t="n">
-        <v>1.56</v>
+        <v>50</v>
       </c>
       <c r="N70" s="4" t="n">
         <v>5</v>

</xml_diff>

<commit_message>
docs: update product description with pre-order notice and sync inventory
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -2952,7 +2952,7 @@
         </is>
       </c>
       <c r="K29" s="8" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L29" s="8" t="n">
         <v>10</v>
@@ -3041,7 +3041,7 @@
         </is>
       </c>
       <c r="K30" s="4" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L30" s="4" t="n">
         <v>10</v>
@@ -3130,7 +3130,7 @@
         </is>
       </c>
       <c r="K31" s="8" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L31" s="8" t="n">
         <v>10</v>
@@ -3219,7 +3219,7 @@
         </is>
       </c>
       <c r="K32" s="4" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L32" s="4" t="n">
         <v>10</v>
@@ -3308,7 +3308,7 @@
         </is>
       </c>
       <c r="K33" s="8" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L33" s="8" t="n">
         <v>10</v>
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="K34" s="4" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L34" s="4" t="n">
         <v>10</v>
@@ -3486,7 +3486,7 @@
         </is>
       </c>
       <c r="K35" s="8" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L35" s="8" t="n">
         <v>10</v>
@@ -3575,7 +3575,7 @@
         </is>
       </c>
       <c r="K36" s="4" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L36" s="4" t="n">
         <v>10</v>
@@ -3664,7 +3664,7 @@
         </is>
       </c>
       <c r="K37" s="8" t="n">
-        <v>39.9</v>
+        <v>34.09</v>
       </c>
       <c r="L37" s="8" t="n">
         <v>10</v>

</xml_diff>

<commit_message>
sync: resolve inventory.xlsx and stage recent updates
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -6646,7 +6646,7 @@
       </c>
       <c r="B71" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C71" s="7" t="inlineStr">
@@ -6735,7 +6735,7 @@
       </c>
       <c r="B72" s="3" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C72" s="3" t="inlineStr">
@@ -6824,7 +6824,7 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C73" s="7" t="inlineStr">
@@ -6913,7 +6913,7 @@
       </c>
       <c r="B74" s="3" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C74" s="3" t="inlineStr">
@@ -7002,7 +7002,7 @@
       </c>
       <c r="B75" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C75" s="7" t="inlineStr">
@@ -7091,7 +7091,7 @@
       </c>
       <c r="B76" s="3" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C76" s="3" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="B77" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C77" s="7" t="inlineStr">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
@@ -7358,7 +7358,7 @@
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat: process MoveOn corrugated metal case for Realme Neo8 with china delivery and SKU disambiguation
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U79"/>
+  <dimension ref="A1:U85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7439,6 +7439,540 @@
         <v/>
       </c>
     </row>
+    <row r="80">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-BK-S</t>
+        </is>
+      </c>
+      <c r="B80" s="3" t="inlineStr">
+        <is>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C80" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+        </is>
+      </c>
+      <c r="D80" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E80" s="2" t="inlineStr">
+        <is>
+          <t>Black</t>
+        </is>
+      </c>
+      <c r="F80" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G80" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H80" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I80" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+        </is>
+      </c>
+      <c r="J80" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-BK-S.jpg</t>
+        </is>
+      </c>
+      <c r="K80" s="4" t="n">
+        <v>147.74</v>
+      </c>
+      <c r="L80" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="M80" s="4" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="N80" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O80" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P80" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q80" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R80" s="4">
+        <f>SUM(K80:Q80)</f>
+        <v/>
+      </c>
+      <c r="S80" s="4">
+        <f>IF(R80&lt;300, R80*1.4, IF(R80&lt;400, R80*1.33, R80*1.25))</f>
+        <v/>
+      </c>
+      <c r="T80" s="5">
+        <f>INT(S80/100)*100 + IF(MOD(ROUND(S80,0),100)&lt;25, 0, IF(MOD(ROUND(S80,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U80" s="4">
+        <f>IF(T80&lt;300, 0, MIN(99, IF(T80&lt;500, T80*7%, IF(T80&lt;700, T80*12%, T80*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-SV-S</t>
+        </is>
+      </c>
+      <c r="B81" s="7" t="inlineStr">
+        <is>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C81" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E81" s="6" t="inlineStr">
+        <is>
+          <t>Silver</t>
+        </is>
+      </c>
+      <c r="F81" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G81" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H81" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I81" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+        </is>
+      </c>
+      <c r="J81" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-SV-S.jpg</t>
+        </is>
+      </c>
+      <c r="K81" s="8" t="n">
+        <v>147.74</v>
+      </c>
+      <c r="L81" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M81" s="8" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="N81" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O81" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P81" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q81" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R81" s="8">
+        <f>SUM(K81:Q81)</f>
+        <v/>
+      </c>
+      <c r="S81" s="8">
+        <f>IF(R81&lt;300, R81*1.4, IF(R81&lt;400, R81*1.33, R81*1.25))</f>
+        <v/>
+      </c>
+      <c r="T81" s="9">
+        <f>INT(S81/100)*100 + IF(MOD(ROUND(S81,0),100)&lt;25, 0, IF(MOD(ROUND(S81,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U81" s="8">
+        <f>IF(T81&lt;300, 0, MIN(99, IF(T81&lt;500, T81*7%, IF(T81&lt;700, T81*12%, T81*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-CL-C</t>
+        </is>
+      </c>
+      <c r="B82" s="3" t="inlineStr">
+        <is>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C82" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+        </is>
+      </c>
+      <c r="D82" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E82" s="2" t="inlineStr">
+        <is>
+          <t>Transparent</t>
+        </is>
+      </c>
+      <c r="F82" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G82" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H82" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I82" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+        </is>
+      </c>
+      <c r="J82" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-CL-C.jpg</t>
+        </is>
+      </c>
+      <c r="K82" s="4" t="n">
+        <v>113.64</v>
+      </c>
+      <c r="L82" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="M82" s="4" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="N82" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O82" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P82" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q82" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R82" s="4">
+        <f>SUM(K82:Q82)</f>
+        <v/>
+      </c>
+      <c r="S82" s="4">
+        <f>IF(R82&lt;300, R82*1.4, IF(R82&lt;400, R82*1.33, R82*1.25))</f>
+        <v/>
+      </c>
+      <c r="T82" s="5">
+        <f>INT(S82/100)*100 + IF(MOD(ROUND(S82,0),100)&lt;25, 0, IF(MOD(ROUND(S82,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U82" s="4">
+        <f>IF(T82&lt;300, 0, MIN(99, IF(T82&lt;500, T82*7%, IF(T82&lt;700, T82*12%, T82*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-RD-S</t>
+        </is>
+      </c>
+      <c r="B83" s="7" t="inlineStr">
+        <is>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C83" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+        </is>
+      </c>
+      <c r="D83" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E83" s="6" t="inlineStr">
+        <is>
+          <t>Burgundy Red</t>
+        </is>
+      </c>
+      <c r="F83" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G83" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H83" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I83" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+        </is>
+      </c>
+      <c r="J83" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-RD-S.jpg</t>
+        </is>
+      </c>
+      <c r="K83" s="8" t="n">
+        <v>147.74</v>
+      </c>
+      <c r="L83" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M83" s="8" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="N83" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O83" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P83" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q83" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R83" s="8">
+        <f>SUM(K83:Q83)</f>
+        <v/>
+      </c>
+      <c r="S83" s="8">
+        <f>IF(R83&lt;300, R83*1.4, IF(R83&lt;400, R83*1.33, R83*1.25))</f>
+        <v/>
+      </c>
+      <c r="T83" s="9">
+        <f>INT(S83/100)*100 + IF(MOD(ROUND(S83,0),100)&lt;25, 0, IF(MOD(ROUND(S83,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U83" s="8">
+        <f>IF(T83&lt;300, 0, MIN(99, IF(T83&lt;500, T83*7%, IF(T83&lt;700, T83*12%, T83*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" s="2" t="inlineStr">
+        <is>
+          <t>RN8-PC-TB-S</t>
+        </is>
+      </c>
+      <c r="B84" s="3" t="inlineStr">
+        <is>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C84" s="3" t="inlineStr">
+        <is>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+        </is>
+      </c>
+      <c r="D84" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E84" s="2" t="inlineStr">
+        <is>
+          <t>Titanium Black</t>
+        </is>
+      </c>
+      <c r="F84" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G84" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H84" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I84" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+        </is>
+      </c>
+      <c r="J84" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-TB-S.jpg</t>
+        </is>
+      </c>
+      <c r="K84" s="4" t="n">
+        <v>147.74</v>
+      </c>
+      <c r="L84" s="4" t="n">
+        <v>60</v>
+      </c>
+      <c r="M84" s="4" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="N84" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O84" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P84" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q84" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R84" s="4">
+        <f>SUM(K84:Q84)</f>
+        <v/>
+      </c>
+      <c r="S84" s="4">
+        <f>IF(R84&lt;300, R84*1.4, IF(R84&lt;400, R84*1.33, R84*1.25))</f>
+        <v/>
+      </c>
+      <c r="T84" s="5">
+        <f>INT(S84/100)*100 + IF(MOD(ROUND(S84,0),100)&lt;25, 0, IF(MOD(ROUND(S84,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U84" s="4">
+        <f>IF(T84&lt;300, 0, MIN(99, IF(T84&lt;500, T84*7%, IF(T84&lt;700, T84*12%, T84*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" s="6" t="inlineStr">
+        <is>
+          <t>RN8-PC-GD-S</t>
+        </is>
+      </c>
+      <c r="B85" s="7" t="inlineStr">
+        <is>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C85" s="7" t="inlineStr">
+        <is>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+        </is>
+      </c>
+      <c r="D85" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E85" s="6" t="inlineStr">
+        <is>
+          <t>Golden</t>
+        </is>
+      </c>
+      <c r="F85" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G85" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H85" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I85" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+        </is>
+      </c>
+      <c r="J85" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-GD-S.jpg</t>
+        </is>
+      </c>
+      <c r="K85" s="8" t="n">
+        <v>147.74</v>
+      </c>
+      <c r="L85" s="8" t="n">
+        <v>60</v>
+      </c>
+      <c r="M85" s="8" t="n">
+        <v>62.4</v>
+      </c>
+      <c r="N85" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O85" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P85" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q85" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R85" s="8">
+        <f>SUM(K85:Q85)</f>
+        <v/>
+      </c>
+      <c r="S85" s="8">
+        <f>IF(R85&lt;300, R85*1.4, IF(R85&lt;400, R85*1.33, R85*1.25))</f>
+        <v/>
+      </c>
+      <c r="T85" s="9">
+        <f>INT(S85/100)*100 + IF(MOD(ROUND(S85,0),100)&lt;25, 0, IF(MOD(ROUND(S85,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U85" s="8">
+        <f>IF(T85&lt;300, 0, MIN(99, IF(T85&lt;500, T85*7%, IF(T85&lt;700, T85*12%, T85*15%))))</f>
+        <v/>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
feat: process Realme Neo8 (Tempered Glass) - pipeline complete
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U85"/>
+  <dimension ref="A1:U91"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -7494,7 +7494,7 @@
         <v>147.74</v>
       </c>
       <c r="L80" s="4" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M80" s="4" t="n">
         <v>62.4</v>
@@ -7583,7 +7583,7 @@
         <v>147.74</v>
       </c>
       <c r="L81" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M81" s="8" t="n">
         <v>62.4</v>
@@ -7672,7 +7672,7 @@
         <v>113.64</v>
       </c>
       <c r="L82" s="4" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M82" s="4" t="n">
         <v>62.4</v>
@@ -7761,7 +7761,7 @@
         <v>147.74</v>
       </c>
       <c r="L83" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M83" s="8" t="n">
         <v>62.4</v>
@@ -7850,7 +7850,7 @@
         <v>147.74</v>
       </c>
       <c r="L84" s="4" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M84" s="4" t="n">
         <v>62.4</v>
@@ -7939,7 +7939,7 @@
         <v>147.74</v>
       </c>
       <c r="L85" s="8" t="n">
-        <v>60</v>
+        <v>50</v>
       </c>
       <c r="M85" s="8" t="n">
         <v>62.4</v>
@@ -7970,6 +7970,540 @@
       </c>
       <c r="U85" s="8">
         <f>IF(T85&lt;300, 0, MIN(99, IF(T85&lt;500, T85*7%, IF(T85&lt;700, T85*12%, T85*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" s="2" t="inlineStr">
+        <is>
+          <t>RN8-GLS-YL-S</t>
+        </is>
+      </c>
+      <c r="B86" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+        </is>
+      </c>
+      <c r="C86" s="3" t="inlineStr">
+        <is>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+        </is>
+      </c>
+      <c r="D86" s="2" t="inlineStr">
+        <is>
+          <t>Tempered Glass</t>
+        </is>
+      </c>
+      <c r="E86" s="2" t="inlineStr">
+        <is>
+          <t>A6077 Collection Yellow</t>
+        </is>
+      </c>
+      <c r="F86" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G86" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H86" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I86" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+        </is>
+      </c>
+      <c r="J86" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-YL-S.jpg</t>
+        </is>
+      </c>
+      <c r="K86" s="4" t="n">
+        <v>156.83</v>
+      </c>
+      <c r="L86" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="M86" s="4" t="n">
+        <v>468</v>
+      </c>
+      <c r="N86" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O86" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P86" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q86" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R86" s="4">
+        <f>SUM(K86:Q86)</f>
+        <v/>
+      </c>
+      <c r="S86" s="4">
+        <f>IF(R86&lt;300, R86*1.4, IF(R86&lt;400, R86*1.33, R86*1.25))</f>
+        <v/>
+      </c>
+      <c r="T86" s="5">
+        <f>INT(S86/100)*100 + IF(MOD(ROUND(S86,0),100)&lt;25, 0, IF(MOD(ROUND(S86,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U86" s="4">
+        <f>IF(T86&lt;300, 0, MIN(99, IF(T86&lt;500, T86*7%, IF(T86&lt;700, T86*12%, T86*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" s="6" t="inlineStr">
+        <is>
+          <t>RN8-GLS-BL-S</t>
+        </is>
+      </c>
+      <c r="B87" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+        </is>
+      </c>
+      <c r="C87" s="7" t="inlineStr">
+        <is>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+        </is>
+      </c>
+      <c r="D87" s="6" t="inlineStr">
+        <is>
+          <t>Tempered Glass</t>
+        </is>
+      </c>
+      <c r="E87" s="6" t="inlineStr">
+        <is>
+          <t>A6078 Yuanzu Blue</t>
+        </is>
+      </c>
+      <c r="F87" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G87" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H87" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I87" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+        </is>
+      </c>
+      <c r="J87" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-BL-S.jpg</t>
+        </is>
+      </c>
+      <c r="K87" s="8" t="n">
+        <v>156.83</v>
+      </c>
+      <c r="L87" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="M87" s="8" t="n">
+        <v>468</v>
+      </c>
+      <c r="N87" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O87" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P87" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q87" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R87" s="8">
+        <f>SUM(K87:Q87)</f>
+        <v/>
+      </c>
+      <c r="S87" s="8">
+        <f>IF(R87&lt;300, R87*1.4, IF(R87&lt;400, R87*1.33, R87*1.25))</f>
+        <v/>
+      </c>
+      <c r="T87" s="9">
+        <f>INT(S87/100)*100 + IF(MOD(ROUND(S87,0),100)&lt;25, 0, IF(MOD(ROUND(S87,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U87" s="8">
+        <f>IF(T87&lt;300, 0, MIN(99, IF(T87&lt;500, T87*7%, IF(T87&lt;700, T87*12%, T87*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>RN8-GLS-GN-S</t>
+        </is>
+      </c>
+      <c r="B88" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+        </is>
+      </c>
+      <c r="C88" s="3" t="inlineStr">
+        <is>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+        </is>
+      </c>
+      <c r="D88" s="2" t="inlineStr">
+        <is>
+          <t>Tempered Glass</t>
+        </is>
+      </c>
+      <c r="E88" s="2" t="inlineStr">
+        <is>
+          <t>A6079 Passion Green</t>
+        </is>
+      </c>
+      <c r="F88" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G88" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H88" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I88" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+        </is>
+      </c>
+      <c r="J88" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-GN-S.jpg</t>
+        </is>
+      </c>
+      <c r="K88" s="4" t="n">
+        <v>156.83</v>
+      </c>
+      <c r="L88" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="M88" s="4" t="n">
+        <v>468</v>
+      </c>
+      <c r="N88" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O88" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P88" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q88" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R88" s="4">
+        <f>SUM(K88:Q88)</f>
+        <v/>
+      </c>
+      <c r="S88" s="4">
+        <f>IF(R88&lt;300, R88*1.4, IF(R88&lt;400, R88*1.33, R88*1.25))</f>
+        <v/>
+      </c>
+      <c r="T88" s="5">
+        <f>INT(S88/100)*100 + IF(MOD(ROUND(S88,0),100)&lt;25, 0, IF(MOD(ROUND(S88,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U88" s="4">
+        <f>IF(T88&lt;300, 0, MIN(99, IF(T88&lt;500, T88*7%, IF(T88&lt;700, T88*12%, T88*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" s="6" t="inlineStr">
+        <is>
+          <t>RN8-GLS-GY-S</t>
+        </is>
+      </c>
+      <c r="B89" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+        </is>
+      </c>
+      <c r="C89" s="7" t="inlineStr">
+        <is>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+        </is>
+      </c>
+      <c r="D89" s="6" t="inlineStr">
+        <is>
+          <t>Tempered Glass</t>
+        </is>
+      </c>
+      <c r="E89" s="6" t="inlineStr">
+        <is>
+          <t>A6080 Diamond Gray</t>
+        </is>
+      </c>
+      <c r="F89" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G89" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H89" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I89" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+        </is>
+      </c>
+      <c r="J89" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-GY-S.jpg</t>
+        </is>
+      </c>
+      <c r="K89" s="8" t="n">
+        <v>156.83</v>
+      </c>
+      <c r="L89" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="M89" s="8" t="n">
+        <v>468</v>
+      </c>
+      <c r="N89" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O89" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P89" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q89" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R89" s="8">
+        <f>SUM(K89:Q89)</f>
+        <v/>
+      </c>
+      <c r="S89" s="8">
+        <f>IF(R89&lt;300, R89*1.4, IF(R89&lt;400, R89*1.33, R89*1.25))</f>
+        <v/>
+      </c>
+      <c r="T89" s="9">
+        <f>INT(S89/100)*100 + IF(MOD(ROUND(S89,0),100)&lt;25, 0, IF(MOD(ROUND(S89,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U89" s="8">
+        <f>IF(T89&lt;300, 0, MIN(99, IF(T89&lt;500, T89*7%, IF(T89&lt;700, T89*12%, T89*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>RN8-GLS-PR-S</t>
+        </is>
+      </c>
+      <c r="B90" s="3" t="inlineStr">
+        <is>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+        </is>
+      </c>
+      <c r="C90" s="3" t="inlineStr">
+        <is>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+        </is>
+      </c>
+      <c r="D90" s="2" t="inlineStr">
+        <is>
+          <t>Tempered Glass</t>
+        </is>
+      </c>
+      <c r="E90" s="2" t="inlineStr">
+        <is>
+          <t>A6081 Ghost Purple</t>
+        </is>
+      </c>
+      <c r="F90" s="2" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G90" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H90" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I90" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+        </is>
+      </c>
+      <c r="J90" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-PR-S.jpg</t>
+        </is>
+      </c>
+      <c r="K90" s="4" t="n">
+        <v>156.83</v>
+      </c>
+      <c r="L90" s="4" t="n">
+        <v>45</v>
+      </c>
+      <c r="M90" s="4" t="n">
+        <v>468</v>
+      </c>
+      <c r="N90" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O90" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P90" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q90" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R90" s="4">
+        <f>SUM(K90:Q90)</f>
+        <v/>
+      </c>
+      <c r="S90" s="4">
+        <f>IF(R90&lt;300, R90*1.4, IF(R90&lt;400, R90*1.33, R90*1.25))</f>
+        <v/>
+      </c>
+      <c r="T90" s="5">
+        <f>INT(S90/100)*100 + IF(MOD(ROUND(S90,0),100)&lt;25, 0, IF(MOD(ROUND(S90,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U90" s="4">
+        <f>IF(T90&lt;300, 0, MIN(99, IF(T90&lt;500, T90*7%, IF(T90&lt;700, T90*12%, T90*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" s="6" t="inlineStr">
+        <is>
+          <t>RN8-GLS-RD-S</t>
+        </is>
+      </c>
+      <c r="B91" s="7" t="inlineStr">
+        <is>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+        </is>
+      </c>
+      <c r="C91" s="7" t="inlineStr">
+        <is>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+        </is>
+      </c>
+      <c r="D91" s="6" t="inlineStr">
+        <is>
+          <t>Tempered Glass</t>
+        </is>
+      </c>
+      <c r="E91" s="6" t="inlineStr">
+        <is>
+          <t>A6082 Alarm Red</t>
+        </is>
+      </c>
+      <c r="F91" s="6" t="inlineStr">
+        <is>
+          <t>Realme Neo8</t>
+        </is>
+      </c>
+      <c r="G91" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H91" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I91" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+        </is>
+      </c>
+      <c r="J91" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-RD-S.jpg</t>
+        </is>
+      </c>
+      <c r="K91" s="8" t="n">
+        <v>156.83</v>
+      </c>
+      <c r="L91" s="8" t="n">
+        <v>45</v>
+      </c>
+      <c r="M91" s="8" t="n">
+        <v>468</v>
+      </c>
+      <c r="N91" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O91" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P91" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q91" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R91" s="8">
+        <f>SUM(K91:Q91)</f>
+        <v/>
+      </c>
+      <c r="S91" s="8">
+        <f>IF(R91&lt;300, R91*1.4, IF(R91&lt;400, R91*1.33, R91*1.25))</f>
+        <v/>
+      </c>
+      <c r="T91" s="9">
+        <f>INT(S91/100)*100 + IF(MOD(ROUND(S91,0),100)&lt;25, 0, IF(MOD(ROUND(S91,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U91" s="8">
+        <f>IF(T91&lt;300, 0, MIN(99, IF(T91&lt;500, T91*7%, IF(T91&lt;700, T91*12%, T91*15%))))</f>
         <v/>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: process Samsung Galaxy S26 Ultra wood grain magnetic case with 20 BDT china delivery
</commit_message>
<xml_diff>
--- a/inventory.xlsx
+++ b/inventory.xlsx
@@ -476,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:U91"/>
+  <dimension ref="A1:U95"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -1883,27 +1883,27 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>S26U-PW-B-N</t>
+          <t>S26U-MI-B-N</t>
         </is>
       </c>
       <c r="B17" s="7" t="inlineStr">
         <is>
-          <t>Luxury Wood Grain Magnetic Case for Samsung Galaxy S26 Ultra – Slim Shockproof Hard Back Cover</t>
+          <t>Magnetic Invisible Stand Armor Case for Samsung Galaxy S26 Ultra – Heavy Duty Metal Lens Frame Hybrid Back Cover</t>
         </is>
       </c>
       <c r="C17" s="7" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
+          <t>Samsung Galaxy S26 Ultra Magnetic Invisible Bracket</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>PCs</t>
+          <t>Metal lens frame Acrylic / TPU</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>Poplar Wood Grain</t>
+          <t>Black – Magnetic Invisible Bracket</t>
         </is>
       </c>
       <c r="F17" s="6" t="inlineStr">
@@ -1923,21 +1923,21 @@
       </c>
       <c r="I17" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
+          <t>https://moveon.global/BD_en/products/0000000PWJ01ZSK1-metal-invisible-lens-bracket-suitable-for-samsung-s26ultra-magnetic-phone-case-s25fe-transparent-s24plus-case/1AC5307428543960</t>
         </is>
       </c>
       <c r="J17" s="7" t="inlineStr"/>
       <c r="K17" s="8" t="n">
-        <v>252.7</v>
+        <v>265.74</v>
       </c>
       <c r="L17" s="8" t="n">
-        <v>18.09</v>
+        <v>50.2</v>
       </c>
       <c r="M17" s="8" t="n">
-        <v>35</v>
+        <v>80</v>
       </c>
       <c r="N17" s="8" t="n">
-        <v>2.54</v>
+        <v>5.09</v>
       </c>
       <c r="O17" s="8" t="n">
         <v>11.5</v>
@@ -1968,32 +1968,32 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>S26U-PW-B-N</t>
+          <t>18P-AC-M-R-N</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>Luxury Wood Grain Magnetic Case for Samsung Galaxy S26 Ultra – Slim Shockproof Hard Back Cover</t>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S26 Ultra Wood Grain Magnetic Case</t>
+          <t>iPhone 18 Pro Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>PCs</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>Dark Gray Wood Grain</t>
+          <t>Wine Red</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S26 Ultra</t>
+          <t>iPhone 18 Pro</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
@@ -2008,21 +2008,21 @@
       </c>
       <c r="I18" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
+          <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
       <c r="J18" s="3" t="inlineStr"/>
       <c r="K18" s="4" t="n">
-        <v>252.7</v>
+        <v>87.25</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>18.09</v>
+        <v>16.55</v>
       </c>
       <c r="M18" s="4" t="n">
-        <v>35</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="N18" s="4" t="n">
-        <v>2.54</v>
+        <v>5.09</v>
       </c>
       <c r="O18" s="4" t="n">
         <v>11.5</v>
@@ -2053,32 +2053,32 @@
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>S26U-MI-B-N</t>
+          <t>18PM-AC-M-R-N</t>
         </is>
       </c>
       <c r="B19" s="7" t="inlineStr">
         <is>
-          <t>Magnetic Invisible Stand Armor Case for Samsung Galaxy S26 Ultra – Heavy Duty Metal Lens Frame Hybrid Back Cover</t>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
         </is>
       </c>
       <c r="C19" s="7" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S26 Ultra Magnetic Invisible Bracket</t>
+          <t>iPhone 18  Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Metal lens frame Acrylic / TPU</t>
+          <t>Acrylic</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>Black – Magnetic Invisible Bracket</t>
+          <t>Wine Red</t>
         </is>
       </c>
       <c r="F19" s="6" t="inlineStr">
         <is>
-          <t>Samsung Galaxy S26 Ultra</t>
+          <t>iPhone 18 Pro Max</t>
         </is>
       </c>
       <c r="G19" s="6" t="inlineStr">
@@ -2093,18 +2093,18 @@
       </c>
       <c r="I19" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000PWJ01ZSK1-metal-invisible-lens-bracket-suitable-for-samsung-s26ultra-magnetic-phone-case-s25fe-transparent-s24plus-case/1AC5307428543960</t>
+          <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
         </is>
       </c>
       <c r="J19" s="7" t="inlineStr"/>
       <c r="K19" s="8" t="n">
-        <v>265.74</v>
+        <v>87.25</v>
       </c>
       <c r="L19" s="8" t="n">
-        <v>50.2</v>
+        <v>16.55</v>
       </c>
       <c r="M19" s="8" t="n">
-        <v>80</v>
+        <v>81.59999999999999</v>
       </c>
       <c r="N19" s="8" t="n">
         <v>5.09</v>
@@ -2138,7 +2138,7 @@
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
         <is>
-          <t>18P-AC-M-R-N</t>
+          <t>18PM-AC-M-B-N</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
@@ -2148,7 +2148,7 @@
       </c>
       <c r="C20" s="3" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro Magnetic Acrylic Case</t>
+          <t>iPhone 18  Pro  Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -2158,7 +2158,7 @@
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Wine Red</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
@@ -2223,17 +2223,17 @@
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>18PM-AC-M-R-N</t>
+          <t>17PM-AC-M-O-N</t>
         </is>
       </c>
       <c r="B21" s="7" t="inlineStr">
         <is>
-          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 17 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
         </is>
       </c>
       <c r="C21" s="7" t="inlineStr">
         <is>
-          <t>iPhone 18  Pro Max Magnetic Acrylic Case</t>
+          <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
@@ -2243,12 +2243,12 @@
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>Wine Red</t>
+          <t>Orange</t>
         </is>
       </c>
       <c r="F21" s="6" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro Max</t>
+          <t>iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="G21" s="6" t="inlineStr">
@@ -2308,17 +2308,17 @@
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
         <is>
-          <t>18PM-AC-M-B-N</t>
+          <t>17PM-AC-M-PK-N</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Luxury Magnetic Clear Acrylic Case for iPhone 18 Pro – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+          <t>Luxury Magnetic Clear Acrylic Case for iPhone 17 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
         </is>
       </c>
       <c r="C22" s="3" t="inlineStr">
         <is>
-          <t>iPhone 18  Pro  Magnetic Acrylic Case</t>
+          <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -2328,12 +2328,12 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Pink</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro</t>
+          <t>iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
@@ -2393,32 +2393,32 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>17PM-AC-M-O-N</t>
+          <t>18PM-HS-S-N</t>
         </is>
       </c>
       <c r="B23" s="7" t="inlineStr">
         <is>
-          <t>Luxury Magnetic Clear Acrylic Case for iPhone 17 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 18 Pro Max – Luxury Anti-Scratch Protective Back Cover</t>
         </is>
       </c>
       <c r="C23" s="7" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
+          <t>iPhone 18 Pro Max Hard Shell Case with Lens Film</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>PCs</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>Orange</t>
+          <t>Elegant Silver</t>
         </is>
       </c>
       <c r="F23" s="6" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max</t>
+          <t>iPhone 18 Pro Max</t>
         </is>
       </c>
       <c r="G23" s="6" t="inlineStr">
@@ -2433,21 +2433,21 @@
       </c>
       <c r="I23" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
+          <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
       <c r="J23" s="7" t="inlineStr"/>
       <c r="K23" s="8" t="n">
-        <v>87.25</v>
+        <v>119.7</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>16.55</v>
+        <v>8.75</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>81.59999999999999</v>
+        <v>38</v>
       </c>
       <c r="N23" s="8" t="n">
-        <v>5.09</v>
+        <v>2.54</v>
       </c>
       <c r="O23" s="8" t="n">
         <v>11.5</v>
@@ -2478,32 +2478,32 @@
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
         <is>
-          <t>17PM-AC-M-PK-N</t>
+          <t>18P-HS-S-N</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr">
         <is>
-          <t>Luxury Magnetic Clear Acrylic Case for iPhone 17 Pro Max – Anti-Yellow Shockproof Hard Hybrid Back Cover</t>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 18 Pro – Luxury Anti-Scratch Protective Back Cover</t>
         </is>
       </c>
       <c r="C24" s="3" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max Magnetic Acrylic Case</t>
+          <t>iPhone 18 Pro Hard Shell Case with Lens Film</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>Acrylic</t>
+          <t>PCs</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Pink</t>
+          <t>Elegant Silver</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max</t>
+          <t>iPhone 18 Pro</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
@@ -2518,21 +2518,21 @@
       </c>
       <c r="I24" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000XI6T00NZT-suitable-for-apple-18promax-phone-case-magnetic-transparent-iphone17-acrylic-silicone-solid-color-skin-feel-frame/1AD8357853016175</t>
+          <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
         </is>
       </c>
       <c r="J24" s="3" t="inlineStr"/>
       <c r="K24" s="4" t="n">
-        <v>87.25</v>
+        <v>119.7</v>
       </c>
       <c r="L24" s="4" t="n">
-        <v>16.55</v>
+        <v>8.75</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>81.59999999999999</v>
+        <v>38</v>
       </c>
       <c r="N24" s="4" t="n">
-        <v>5.09</v>
+        <v>2.54</v>
       </c>
       <c r="O24" s="4" t="n">
         <v>11.5</v>
@@ -2563,17 +2563,17 @@
     <row r="25">
       <c r="A25" s="6" t="inlineStr">
         <is>
-          <t>18PM-HS-S-N</t>
+          <t>17PM-HS-S-N</t>
         </is>
       </c>
       <c r="B25" s="7" t="inlineStr">
         <is>
-          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 18 Pro Max – Luxury Anti-Scratch Protective Back Cover</t>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 17 Pro Max – Luxury Anti-Scratch Protective Back Cover</t>
         </is>
       </c>
       <c r="C25" s="7" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro Max Hard Shell Case with Lens Film</t>
+          <t>iPhone 17 Pro Max Hard Shell Case with Lens Film</t>
         </is>
       </c>
       <c r="D25" s="6" t="inlineStr">
@@ -2588,7 +2588,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro Max</t>
+          <t>iPhone 17 Pro Max</t>
         </is>
       </c>
       <c r="G25" s="6" t="inlineStr">
@@ -2648,17 +2648,17 @@
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
         <is>
-          <t>18P-HS-S-N</t>
+          <t>17P-HS-S-N</t>
         </is>
       </c>
       <c r="B26" s="3" t="inlineStr">
         <is>
-          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 18 Pro – Luxury Anti-Scratch Protective Back Cover</t>
+          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 17 Pro – Luxury Anti-Scratch Protective Back Cover</t>
         </is>
       </c>
       <c r="C26" s="3" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro Hard Shell Case with Lens Film</t>
+          <t>iPhone 17 Pro Hard Shell Case with Lens Film</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -2673,7 +2673,7 @@
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>iPhone 18 Pro</t>
+          <t>iPhone 17 Pro</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
@@ -2733,32 +2733,32 @@
     <row r="27">
       <c r="A27" s="6" t="inlineStr">
         <is>
-          <t>17PM-HS-S-N</t>
+          <t>RN8-SIL-WT-S</t>
         </is>
       </c>
       <c r="B27" s="7" t="inlineStr">
         <is>
-          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 17 Pro Max – Luxury Anti-Scratch Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
         </is>
       </c>
       <c r="C27" s="7" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max Hard Shell Case with Lens Film</t>
+          <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
       <c r="D27" s="6" t="inlineStr">
         <is>
-          <t>PCs</t>
+          <t>Liquid Silicone</t>
         </is>
       </c>
       <c r="E27" s="6" t="inlineStr">
         <is>
-          <t>Elegant Silver</t>
+          <t>Antique White</t>
         </is>
       </c>
       <c r="F27" s="6" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Max</t>
+          <t>Realme Neo8</t>
         </is>
       </c>
       <c r="G27" s="6" t="inlineStr">
@@ -2773,21 +2773,25 @@
       </c>
       <c r="I27" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
-        </is>
-      </c>
-      <c r="J27" s="7" t="inlineStr"/>
+          <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
+        </is>
+      </c>
+      <c r="J27" s="7" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S.jpg</t>
+        </is>
+      </c>
       <c r="K27" s="8" t="n">
-        <v>119.7</v>
+        <v>34.09</v>
       </c>
       <c r="L27" s="8" t="n">
-        <v>8.75</v>
+        <v>10</v>
       </c>
       <c r="M27" s="8" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="N27" s="8" t="n">
-        <v>2.54</v>
+        <v>5</v>
       </c>
       <c r="O27" s="8" t="n">
         <v>11.5</v>
@@ -2818,32 +2822,32 @@
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
-          <t>17P-HS-S-N</t>
+          <t>RN8-SIL-PR-S</t>
         </is>
       </c>
       <c r="B28" s="3" t="inlineStr">
         <is>
-          <t>Ultra-Slim Matte Hard Case with Camera Lens Protector for iPhone 17 Pro – Luxury Anti-Scratch Protective Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
         </is>
       </c>
       <c r="C28" s="3" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro Hard Shell Case with Lens Film</t>
+          <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>PCs</t>
+          <t>Liquid Silicone</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Elegant Silver</t>
+          <t>Grass Purple</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>iPhone 17 Pro</t>
+          <t>Realme Neo8</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
@@ -2858,21 +2862,25 @@
       </c>
       <c r="I28" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000BB3D8VSG8-suitable-for-iphone18promax-mobile-phone-case-ultra-thin-matte-heat-dissipation-apple-17-lens-film-all-inclusive-anti-fall-hard-case/1AC6111333736340</t>
-        </is>
-      </c>
-      <c r="J28" s="3" t="inlineStr"/>
+          <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
+        </is>
+      </c>
       <c r="K28" s="4" t="n">
-        <v>119.7</v>
+        <v>34.09</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>8.75</v>
+        <v>10</v>
       </c>
       <c r="M28" s="4" t="n">
-        <v>38</v>
+        <v>50</v>
       </c>
       <c r="N28" s="4" t="n">
-        <v>2.54</v>
+        <v>5</v>
       </c>
       <c r="O28" s="4" t="n">
         <v>11.5</v>
@@ -2903,7 +2911,7 @@
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-WT-S</t>
+          <t>RN8-SIL-GN-S</t>
         </is>
       </c>
       <c r="B29" s="7" t="inlineStr">
@@ -2923,7 +2931,7 @@
       </c>
       <c r="E29" s="6" t="inlineStr">
         <is>
-          <t>Antique White</t>
+          <t>Dark Night Green</t>
         </is>
       </c>
       <c r="F29" s="6" t="inlineStr">
@@ -2948,7 +2956,7 @@
       </c>
       <c r="J29" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S.jpg</t>
         </is>
       </c>
       <c r="K29" s="8" t="n">
@@ -2992,7 +3000,7 @@
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-PR-S</t>
+          <t>RN8-SIL-BL-S</t>
         </is>
       </c>
       <c r="B30" s="3" t="inlineStr">
@@ -3012,7 +3020,7 @@
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Grass Purple</t>
+          <t>Royal Blue</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
@@ -3037,7 +3045,7 @@
       </c>
       <c r="J30" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S.jpg</t>
         </is>
       </c>
       <c r="K30" s="4" t="n">
@@ -3081,7 +3089,7 @@
     <row r="31">
       <c r="A31" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-GN-S</t>
+          <t>RN8-SIL-BK-S</t>
         </is>
       </c>
       <c r="B31" s="7" t="inlineStr">
@@ -3101,7 +3109,7 @@
       </c>
       <c r="E31" s="6" t="inlineStr">
         <is>
-          <t>Dark Night Green</t>
+          <t>Classic Black</t>
         </is>
       </c>
       <c r="F31" s="6" t="inlineStr">
@@ -3126,7 +3134,7 @@
       </c>
       <c r="J31" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S.jpg</t>
         </is>
       </c>
       <c r="K31" s="8" t="n">
@@ -3170,7 +3178,7 @@
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-BL-S</t>
+          <t>RN8-SIL-GY-S</t>
         </is>
       </c>
       <c r="B32" s="3" t="inlineStr">
@@ -3190,7 +3198,7 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Royal Blue</t>
+          <t>Lavender Gray</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
@@ -3215,7 +3223,7 @@
       </c>
       <c r="J32" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GY-S.jpg</t>
         </is>
       </c>
       <c r="K32" s="4" t="n">
@@ -3259,7 +3267,7 @@
     <row r="33">
       <c r="A33" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-BK-S</t>
+          <t>RN8-SIL-RD-S</t>
         </is>
       </c>
       <c r="B33" s="7" t="inlineStr">
@@ -3279,7 +3287,7 @@
       </c>
       <c r="E33" s="6" t="inlineStr">
         <is>
-          <t>Classic Black</t>
+          <t>Camellia Red</t>
         </is>
       </c>
       <c r="F33" s="6" t="inlineStr">
@@ -3304,7 +3312,7 @@
       </c>
       <c r="J33" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-RD-S.jpg</t>
         </is>
       </c>
       <c r="K33" s="8" t="n">
@@ -3348,7 +3356,7 @@
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-GY-S</t>
+          <t>RN8-SIL-TL-S</t>
         </is>
       </c>
       <c r="B34" s="3" t="inlineStr">
@@ -3368,7 +3376,7 @@
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Lavender Gray</t>
+          <t>Light Teal</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
@@ -3393,7 +3401,7 @@
       </c>
       <c r="J34" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GY-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-TL-S.jpg</t>
         </is>
       </c>
       <c r="K34" s="4" t="n">
@@ -3437,7 +3445,7 @@
     <row r="35">
       <c r="A35" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-RD-S</t>
+          <t>RN8-SIL-CL-C</t>
         </is>
       </c>
       <c r="B35" s="7" t="inlineStr">
@@ -3457,7 +3465,7 @@
       </c>
       <c r="E35" s="6" t="inlineStr">
         <is>
-          <t>Camellia Red</t>
+          <t>Transparent</t>
         </is>
       </c>
       <c r="F35" s="6" t="inlineStr">
@@ -3482,7 +3490,7 @@
       </c>
       <c r="J35" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-RD-S.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-CL-C.jpg</t>
         </is>
       </c>
       <c r="K35" s="8" t="n">
@@ -3526,27 +3534,27 @@
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-TL-S</t>
+          <t>RN8-TPU-WT-M</t>
         </is>
       </c>
       <c r="B36" s="3" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Magnetic Ultra-Thin Shockproof Case for Realme GT Neo 8 – Slim Soft TPU Full Protection Back Cover</t>
         </is>
       </c>
       <c r="C36" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>Liquid Silicone</t>
+          <t>TPU</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Light Teal</t>
+          <t>Transparent White</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
@@ -3566,16 +3574,16 @@
       </c>
       <c r="I36" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
+          <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
         </is>
       </c>
       <c r="J36" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-TL-S.jpg</t>
+          <t>Realme Neo8/TPU/sku/RN8-TPU-WT-M.jpg</t>
         </is>
       </c>
       <c r="K36" s="4" t="n">
-        <v>34.09</v>
+        <v>133</v>
       </c>
       <c r="L36" s="4" t="n">
         <v>10</v>
@@ -3615,27 +3623,27 @@
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-CL-C</t>
+          <t>RN8-TPU-BK-M</t>
         </is>
       </c>
       <c r="B37" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Skin-Friendly Soft Cube Anti-Drop Protective Back Cover</t>
+          <t>Magnetic Ultra-Thin Shockproof Case for Realme GT Neo 8 – Slim Soft TPU Full Protection Back Cover</t>
         </is>
       </c>
       <c r="C37" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 phone case, simple solid color cube liquid silicone full-cover anti-drop soft case, new model</t>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>Liquid Silicone</t>
+          <t>TPU</t>
         </is>
       </c>
       <c r="E37" s="6" t="inlineStr">
         <is>
-          <t>Transparent</t>
+          <t>Transparent Black</t>
         </is>
       </c>
       <c r="F37" s="6" t="inlineStr">
@@ -3655,16 +3663,16 @@
       </c>
       <c r="I37" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000MJPDSKGCI-suitable-for-realme-neo8-phone-case-simple-solid-color-cube-liquid-silicone-full-cover-anti-drop-soft-case-new-model/1AD8354574484115</t>
+          <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
         </is>
       </c>
       <c r="J37" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-CL-C.jpg</t>
+          <t>Realme Neo8/TPU/sku/RN8-TPU-BK-M.jpg</t>
         </is>
       </c>
       <c r="K37" s="8" t="n">
-        <v>34.09</v>
+        <v>133</v>
       </c>
       <c r="L37" s="8" t="n">
         <v>10</v>
@@ -3704,32 +3712,32 @@
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
         <is>
-          <t>RN8-TPU-WT-M</t>
+          <t>H600L-SIL-BK-M</t>
         </is>
       </c>
       <c r="B38" s="3" t="inlineStr">
         <is>
-          <t>Magnetic Ultra-Thin Shockproof Case for Realme GT Neo 8 – Slim Soft TPU Full Protection Back Cover</t>
+          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
         </is>
       </c>
       <c r="C38" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
+          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>Silicone</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>Transparent White</t>
+          <t>Moiré Black</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>Realme Neo8</t>
+          <t>Honor 600 lite</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
@@ -3744,22 +3752,22 @@
       </c>
       <c r="I38" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
+          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
         </is>
       </c>
       <c r="J38" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/TPU/sku/RN8-TPU-WT-M.jpg</t>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-BK-M.jpg</t>
         </is>
       </c>
       <c r="K38" s="4" t="n">
-        <v>133</v>
+        <v>186.2</v>
       </c>
       <c r="L38" s="4" t="n">
         <v>10</v>
       </c>
       <c r="M38" s="4" t="n">
-        <v>50</v>
+        <v>156</v>
       </c>
       <c r="N38" s="4" t="n">
         <v>5</v>
@@ -3793,32 +3801,32 @@
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>RN8-TPU-BK-M</t>
+          <t>H600L-SIL-BL-M</t>
         </is>
       </c>
       <c r="B39" s="7" t="inlineStr">
         <is>
-          <t>Magnetic Ultra-Thin Shockproof Case for Realme GT Neo 8 – Slim Soft TPU Full Protection Back Cover</t>
+          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
         </is>
       </c>
       <c r="C39" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 Mobile Phone Case, Magnetic Ultra-Thin Soft Case, Realme Thin Neo8 Protective Case, Tpu Full Cover</t>
+          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>Silicone</t>
         </is>
       </c>
       <c r="E39" s="6" t="inlineStr">
         <is>
-          <t>Transparent Black</t>
+          <t>Gentleman Blue</t>
         </is>
       </c>
       <c r="F39" s="6" t="inlineStr">
         <is>
-          <t>Realme Neo8</t>
+          <t>Honor 600 lite</t>
         </is>
       </c>
       <c r="G39" s="6" t="inlineStr">
@@ -3833,22 +3841,22 @@
       </c>
       <c r="I39" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000J0H1734SE-suitable-for-realme-neo8-mobile-phone-case-magnetic-ultra-thin-soft-case-realme-thin-neo8-protective-case-tpu-full-cover/1AD8318293575646</t>
+          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
         </is>
       </c>
       <c r="J39" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/TPU/sku/RN8-TPU-BK-M.jpg</t>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-BL-M.jpg</t>
         </is>
       </c>
       <c r="K39" s="8" t="n">
-        <v>133</v>
+        <v>186.2</v>
       </c>
       <c r="L39" s="8" t="n">
         <v>10</v>
       </c>
       <c r="M39" s="8" t="n">
-        <v>50</v>
+        <v>156</v>
       </c>
       <c r="N39" s="8" t="n">
         <v>5</v>
@@ -3882,7 +3890,7 @@
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
         <is>
-          <t>H600L-SIL-BK-M</t>
+          <t>H600L-SIL-GN-M</t>
         </is>
       </c>
       <c r="B40" s="3" t="inlineStr">
@@ -3902,7 +3910,7 @@
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>Moiré Black</t>
+          <t>Dark Night Green</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
@@ -3927,7 +3935,7 @@
       </c>
       <c r="J40" s="3" t="inlineStr">
         <is>
-          <t>Honor 600 lite/Silicone/sku/H600L-SIL-BK-M.jpg</t>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-GN-M.jpg</t>
         </is>
       </c>
       <c r="K40" s="4" t="n">
@@ -3971,7 +3979,7 @@
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>H600L-SIL-BL-M</t>
+          <t>H600L-SIL-RD-M</t>
         </is>
       </c>
       <c r="B41" s="7" t="inlineStr">
@@ -3991,7 +3999,7 @@
       </c>
       <c r="E41" s="6" t="inlineStr">
         <is>
-          <t>Gentleman Blue</t>
+          <t>Charming Red</t>
         </is>
       </c>
       <c r="F41" s="6" t="inlineStr">
@@ -4016,7 +4024,7 @@
       </c>
       <c r="J41" s="7" t="inlineStr">
         <is>
-          <t>Honor 600 lite/Silicone/sku/H600L-SIL-BL-M.jpg</t>
+          <t>Honor 600 lite/Silicone/sku/H600L-SIL-RD-M.jpg</t>
         </is>
       </c>
       <c r="K41" s="8" t="n">
@@ -4060,32 +4068,32 @@
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
         <is>
-          <t>H600L-SIL-GN-M</t>
+          <t>HX80I-TPU-SV-E</t>
         </is>
       </c>
       <c r="B42" s="3" t="inlineStr">
         <is>
-          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
         </is>
       </c>
       <c r="C42" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Silicone</t>
+          <t>TPU</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>Dark Night Green</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>Honor 600 lite</t>
+          <t>Honor X80i</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
@@ -4100,22 +4108,22 @@
       </c>
       <c r="I42" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
       <c r="J42" s="3" t="inlineStr">
         <is>
-          <t>Honor 600 lite/Silicone/sku/H600L-SIL-GN-M.jpg</t>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-SV-E.jpg</t>
         </is>
       </c>
       <c r="K42" s="4" t="n">
-        <v>186.2</v>
+        <v>234.08</v>
       </c>
       <c r="L42" s="4" t="n">
         <v>10</v>
       </c>
       <c r="M42" s="4" t="n">
-        <v>156</v>
+        <v>50</v>
       </c>
       <c r="N42" s="4" t="n">
         <v>5</v>
@@ -4149,32 +4157,32 @@
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>H600L-SIL-RD-M</t>
+          <t>HX80I-TPU-BK-E</t>
         </is>
       </c>
       <c r="B43" s="7" t="inlineStr">
         <is>
-          <t>Magnetic Liquid Silicone Case for Honor 600 Lite – Moiré Texture Anti-Scratch Soft Protective Back Cover</t>
+          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
         </is>
       </c>
       <c r="C43" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Honor 600Lite Foreign Version Mobile Phone Case Protective Cover with Built-In Magnetic Suction, Lightweight, Fine Holes, and Hard Shell</t>
+          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>Silicone</t>
+          <t>TPU</t>
         </is>
       </c>
       <c r="E43" s="6" t="inlineStr">
         <is>
-          <t>Charming Red</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="F43" s="6" t="inlineStr">
         <is>
-          <t>Honor 600 lite</t>
+          <t>Honor X80i</t>
         </is>
       </c>
       <c r="G43" s="6" t="inlineStr">
@@ -4189,22 +4197,22 @@
       </c>
       <c r="I43" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000DCI2M1DIF-suitable-for-honor-600lite-foreign-version-mobile-phone-case-protective-cover-with-built-in-magnetic-suction-lightweight-fine-holes-and-hard-shell/1AD8320205925874</t>
+          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
         </is>
       </c>
       <c r="J43" s="7" t="inlineStr">
         <is>
-          <t>Honor 600 lite/Silicone/sku/H600L-SIL-RD-M.jpg</t>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-BK-E.jpg</t>
         </is>
       </c>
       <c r="K43" s="8" t="n">
-        <v>186.2</v>
+        <v>234.08</v>
       </c>
       <c r="L43" s="8" t="n">
         <v>10</v>
       </c>
       <c r="M43" s="8" t="n">
-        <v>156</v>
+        <v>50</v>
       </c>
       <c r="N43" s="8" t="n">
         <v>5</v>
@@ -4238,7 +4246,7 @@
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
         <is>
-          <t>HX80I-TPU-SV-E</t>
+          <t>HX80I-TPU-PR-E</t>
         </is>
       </c>
       <c r="B44" s="3" t="inlineStr">
@@ -4258,7 +4266,7 @@
       </c>
       <c r="E44" s="2" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Purple</t>
         </is>
       </c>
       <c r="F44" s="2" t="inlineStr">
@@ -4283,7 +4291,7 @@
       </c>
       <c r="J44" s="3" t="inlineStr">
         <is>
-          <t>Honor X80i/TPU/sku/HX80I-TPU-SV-E.jpg</t>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-PR-E.jpg</t>
         </is>
       </c>
       <c r="K44" s="4" t="n">
@@ -4327,7 +4335,7 @@
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>HX80I-TPU-BK-E</t>
+          <t>HX80I-TPU-BL-E</t>
         </is>
       </c>
       <c r="B45" s="7" t="inlineStr">
@@ -4347,7 +4355,7 @@
       </c>
       <c r="E45" s="6" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="F45" s="6" t="inlineStr">
@@ -4372,7 +4380,7 @@
       </c>
       <c r="J45" s="7" t="inlineStr">
         <is>
-          <t>Honor X80i/TPU/sku/HX80I-TPU-BK-E.jpg</t>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-BL-E.jpg</t>
         </is>
       </c>
       <c r="K45" s="8" t="n">
@@ -4416,7 +4424,7 @@
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
         <is>
-          <t>HX80I-TPU-PR-E</t>
+          <t>HX80I-TPU-PK-E</t>
         </is>
       </c>
       <c r="B46" s="3" t="inlineStr">
@@ -4436,7 +4444,7 @@
       </c>
       <c r="E46" s="2" t="inlineStr">
         <is>
-          <t>Purple</t>
+          <t>Pink</t>
         </is>
       </c>
       <c r="F46" s="2" t="inlineStr">
@@ -4461,7 +4469,7 @@
       </c>
       <c r="J46" s="3" t="inlineStr">
         <is>
-          <t>Honor X80i/TPU/sku/HX80I-TPU-PR-E.jpg</t>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-PK-E.jpg</t>
         </is>
       </c>
       <c r="K46" s="4" t="n">
@@ -4505,7 +4513,7 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>HX80I-TPU-BL-E</t>
+          <t>HX80I-TPU-GN-E</t>
         </is>
       </c>
       <c r="B47" s="7" t="inlineStr">
@@ -4525,7 +4533,7 @@
       </c>
       <c r="E47" s="6" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="F47" s="6" t="inlineStr">
@@ -4550,7 +4558,7 @@
       </c>
       <c r="J47" s="7" t="inlineStr">
         <is>
-          <t>Honor X80i/TPU/sku/HX80I-TPU-BL-E.jpg</t>
+          <t>Honor X80i/TPU/sku/HX80I-TPU-GN-E.jpg</t>
         </is>
       </c>
       <c r="K47" s="8" t="n">
@@ -4594,32 +4602,32 @@
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
         <is>
-          <t>HX80I-TPU-PK-E</t>
+          <t>HX80I-PC-GY-M</t>
         </is>
       </c>
       <c r="B48" s="3" t="inlineStr">
         <is>
-          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
         </is>
       </c>
       <c r="C48" s="3" t="inlineStr">
         <is>
-          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>Hard PC</t>
         </is>
       </c>
       <c r="E48" s="2" t="inlineStr">
         <is>
-          <t>Pink</t>
+          <t>Titanium Gray</t>
         </is>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
-          <t>Honor X80i</t>
+          <t>Honor x80i</t>
         </is>
       </c>
       <c r="G48" s="2" t="inlineStr">
@@ -4634,16 +4642,16 @@
       </c>
       <c r="I48" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
       <c r="J48" s="3" t="inlineStr">
         <is>
-          <t>Honor X80i/TPU/sku/HX80I-TPU-PK-E.jpg</t>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-GY-M.jpg</t>
         </is>
       </c>
       <c r="K48" s="4" t="n">
-        <v>234.08</v>
+        <v>478.8</v>
       </c>
       <c r="L48" s="4" t="n">
         <v>10</v>
@@ -4683,32 +4691,32 @@
     <row r="49">
       <c r="A49" s="6" t="inlineStr">
         <is>
-          <t>HX80I-TPU-GN-E</t>
+          <t>HX80I-PC-WT-M</t>
         </is>
       </c>
       <c r="B49" s="7" t="inlineStr">
         <is>
-          <t>Invisible Kickstand Airbag Shockproof Case for Honor X80i / X70 / X60 Pro – Clear Hybrid TPU Protective Back Cover</t>
+          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
         </is>
       </c>
       <c r="C49" s="7" t="inlineStr">
         <is>
-          <t>Sangjieshi Suitable for Honor X80Promax Mobile Phone Case X70 with Stand X60Pro Transparent X50 Full-Cover Airbag</t>
+          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
         </is>
       </c>
       <c r="D49" s="6" t="inlineStr">
         <is>
-          <t>TPU</t>
+          <t>Hard PC</t>
         </is>
       </c>
       <c r="E49" s="6" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Silver White</t>
         </is>
       </c>
       <c r="F49" s="6" t="inlineStr">
         <is>
-          <t>Honor X80i</t>
+          <t>Honor x80i</t>
         </is>
       </c>
       <c r="G49" s="6" t="inlineStr">
@@ -4723,16 +4731,16 @@
       </c>
       <c r="I49" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000125WCGFR9-sangjieshi-suitable-for-honor-x80promax-mobile-phone-case-x70-with-stand-x60pro-transparent-x50-full-cover-airbag/1AD8341131122671</t>
+          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
         </is>
       </c>
       <c r="J49" s="7" t="inlineStr">
         <is>
-          <t>Honor X80i/TPU/sku/HX80I-TPU-GN-E.jpg</t>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-WT-M.jpg</t>
         </is>
       </c>
       <c r="K49" s="8" t="n">
-        <v>234.08</v>
+        <v>478.8</v>
       </c>
       <c r="L49" s="8" t="n">
         <v>10</v>
@@ -4772,7 +4780,7 @@
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
         <is>
-          <t>HX80I-PC-GY-M</t>
+          <t>HX80I-PC-GN-M</t>
         </is>
       </c>
       <c r="B50" s="3" t="inlineStr">
@@ -4792,7 +4800,7 @@
       </c>
       <c r="E50" s="2" t="inlineStr">
         <is>
-          <t>Titanium Gray</t>
+          <t>Feitianqing</t>
         </is>
       </c>
       <c r="F50" s="2" t="inlineStr">
@@ -4817,7 +4825,7 @@
       </c>
       <c r="J50" s="3" t="inlineStr">
         <is>
-          <t>Honor x80i/Hard PC/sku/HX80I-PC-GY-M.jpg</t>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-GN-M.jpg</t>
         </is>
       </c>
       <c r="K50" s="4" t="n">
@@ -4861,7 +4869,7 @@
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>HX80I-PC-WT-M</t>
+          <t>HX80I-PC-GD-M</t>
         </is>
       </c>
       <c r="B51" s="7" t="inlineStr">
@@ -4881,7 +4889,7 @@
       </c>
       <c r="E51" s="6" t="inlineStr">
         <is>
-          <t>Silver White</t>
+          <t>Desert Gold</t>
         </is>
       </c>
       <c r="F51" s="6" t="inlineStr">
@@ -4906,7 +4914,7 @@
       </c>
       <c r="J51" s="7" t="inlineStr">
         <is>
-          <t>Honor x80i/Hard PC/sku/HX80I-PC-WT-M.jpg</t>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-GD-M.jpg</t>
         </is>
       </c>
       <c r="K51" s="8" t="n">
@@ -4950,7 +4958,7 @@
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
         <is>
-          <t>HX80I-PC-GN-M</t>
+          <t>HX80I-PC-BK-M</t>
         </is>
       </c>
       <c r="B52" s="3" t="inlineStr">
@@ -4970,7 +4978,7 @@
       </c>
       <c r="E52" s="2" t="inlineStr">
         <is>
-          <t>Feitianqing</t>
+          <t>Graphite Black</t>
         </is>
       </c>
       <c r="F52" s="2" t="inlineStr">
@@ -4995,7 +5003,7 @@
       </c>
       <c r="J52" s="3" t="inlineStr">
         <is>
-          <t>Honor x80i/Hard PC/sku/HX80I-PC-GN-M.jpg</t>
+          <t>Honor x80i/Hard PC/sku/HX80I-PC-BK-M.jpg</t>
         </is>
       </c>
       <c r="K52" s="4" t="n">
@@ -5039,7 +5047,7 @@
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>HX80I-PC-GD-M</t>
+          <t>H600L-PC-GY-M</t>
         </is>
       </c>
       <c r="B53" s="7" t="inlineStr">
@@ -5059,12 +5067,12 @@
       </c>
       <c r="E53" s="6" t="inlineStr">
         <is>
-          <t>Desert Gold</t>
+          <t>Titanium Gray</t>
         </is>
       </c>
       <c r="F53" s="6" t="inlineStr">
         <is>
-          <t>Honor x80i</t>
+          <t>Honor 600lite foreign version</t>
         </is>
       </c>
       <c r="G53" s="6" t="inlineStr">
@@ -5084,7 +5092,7 @@
       </c>
       <c r="J53" s="7" t="inlineStr">
         <is>
-          <t>Honor x80i/Hard PC/sku/HX80I-PC-GD-M.jpg</t>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GY-M.jpg</t>
         </is>
       </c>
       <c r="K53" s="8" t="n">
@@ -5128,7 +5136,7 @@
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
         <is>
-          <t>HX80I-PC-BK-M</t>
+          <t>H600L-PC-WT-M</t>
         </is>
       </c>
       <c r="B54" s="3" t="inlineStr">
@@ -5148,12 +5156,12 @@
       </c>
       <c r="E54" s="2" t="inlineStr">
         <is>
-          <t>Graphite Black</t>
+          <t>Silver White</t>
         </is>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
-          <t>Honor x80i</t>
+          <t>Honor 600lite foreign version</t>
         </is>
       </c>
       <c r="G54" s="2" t="inlineStr">
@@ -5173,7 +5181,7 @@
       </c>
       <c r="J54" s="3" t="inlineStr">
         <is>
-          <t>Honor x80i/Hard PC/sku/HX80I-PC-BK-M.jpg</t>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-WT-M.jpg</t>
         </is>
       </c>
       <c r="K54" s="4" t="n">
@@ -5217,7 +5225,7 @@
     <row r="55">
       <c r="A55" s="6" t="inlineStr">
         <is>
-          <t>H600L-PC-GY-M</t>
+          <t>H600L-PC-GN-M</t>
         </is>
       </c>
       <c r="B55" s="7" t="inlineStr">
@@ -5237,7 +5245,7 @@
       </c>
       <c r="E55" s="6" t="inlineStr">
         <is>
-          <t>Titanium Gray</t>
+          <t>Feitianqing</t>
         </is>
       </c>
       <c r="F55" s="6" t="inlineStr">
@@ -5262,7 +5270,7 @@
       </c>
       <c r="J55" s="7" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GY-M.jpg</t>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GN-M.jpg</t>
         </is>
       </c>
       <c r="K55" s="8" t="n">
@@ -5306,7 +5314,7 @@
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
         <is>
-          <t>H600L-PC-WT-M</t>
+          <t>H600L-PC-GD-M</t>
         </is>
       </c>
       <c r="B56" s="3" t="inlineStr">
@@ -5326,7 +5334,7 @@
       </c>
       <c r="E56" s="2" t="inlineStr">
         <is>
-          <t>Silver White</t>
+          <t>Desert Gold</t>
         </is>
       </c>
       <c r="F56" s="2" t="inlineStr">
@@ -5351,7 +5359,7 @@
       </c>
       <c r="J56" s="3" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-WT-M.jpg</t>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GD-M.jpg</t>
         </is>
       </c>
       <c r="K56" s="4" t="n">
@@ -5395,7 +5403,7 @@
     <row r="57">
       <c r="A57" s="6" t="inlineStr">
         <is>
-          <t>H600L-PC-GN-M</t>
+          <t>H600L-PC-BK-M</t>
         </is>
       </c>
       <c r="B57" s="7" t="inlineStr">
@@ -5415,7 +5423,7 @@
       </c>
       <c r="E57" s="6" t="inlineStr">
         <is>
-          <t>Feitianqing</t>
+          <t>Graphite Black</t>
         </is>
       </c>
       <c r="F57" s="6" t="inlineStr">
@@ -5440,7 +5448,7 @@
       </c>
       <c r="J57" s="7" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GN-M.jpg</t>
+          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-BK-M.jpg</t>
         </is>
       </c>
       <c r="K57" s="8" t="n">
@@ -5484,17 +5492,17 @@
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
         <is>
-          <t>H600L-PC-GD-M</t>
+          <t>RN8-PC-RK-M</t>
         </is>
       </c>
       <c r="B58" s="3" t="inlineStr">
         <is>
-          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
         </is>
       </c>
       <c r="C58" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -5504,12 +5512,12 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>Desert Gold</t>
+          <t>Peak Rock Color</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version</t>
+          <t>Realme Neo8</t>
         </is>
       </c>
       <c r="G58" s="2" t="inlineStr">
@@ -5524,22 +5532,22 @@
       </c>
       <c r="I58" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
         </is>
       </c>
       <c r="J58" s="3" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-GD-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-RK-M.jpg</t>
         </is>
       </c>
       <c r="K58" s="4" t="n">
-        <v>478.8</v>
+        <v>367.08</v>
       </c>
       <c r="L58" s="4" t="n">
         <v>10</v>
       </c>
       <c r="M58" s="4" t="n">
-        <v>50</v>
+        <v>31.2</v>
       </c>
       <c r="N58" s="4" t="n">
         <v>5</v>
@@ -5573,17 +5581,17 @@
     <row r="59">
       <c r="A59" s="6" t="inlineStr">
         <is>
-          <t>H600L-PC-BK-M</t>
+          <t>RN8-PC-GD-M</t>
         </is>
       </c>
       <c r="B59" s="7" t="inlineStr">
         <is>
-          <t>Micro-Matte Magnetic Shockproof Case for Honor 600 Lite / Honor X80i – Ultra-Slim Hard Protective Back Cover</t>
+          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
         </is>
       </c>
       <c r="C59" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Huawei Honor X80I Mobile Phone Case, Honor 600Lite Micro-Matte Magnetic Protective Cover, All-Inclusive Anti-Fall Cover</t>
+          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
         </is>
       </c>
       <c r="D59" s="6" t="inlineStr">
@@ -5593,12 +5601,12 @@
       </c>
       <c r="E59" s="6" t="inlineStr">
         <is>
-          <t>Graphite Black</t>
+          <t>Desert Gold</t>
         </is>
       </c>
       <c r="F59" s="6" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version</t>
+          <t>Realme Neo8</t>
         </is>
       </c>
       <c r="G59" s="6" t="inlineStr">
@@ -5613,22 +5621,22 @@
       </c>
       <c r="I59" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000J9OECX1V4-suitable-for-huawei-honor-x80i-mobile-phone-case-honor-600lite-micro-matte-magnetic-protective-cover-all-inclusive-anti-fall-cover/1AD8344754691479</t>
+          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
         </is>
       </c>
       <c r="J59" s="7" t="inlineStr">
         <is>
-          <t>Honor 600lite foreign version/Hard PC/sku/H600L-PC-BK-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-GD-M.jpg</t>
         </is>
       </c>
       <c r="K59" s="8" t="n">
-        <v>478.8</v>
+        <v>367.08</v>
       </c>
       <c r="L59" s="8" t="n">
         <v>10</v>
       </c>
       <c r="M59" s="8" t="n">
-        <v>50</v>
+        <v>31.2</v>
       </c>
       <c r="N59" s="8" t="n">
         <v>5</v>
@@ -5662,7 +5670,7 @@
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-RK-M</t>
+          <t>RN8-PC-BL-M</t>
         </is>
       </c>
       <c r="B60" s="3" t="inlineStr">
@@ -5682,7 +5690,7 @@
       </c>
       <c r="E60" s="2" t="inlineStr">
         <is>
-          <t>Peak Rock Color</t>
+          <t>Wave Blue</t>
         </is>
       </c>
       <c r="F60" s="2" t="inlineStr">
@@ -5707,7 +5715,7 @@
       </c>
       <c r="J60" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-RK-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-BL-M.jpg</t>
         </is>
       </c>
       <c r="K60" s="4" t="n">
@@ -5751,7 +5759,7 @@
     <row r="61">
       <c r="A61" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-GD-M</t>
+          <t>RN8-PC-PK-M</t>
         </is>
       </c>
       <c r="B61" s="7" t="inlineStr">
@@ -5771,7 +5779,7 @@
       </c>
       <c r="E61" s="6" t="inlineStr">
         <is>
-          <t>Desert Gold</t>
+          <t>Sakura Pink</t>
         </is>
       </c>
       <c r="F61" s="6" t="inlineStr">
@@ -5796,7 +5804,7 @@
       </c>
       <c r="J61" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-GD-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-PK-M.jpg</t>
         </is>
       </c>
       <c r="K61" s="8" t="n">
@@ -5840,7 +5848,7 @@
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-BL-M</t>
+          <t>RN8-PC-CG-M</t>
         </is>
       </c>
       <c r="B62" s="3" t="inlineStr">
@@ -5860,7 +5868,7 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>Wave Blue</t>
+          <t>Carbon Gray</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
@@ -5885,7 +5893,7 @@
       </c>
       <c r="J62" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-BL-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-CG-M.jpg</t>
         </is>
       </c>
       <c r="K62" s="4" t="n">
@@ -5929,7 +5937,7 @@
     <row r="63">
       <c r="A63" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-PK-M</t>
+          <t>RN8-PC-PR-M</t>
         </is>
       </c>
       <c r="B63" s="7" t="inlineStr">
@@ -5949,7 +5957,7 @@
       </c>
       <c r="E63" s="6" t="inlineStr">
         <is>
-          <t>Sakura Pink</t>
+          <t>Sunset Purple</t>
         </is>
       </c>
       <c r="F63" s="6" t="inlineStr">
@@ -5974,7 +5982,7 @@
       </c>
       <c r="J63" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-PK-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-PR-M.jpg</t>
         </is>
       </c>
       <c r="K63" s="8" t="n">
@@ -6018,7 +6026,7 @@
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-CG-M</t>
+          <t>RN8-PC-TG-M</t>
         </is>
       </c>
       <c r="B64" s="3" t="inlineStr">
@@ -6038,7 +6046,7 @@
       </c>
       <c r="E64" s="2" t="inlineStr">
         <is>
-          <t>Carbon Gray</t>
+          <t>Titanium Gray</t>
         </is>
       </c>
       <c r="F64" s="2" t="inlineStr">
@@ -6063,7 +6071,7 @@
       </c>
       <c r="J64" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-CG-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-TG-M.jpg</t>
         </is>
       </c>
       <c r="K64" s="4" t="n">
@@ -6107,7 +6115,7 @@
     <row r="65">
       <c r="A65" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-PR-M</t>
+          <t>RN8-PC-BK-M</t>
         </is>
       </c>
       <c r="B65" s="7" t="inlineStr">
@@ -6127,7 +6135,7 @@
       </c>
       <c r="E65" s="6" t="inlineStr">
         <is>
-          <t>Sunset Purple</t>
+          <t>Classic Black</t>
         </is>
       </c>
       <c r="F65" s="6" t="inlineStr">
@@ -6152,7 +6160,7 @@
       </c>
       <c r="J65" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-PR-M.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-BK-M.jpg</t>
         </is>
       </c>
       <c r="K65" s="8" t="n">
@@ -6196,27 +6204,27 @@
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-TG-M</t>
+          <t>RN8-SIL-BK-M</t>
         </is>
       </c>
       <c r="B66" s="3" t="inlineStr">
         <is>
-          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C66" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
         <is>
-          <t>Hard PC</t>
+          <t>Silicone</t>
         </is>
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Titanium Gray</t>
+          <t>Obsidian Black</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
@@ -6236,22 +6244,22 @@
       </c>
       <c r="I66" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
         </is>
       </c>
       <c r="J66" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-TG-M.jpg</t>
+          <t>Realme Neo8/Silicone/sku/RN8-SIL-BK-M.jpg</t>
         </is>
       </c>
       <c r="K66" s="4" t="n">
-        <v>367.08</v>
+        <v>363.66</v>
       </c>
       <c r="L66" s="4" t="n">
         <v>10</v>
       </c>
       <c r="M66" s="4" t="n">
-        <v>31.2</v>
+        <v>50</v>
       </c>
       <c r="N66" s="4" t="n">
         <v>5</v>
@@ -6285,27 +6293,27 @@
     <row r="67">
       <c r="A67" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-BK-M</t>
+          <t>RN8-SIL-GY-M</t>
         </is>
       </c>
       <c r="B67" s="7" t="inlineStr">
         <is>
-          <t>Magnetic Heat Dissipation Matte Back Cover for Realme GT Neo 8 / Neo 7 – Ultra Thin Breathable Cooling Case with Ring Magnet</t>
+          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C67" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Realmeneo8 Mobile Phone Case, New Model, Realme Realmeneo7 Ultra-Thin Heat Dissipation Matte Fine Ring Magnetic Suction</t>
+          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
         </is>
       </c>
       <c r="D67" s="6" t="inlineStr">
         <is>
-          <t>Hard PC</t>
+          <t>Silicone</t>
         </is>
       </c>
       <c r="E67" s="6" t="inlineStr">
         <is>
-          <t>Classic Black</t>
+          <t>Matte Gray</t>
         </is>
       </c>
       <c r="F67" s="6" t="inlineStr">
@@ -6325,22 +6333,22 @@
       </c>
       <c r="I67" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000EPYKRSUQ2-suitable-for-realmeneo8-mobile-phone-case-new-model-realme-realmeneo7-ultra-thin-heat-dissipation-matte-fine-ring-magnetic-suction/1AD8326183006533</t>
+          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
         </is>
       </c>
       <c r="J67" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-BK-M.jpg</t>
+          <t>Realme Neo8/Silicone/sku/RN8-SIL-GY-M.jpg</t>
         </is>
       </c>
       <c r="K67" s="8" t="n">
-        <v>367.08</v>
+        <v>363.66</v>
       </c>
       <c r="L67" s="8" t="n">
         <v>10</v>
       </c>
       <c r="M67" s="8" t="n">
-        <v>31.2</v>
+        <v>50</v>
       </c>
       <c r="N67" s="8" t="n">
         <v>5</v>
@@ -6374,7 +6382,7 @@
     <row r="68">
       <c r="A68" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-BK-M</t>
+          <t>RN8-SIL-OR-M</t>
         </is>
       </c>
       <c r="B68" s="3" t="inlineStr">
@@ -6394,7 +6402,7 @@
       </c>
       <c r="E68" s="2" t="inlineStr">
         <is>
-          <t>Obsidian Black</t>
+          <t>Terracotta Orange</t>
         </is>
       </c>
       <c r="F68" s="2" t="inlineStr">
@@ -6419,7 +6427,7 @@
       </c>
       <c r="J68" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Silicone/sku/RN8-SIL-BK-M.jpg</t>
+          <t>Realme Neo8/Silicone/sku/RN8-SIL-OR-M.jpg</t>
         </is>
       </c>
       <c r="K68" s="4" t="n">
@@ -6463,27 +6471,27 @@
     <row r="69">
       <c r="A69" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-GY-M</t>
+          <t>RN8-SIL-GN-S-V2</t>
         </is>
       </c>
       <c r="B69" s="7" t="inlineStr">
         <is>
-          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C69" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
+          <t>Suitable for Realme Neo8 Mobile Phone Case Realmeneo8 New Model Rmx8899 Protective Cover Gt8 Liquid Silicone</t>
         </is>
       </c>
       <c r="D69" s="6" t="inlineStr">
         <is>
-          <t>Silicone</t>
+          <t>Liquid Silicone</t>
         </is>
       </c>
       <c r="E69" s="6" t="inlineStr">
         <is>
-          <t>Matte Gray</t>
+          <t>Mambo Green</t>
         </is>
       </c>
       <c r="F69" s="6" t="inlineStr">
@@ -6503,19 +6511,19 @@
       </c>
       <c r="I69" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
+          <t>https://moveon.global/BD_en/products/0000000AVTXCRWTL-suitable-for-realme-neo8-mobile-phone-case-realmeneo8-new-model-rmx8899-protective-cover-gt8-liquid-silicone/1AD8321207196552</t>
         </is>
       </c>
       <c r="J69" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Silicone/sku/RN8-SIL-GY-M.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S-V2.jpg</t>
         </is>
       </c>
       <c r="K69" s="8" t="n">
-        <v>363.66</v>
+        <v>268.2</v>
       </c>
       <c r="L69" s="8" t="n">
-        <v>10</v>
+        <v>79.55</v>
       </c>
       <c r="M69" s="8" t="n">
         <v>50</v>
@@ -6552,27 +6560,27 @@
     <row r="70">
       <c r="A70" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-OR-M</t>
+          <t>RN8-SIL-YL-S-V2</t>
         </is>
       </c>
       <c r="B70" s="3" t="inlineStr">
         <is>
-          <t>Magnetic Graphene Cooling Silicone Case for Realme GT Neo 8 – Snowflake Heat Dissipation Airbag Anti-Drop Back Cover</t>
+          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
         </is>
       </c>
       <c r="C70" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 Mobile Phone Case, New Creative Graphene Cooling Airbag Anti-Fall Silicone Case Realmeneo8</t>
+          <t>Suitable for Realme Neo8 Mobile Phone Case Realmeneo8 New Model Rmx8899 Protective Cover Gt8 Liquid Silicone</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
         <is>
-          <t>Silicone</t>
+          <t>Liquid Silicone</t>
         </is>
       </c>
       <c r="E70" s="2" t="inlineStr">
         <is>
-          <t>Terracotta Orange</t>
+          <t>Cream Yellow</t>
         </is>
       </c>
       <c r="F70" s="2" t="inlineStr">
@@ -6592,19 +6600,19 @@
       </c>
       <c r="I70" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000MV152HHVF-suitable-for-realme-neo8-mobile-phone-case-new-creative-graphene-cooling-airbag-anti-fall-silicone-case-realmeneo8/1AD8330600315865</t>
+          <t>https://moveon.global/BD_en/products/0000000AVTXCRWTL-suitable-for-realme-neo8-mobile-phone-case-realmeneo8-new-model-rmx8899-protective-cover-gt8-liquid-silicone/1AD8321207196552</t>
         </is>
       </c>
       <c r="J70" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Silicone/sku/RN8-SIL-OR-M.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-YL-S-V2.jpg</t>
         </is>
       </c>
       <c r="K70" s="4" t="n">
-        <v>363.66</v>
+        <v>268.2</v>
       </c>
       <c r="L70" s="4" t="n">
-        <v>10</v>
+        <v>79.55</v>
       </c>
       <c r="M70" s="4" t="n">
         <v>50</v>
@@ -6641,7 +6649,7 @@
     <row r="71">
       <c r="A71" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-GN-S-V2</t>
+          <t>RN8-SIL-PR-S-V2</t>
         </is>
       </c>
       <c r="B71" s="7" t="inlineStr">
@@ -6661,7 +6669,7 @@
       </c>
       <c r="E71" s="6" t="inlineStr">
         <is>
-          <t>Mambo Green</t>
+          <t>Purple Bean</t>
         </is>
       </c>
       <c r="F71" s="6" t="inlineStr">
@@ -6686,7 +6694,7 @@
       </c>
       <c r="J71" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GN-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S-V2.jpg</t>
         </is>
       </c>
       <c r="K71" s="8" t="n">
@@ -6730,7 +6738,7 @@
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-YL-S-V2</t>
+          <t>RN8-SIL-PK-S-V2</t>
         </is>
       </c>
       <c r="B72" s="3" t="inlineStr">
@@ -6750,7 +6758,7 @@
       </c>
       <c r="E72" s="2" t="inlineStr">
         <is>
-          <t>Cream Yellow</t>
+          <t>Sand Pink</t>
         </is>
       </c>
       <c r="F72" s="2" t="inlineStr">
@@ -6775,7 +6783,7 @@
       </c>
       <c r="J72" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-YL-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PK-S-V2.jpg</t>
         </is>
       </c>
       <c r="K72" s="4" t="n">
@@ -6819,7 +6827,7 @@
     <row r="73">
       <c r="A73" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-PR-S-V2</t>
+          <t>RN8-SIL-BL-S-V2</t>
         </is>
       </c>
       <c r="B73" s="7" t="inlineStr">
@@ -6839,7 +6847,7 @@
       </c>
       <c r="E73" s="6" t="inlineStr">
         <is>
-          <t>Purple Bean</t>
+          <t>Sky Blue</t>
         </is>
       </c>
       <c r="F73" s="6" t="inlineStr">
@@ -6864,7 +6872,7 @@
       </c>
       <c r="J73" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PR-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S-V2.jpg</t>
         </is>
       </c>
       <c r="K73" s="8" t="n">
@@ -6908,7 +6916,7 @@
     <row r="74">
       <c r="A74" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-PK-S-V2</t>
+          <t>RN8-SIL-WT-S-V2</t>
         </is>
       </c>
       <c r="B74" s="3" t="inlineStr">
@@ -6928,7 +6936,7 @@
       </c>
       <c r="E74" s="2" t="inlineStr">
         <is>
-          <t>Sand Pink</t>
+          <t>Antique White</t>
         </is>
       </c>
       <c r="F74" s="2" t="inlineStr">
@@ -6953,7 +6961,7 @@
       </c>
       <c r="J74" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-PK-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S-V2.jpg</t>
         </is>
       </c>
       <c r="K74" s="4" t="n">
@@ -6997,7 +7005,7 @@
     <row r="75">
       <c r="A75" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-BL-S-V2</t>
+          <t>RN8-SIL-BK-S-V2</t>
         </is>
       </c>
       <c r="B75" s="7" t="inlineStr">
@@ -7017,7 +7025,7 @@
       </c>
       <c r="E75" s="6" t="inlineStr">
         <is>
-          <t>Sky Blue</t>
+          <t>Classic Black</t>
         </is>
       </c>
       <c r="F75" s="6" t="inlineStr">
@@ -7042,7 +7050,7 @@
       </c>
       <c r="J75" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BL-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S-V2.jpg</t>
         </is>
       </c>
       <c r="K75" s="8" t="n">
@@ -7086,7 +7094,7 @@
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-WT-S-V2</t>
+          <t>RN8-SIL-GY-S-V2</t>
         </is>
       </c>
       <c r="B76" s="3" t="inlineStr">
@@ -7106,7 +7114,7 @@
       </c>
       <c r="E76" s="2" t="inlineStr">
         <is>
-          <t>Antique White</t>
+          <t>Charcoal Gray</t>
         </is>
       </c>
       <c r="F76" s="2" t="inlineStr">
@@ -7131,7 +7139,7 @@
       </c>
       <c r="J76" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GY-S-V2.jpg</t>
         </is>
       </c>
       <c r="K76" s="4" t="n">
@@ -7175,7 +7183,7 @@
     <row r="77">
       <c r="A77" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-BK-S-V2</t>
+          <t>RN8-SIL-WT-S-V3</t>
         </is>
       </c>
       <c r="B77" s="7" t="inlineStr">
@@ -7195,7 +7203,7 @@
       </c>
       <c r="E77" s="6" t="inlineStr">
         <is>
-          <t>Classic Black</t>
+          <t>Pure White</t>
         </is>
       </c>
       <c r="F77" s="6" t="inlineStr">
@@ -7220,7 +7228,7 @@
       </c>
       <c r="J77" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-BK-S-V2.jpg</t>
+          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S-V3.jpg</t>
         </is>
       </c>
       <c r="K77" s="8" t="n">
@@ -7264,27 +7272,27 @@
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
         <is>
-          <t>RN8-SIL-GY-S-V2</t>
+          <t>RN8-PC-BK-S</t>
         </is>
       </c>
       <c r="B78" s="3" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
         </is>
       </c>
       <c r="C78" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 Mobile Phone Case Realmeneo8 New Model Rmx8899 Protective Cover Gt8 Liquid Silicone</t>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
         <is>
-          <t>Liquid Silicone</t>
+          <t>Hard PC</t>
         </is>
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>Charcoal Gray</t>
+          <t>Black</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -7304,22 +7312,22 @@
       </c>
       <c r="I78" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000AVTXCRWTL-suitable-for-realme-neo8-mobile-phone-case-realmeneo8-new-model-rmx8899-protective-cover-gt8-liquid-silicone/1AD8321207196552</t>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
         </is>
       </c>
       <c r="J78" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-GY-S-V2.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-BK-S.jpg</t>
         </is>
       </c>
       <c r="K78" s="4" t="n">
-        <v>268.2</v>
+        <v>147.74</v>
       </c>
       <c r="L78" s="4" t="n">
-        <v>79.55</v>
+        <v>50</v>
       </c>
       <c r="M78" s="4" t="n">
-        <v>50</v>
+        <v>62.4</v>
       </c>
       <c r="N78" s="4" t="n">
         <v>5</v>
@@ -7353,27 +7361,27 @@
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>RN8-SIL-WT-S-V3</t>
+          <t>RN8-PC-SV-S</t>
         </is>
       </c>
       <c r="B79" s="7" t="inlineStr">
         <is>
-          <t>Luxury Liquid Silicone Shockproof Case for Realme GT Neo 8 – Camera Lens Protection Soft Anti-Drop Back Cover</t>
+          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
         </is>
       </c>
       <c r="C79" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Realme Neo8 Mobile Phone Case Realmeneo8 New Model Rmx8899 Protective Cover Gt8 Liquid Silicone</t>
+          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>Liquid Silicone</t>
+          <t>Hard PC</t>
         </is>
       </c>
       <c r="E79" s="6" t="inlineStr">
         <is>
-          <t>Pure White</t>
+          <t>Silver</t>
         </is>
       </c>
       <c r="F79" s="6" t="inlineStr">
@@ -7393,22 +7401,22 @@
       </c>
       <c r="I79" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000AVTXCRWTL-suitable-for-realme-neo8-mobile-phone-case-realmeneo8-new-model-rmx8899-protective-cover-gt8-liquid-silicone/1AD8321207196552</t>
+          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
         </is>
       </c>
       <c r="J79" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Liquid Silicone/sku/RN8-SIL-WT-S-V3.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-SV-S.jpg</t>
         </is>
       </c>
       <c r="K79" s="8" t="n">
-        <v>268.2</v>
+        <v>147.74</v>
       </c>
       <c r="L79" s="8" t="n">
-        <v>79.55</v>
+        <v>50</v>
       </c>
       <c r="M79" s="8" t="n">
-        <v>50</v>
+        <v>62.4</v>
       </c>
       <c r="N79" s="8" t="n">
         <v>5</v>
@@ -7442,7 +7450,7 @@
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-BK-S</t>
+          <t>RN8-PC-CL-C</t>
         </is>
       </c>
       <c r="B80" s="3" t="inlineStr">
@@ -7462,7 +7470,7 @@
       </c>
       <c r="E80" s="2" t="inlineStr">
         <is>
-          <t>Black</t>
+          <t>Transparent</t>
         </is>
       </c>
       <c r="F80" s="2" t="inlineStr">
@@ -7487,11 +7495,11 @@
       </c>
       <c r="J80" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-BK-S.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-CL-C.jpg</t>
         </is>
       </c>
       <c r="K80" s="4" t="n">
-        <v>147.74</v>
+        <v>113.64</v>
       </c>
       <c r="L80" s="4" t="n">
         <v>50</v>
@@ -7531,7 +7539,7 @@
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-SV-S</t>
+          <t>RN8-PC-RD-S</t>
         </is>
       </c>
       <c r="B81" s="7" t="inlineStr">
@@ -7551,7 +7559,7 @@
       </c>
       <c r="E81" s="6" t="inlineStr">
         <is>
-          <t>Silver</t>
+          <t>Burgundy Red</t>
         </is>
       </c>
       <c r="F81" s="6" t="inlineStr">
@@ -7576,7 +7584,7 @@
       </c>
       <c r="J81" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-SV-S.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-RD-S.jpg</t>
         </is>
       </c>
       <c r="K81" s="8" t="n">
@@ -7620,7 +7628,7 @@
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-CL-C</t>
+          <t>RN8-PC-TB-S</t>
         </is>
       </c>
       <c r="B82" s="3" t="inlineStr">
@@ -7640,7 +7648,7 @@
       </c>
       <c r="E82" s="2" t="inlineStr">
         <is>
-          <t>Transparent</t>
+          <t>Titanium Black</t>
         </is>
       </c>
       <c r="F82" s="2" t="inlineStr">
@@ -7665,11 +7673,11 @@
       </c>
       <c r="J82" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-CL-C.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-TB-S.jpg</t>
         </is>
       </c>
       <c r="K82" s="4" t="n">
-        <v>113.64</v>
+        <v>147.74</v>
       </c>
       <c r="L82" s="4" t="n">
         <v>50</v>
@@ -7709,7 +7717,7 @@
     <row r="83">
       <c r="A83" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-RD-S</t>
+          <t>RN8-PC-GD-S</t>
         </is>
       </c>
       <c r="B83" s="7" t="inlineStr">
@@ -7729,7 +7737,7 @@
       </c>
       <c r="E83" s="6" t="inlineStr">
         <is>
-          <t>Burgundy Red</t>
+          <t>Golden</t>
         </is>
       </c>
       <c r="F83" s="6" t="inlineStr">
@@ -7754,7 +7762,7 @@
       </c>
       <c r="J83" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-RD-S.jpg</t>
+          <t>Realme Neo8/Hard PC/sku/RN8-PC-GD-S.jpg</t>
         </is>
       </c>
       <c r="K83" s="8" t="n">
@@ -7798,27 +7806,27 @@
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
         <is>
-          <t>RN8-PC-TB-S</t>
+          <t>RN8-GLS-YL-S</t>
         </is>
       </c>
       <c r="B84" s="3" t="inlineStr">
         <is>
-          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
         </is>
       </c>
       <c r="C84" s="3" t="inlineStr">
         <is>
-          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
         <is>
-          <t>Hard PC</t>
+          <t>Tempered Glass</t>
         </is>
       </c>
       <c r="E84" s="2" t="inlineStr">
         <is>
-          <t>Titanium Black</t>
+          <t>A6077 Collection Yellow</t>
         </is>
       </c>
       <c r="F84" s="2" t="inlineStr">
@@ -7838,22 +7846,22 @@
       </c>
       <c r="I84" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
         </is>
       </c>
       <c r="J84" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-TB-S.jpg</t>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-YL-S.jpg</t>
         </is>
       </c>
       <c r="K84" s="4" t="n">
-        <v>147.74</v>
+        <v>156.83</v>
       </c>
       <c r="L84" s="4" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="M84" s="4" t="n">
-        <v>62.4</v>
+        <v>468</v>
       </c>
       <c r="N84" s="4" t="n">
         <v>5</v>
@@ -7887,27 +7895,27 @@
     <row r="85">
       <c r="A85" s="6" t="inlineStr">
         <is>
-          <t>RN8-PC-GD-S</t>
+          <t>RN8-GLS-BL-S</t>
         </is>
       </c>
       <c r="B85" s="7" t="inlineStr">
         <is>
-          <t>Corrugated Metallic Paint Hard Case with Metal Buttons for Realme GT Neo 8 – Luxury Shockproof Anti-Drop Protective Back Cover</t>
+          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
         </is>
       </c>
       <c r="C85" s="7" t="inlineStr">
         <is>
-          <t>Suitable for Oppo Find X9 Ultra corrugated metal paint phone case, Reno 16 metal button case, Realme GT8 hard case</t>
+          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
         </is>
       </c>
       <c r="D85" s="6" t="inlineStr">
         <is>
-          <t>Hard PC</t>
+          <t>Tempered Glass</t>
         </is>
       </c>
       <c r="E85" s="6" t="inlineStr">
         <is>
-          <t>Golden</t>
+          <t>A6078 Yuanzu Blue</t>
         </is>
       </c>
       <c r="F85" s="6" t="inlineStr">
@@ -7927,22 +7935,22 @@
       </c>
       <c r="I85" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000E102ORKG6-suitable-for-oppo-find-x9-ultra-corrugated-metal-paint-phone-case-reno-16-metal-button-case-realme-gt8-hard-case/1AD8372161823684</t>
+          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
         </is>
       </c>
       <c r="J85" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Hard PC/sku/RN8-PC-GD-S.jpg</t>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-BL-S.jpg</t>
         </is>
       </c>
       <c r="K85" s="8" t="n">
-        <v>147.74</v>
+        <v>156.83</v>
       </c>
       <c r="L85" s="8" t="n">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="M85" s="8" t="n">
-        <v>62.4</v>
+        <v>468</v>
       </c>
       <c r="N85" s="8" t="n">
         <v>5</v>
@@ -7976,7 +7984,7 @@
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
         <is>
-          <t>RN8-GLS-YL-S</t>
+          <t>RN8-GLS-GN-S</t>
         </is>
       </c>
       <c r="B86" s="3" t="inlineStr">
@@ -7996,7 +8004,7 @@
       </c>
       <c r="E86" s="2" t="inlineStr">
         <is>
-          <t>A6077 Collection Yellow</t>
+          <t>A6079 Passion Green</t>
         </is>
       </c>
       <c r="F86" s="2" t="inlineStr">
@@ -8021,7 +8029,7 @@
       </c>
       <c r="J86" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-YL-S.jpg</t>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-GN-S.jpg</t>
         </is>
       </c>
       <c r="K86" s="4" t="n">
@@ -8065,7 +8073,7 @@
     <row r="87">
       <c r="A87" s="6" t="inlineStr">
         <is>
-          <t>RN8-GLS-BL-S</t>
+          <t>RN8-GLS-GY-S</t>
         </is>
       </c>
       <c r="B87" s="7" t="inlineStr">
@@ -8085,7 +8093,7 @@
       </c>
       <c r="E87" s="6" t="inlineStr">
         <is>
-          <t>A6078 Yuanzu Blue</t>
+          <t>A6080 Diamond Gray</t>
         </is>
       </c>
       <c r="F87" s="6" t="inlineStr">
@@ -8110,7 +8118,7 @@
       </c>
       <c r="J87" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-BL-S.jpg</t>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-GY-S.jpg</t>
         </is>
       </c>
       <c r="K87" s="8" t="n">
@@ -8154,7 +8162,7 @@
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
         <is>
-          <t>RN8-GLS-GN-S</t>
+          <t>RN8-GLS-PR-S</t>
         </is>
       </c>
       <c r="B88" s="3" t="inlineStr">
@@ -8174,7 +8182,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>A6079 Passion Green</t>
+          <t>A6081 Ghost Purple</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -8199,7 +8207,7 @@
       </c>
       <c r="J88" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-GN-S.jpg</t>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-PR-S.jpg</t>
         </is>
       </c>
       <c r="K88" s="4" t="n">
@@ -8243,7 +8251,7 @@
     <row r="89">
       <c r="A89" s="6" t="inlineStr">
         <is>
-          <t>RN8-GLS-GY-S</t>
+          <t>RN8-GLS-RD-S</t>
         </is>
       </c>
       <c r="B89" s="7" t="inlineStr">
@@ -8263,7 +8271,7 @@
       </c>
       <c r="E89" s="6" t="inlineStr">
         <is>
-          <t>A6080 Diamond Gray</t>
+          <t>A6082 Alarm Red</t>
         </is>
       </c>
       <c r="F89" s="6" t="inlineStr">
@@ -8288,7 +8296,7 @@
       </c>
       <c r="J89" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-GY-S.jpg</t>
+          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-RD-S.jpg</t>
         </is>
       </c>
       <c r="K89" s="8" t="n">
@@ -8332,32 +8340,32 @@
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
         <is>
-          <t>RN8-GLS-PR-S</t>
+          <t>S26U-PC-LG-W</t>
         </is>
       </c>
       <c r="B90" s="3" t="inlineStr">
         <is>
-          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+          <t>Frameless Wood Grain Magnetic Hard Case for Samsung Galaxy S26 Ultra – Luxury Shockproof Ultra-Slim Armor Protective Back Cover</t>
         </is>
       </c>
       <c r="C90" s="3" t="inlineStr">
         <is>
-          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+          <t>Foreign Trade Cross-Border Applicable Samsung S26Ultra Mobile Phone Case Frameless Wood Grain Magnetic Suction S25U Anti-Fall 24 Protective Case</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
         <is>
-          <t>Tempered Glass</t>
+          <t>Hard PC</t>
         </is>
       </c>
       <c r="E90" s="2" t="inlineStr">
         <is>
-          <t>A6081 Ghost Purple</t>
+          <t>Light Gray Wood Grain</t>
         </is>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
-          <t>Realme Neo8</t>
+          <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
       <c r="G90" s="2" t="inlineStr">
@@ -8372,22 +8380,22 @@
       </c>
       <c r="I90" s="3" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
         </is>
       </c>
       <c r="J90" s="3" t="inlineStr">
         <is>
-          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-PR-S.jpg</t>
+          <t>Samsung Galaxy S26 Ultra/Hard PC/sku/S26U-PC-LG-W.jpg</t>
         </is>
       </c>
       <c r="K90" s="4" t="n">
-        <v>156.83</v>
+        <v>215.93</v>
       </c>
       <c r="L90" s="4" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="M90" s="4" t="n">
-        <v>468</v>
+        <v>50</v>
       </c>
       <c r="N90" s="4" t="n">
         <v>5</v>
@@ -8421,32 +8429,32 @@
     <row r="91">
       <c r="A91" s="6" t="inlineStr">
         <is>
-          <t>RN8-GLS-RD-S</t>
+          <t>S26U-PC-DG-W</t>
         </is>
       </c>
       <c r="B91" s="7" t="inlineStr">
         <is>
-          <t>Luxury Tempered Glass Shockproof Protective Back Cover for Realme Neo8 – Ultra-Slim Anti-Drop Case</t>
+          <t>Frameless Wood Grain Magnetic Hard Case for Samsung Galaxy S26 Ultra – Luxury Shockproof Ultra-Slim Armor Protective Back Cover</t>
         </is>
       </c>
       <c r="C91" s="7" t="inlineStr">
         <is>
-          <t>Transformers-Themed Glass Case for Realme Neo8, New Stylish and High-End Protective Cover, Ultra-Thin and Shockproof</t>
+          <t>Foreign Trade Cross-Border Applicable Samsung S26Ultra Mobile Phone Case Frameless Wood Grain Magnetic Suction S25U Anti-Fall 24 Protective Case</t>
         </is>
       </c>
       <c r="D91" s="6" t="inlineStr">
         <is>
-          <t>Tempered Glass</t>
+          <t>Hard PC</t>
         </is>
       </c>
       <c r="E91" s="6" t="inlineStr">
         <is>
-          <t>A6082 Alarm Red</t>
+          <t>Dark Gray Wood Grain</t>
         </is>
       </c>
       <c r="F91" s="6" t="inlineStr">
         <is>
-          <t>Realme Neo8</t>
+          <t>Samsung Galaxy S26 Ultra</t>
         </is>
       </c>
       <c r="G91" s="6" t="inlineStr">
@@ -8461,22 +8469,22 @@
       </c>
       <c r="I91" s="7" t="inlineStr">
         <is>
-          <t>https://moveon.global/BD_en/products/0000000YB9IRZNPB-transformers-themed-glass-case-for-realme-neo8-new-stylish-and-high-end-protective-cover-ultra-thin-and-shockproof/1AD8329701440673</t>
+          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
         </is>
       </c>
       <c r="J91" s="7" t="inlineStr">
         <is>
-          <t>Realme Neo8/Tempered Glass/sku/RN8-GLS-RD-S.jpg</t>
+          <t>Samsung Galaxy S26 Ultra/Hard PC/sku/S26U-PC-DG-W.jpg</t>
         </is>
       </c>
       <c r="K91" s="8" t="n">
-        <v>156.83</v>
+        <v>215.93</v>
       </c>
       <c r="L91" s="8" t="n">
-        <v>45</v>
+        <v>20</v>
       </c>
       <c r="M91" s="8" t="n">
-        <v>468</v>
+        <v>50</v>
       </c>
       <c r="N91" s="8" t="n">
         <v>5</v>
@@ -8504,6 +8512,362 @@
       </c>
       <c r="U91" s="8">
         <f>IF(T91&lt;300, 0, MIN(99, IF(T91&lt;500, T91*7%, IF(T91&lt;700, T91*12%, T91*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" s="2" t="inlineStr">
+        <is>
+          <t>S26U-PC-LY-W</t>
+        </is>
+      </c>
+      <c r="B92" s="3" t="inlineStr">
+        <is>
+          <t>Frameless Wood Grain Magnetic Hard Case for Samsung Galaxy S26 Ultra – Luxury Shockproof Ultra-Slim Armor Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C92" s="3" t="inlineStr">
+        <is>
+          <t>Foreign Trade Cross-Border Applicable Samsung S26Ultra Mobile Phone Case Frameless Wood Grain Magnetic Suction S25U Anti-Fall 24 Protective Case</t>
+        </is>
+      </c>
+      <c r="D92" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E92" s="2" t="inlineStr">
+        <is>
+          <t>Light Yellow Wood Grain</t>
+        </is>
+      </c>
+      <c r="F92" s="2" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra</t>
+        </is>
+      </c>
+      <c r="G92" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H92" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I92" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
+        </is>
+      </c>
+      <c r="J92" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra/Hard PC/sku/S26U-PC-LY-W.jpg</t>
+        </is>
+      </c>
+      <c r="K92" s="4" t="n">
+        <v>215.93</v>
+      </c>
+      <c r="L92" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M92" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="N92" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O92" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P92" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q92" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R92" s="4">
+        <f>SUM(K92:Q92)</f>
+        <v/>
+      </c>
+      <c r="S92" s="4">
+        <f>IF(R92&lt;300, R92*1.4, IF(R92&lt;400, R92*1.33, R92*1.25))</f>
+        <v/>
+      </c>
+      <c r="T92" s="5">
+        <f>INT(S92/100)*100 + IF(MOD(ROUND(S92,0),100)&lt;25, 0, IF(MOD(ROUND(S92,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U92" s="4">
+        <f>IF(T92&lt;300, 0, MIN(99, IF(T92&lt;500, T92*7%, IF(T92&lt;700, T92*12%, T92*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" s="6" t="inlineStr">
+        <is>
+          <t>S26U-PC-PL-W</t>
+        </is>
+      </c>
+      <c r="B93" s="7" t="inlineStr">
+        <is>
+          <t>Frameless Wood Grain Magnetic Hard Case for Samsung Galaxy S26 Ultra – Luxury Shockproof Ultra-Slim Armor Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C93" s="7" t="inlineStr">
+        <is>
+          <t>Foreign Trade Cross-Border Applicable Samsung S26Ultra Mobile Phone Case Frameless Wood Grain Magnetic Suction S25U Anti-Fall 24 Protective Case</t>
+        </is>
+      </c>
+      <c r="D93" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E93" s="6" t="inlineStr">
+        <is>
+          <t>Poplar Wood Grain</t>
+        </is>
+      </c>
+      <c r="F93" s="6" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra</t>
+        </is>
+      </c>
+      <c r="G93" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H93" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I93" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
+        </is>
+      </c>
+      <c r="J93" s="7" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra/Hard PC/sku/S26U-PC-PL-W.jpg</t>
+        </is>
+      </c>
+      <c r="K93" s="8" t="n">
+        <v>215.93</v>
+      </c>
+      <c r="L93" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="M93" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="N93" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O93" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P93" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q93" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R93" s="8">
+        <f>SUM(K93:Q93)</f>
+        <v/>
+      </c>
+      <c r="S93" s="8">
+        <f>IF(R93&lt;300, R93*1.4, IF(R93&lt;400, R93*1.33, R93*1.25))</f>
+        <v/>
+      </c>
+      <c r="T93" s="9">
+        <f>INT(S93/100)*100 + IF(MOD(ROUND(S93,0),100)&lt;25, 0, IF(MOD(ROUND(S93,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U93" s="8">
+        <f>IF(T93&lt;300, 0, MIN(99, IF(T93&lt;500, T93*7%, IF(T93&lt;700, T93*12%, T93*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>S26U-PC-RP-W</t>
+        </is>
+      </c>
+      <c r="B94" s="3" t="inlineStr">
+        <is>
+          <t>Frameless Wood Grain Magnetic Hard Case for Samsung Galaxy S26 Ultra – Luxury Shockproof Ultra-Slim Armor Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C94" s="3" t="inlineStr">
+        <is>
+          <t>Foreign Trade Cross-Border Applicable Samsung S26Ultra Mobile Phone Case Frameless Wood Grain Magnetic Suction S25U Anti-Fall 24 Protective Case</t>
+        </is>
+      </c>
+      <c r="D94" s="2" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E94" s="2" t="inlineStr">
+        <is>
+          <t>Red Poplar Wood Grain</t>
+        </is>
+      </c>
+      <c r="F94" s="2" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra</t>
+        </is>
+      </c>
+      <c r="G94" s="2" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H94" s="2" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I94" s="3" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
+        </is>
+      </c>
+      <c r="J94" s="3" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra/Hard PC/sku/S26U-PC-RP-W.jpg</t>
+        </is>
+      </c>
+      <c r="K94" s="4" t="n">
+        <v>215.93</v>
+      </c>
+      <c r="L94" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="M94" s="4" t="n">
+        <v>50</v>
+      </c>
+      <c r="N94" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="O94" s="4" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P94" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q94" s="4" t="n">
+        <v>0</v>
+      </c>
+      <c r="R94" s="4">
+        <f>SUM(K94:Q94)</f>
+        <v/>
+      </c>
+      <c r="S94" s="4">
+        <f>IF(R94&lt;300, R94*1.4, IF(R94&lt;400, R94*1.33, R94*1.25))</f>
+        <v/>
+      </c>
+      <c r="T94" s="5">
+        <f>INT(S94/100)*100 + IF(MOD(ROUND(S94,0),100)&lt;25, 0, IF(MOD(ROUND(S94,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U94" s="4">
+        <f>IF(T94&lt;300, 0, MIN(99, IF(T94&lt;500, T94*7%, IF(T94&lt;700, T94*12%, T94*15%))))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" s="6" t="inlineStr">
+        <is>
+          <t>S26U-PC-CB-W</t>
+        </is>
+      </c>
+      <c r="B95" s="7" t="inlineStr">
+        <is>
+          <t>Frameless Wood Grain Magnetic Hard Case for Samsung Galaxy S26 Ultra – Luxury Shockproof Ultra-Slim Armor Protective Back Cover</t>
+        </is>
+      </c>
+      <c r="C95" s="7" t="inlineStr">
+        <is>
+          <t>Foreign Trade Cross-Border Applicable Samsung S26Ultra Mobile Phone Case Frameless Wood Grain Magnetic Suction S25U Anti-Fall 24 Protective Case</t>
+        </is>
+      </c>
+      <c r="D95" s="6" t="inlineStr">
+        <is>
+          <t>Hard PC</t>
+        </is>
+      </c>
+      <c r="E95" s="6" t="inlineStr">
+        <is>
+          <t>Cowboy Wood Grain</t>
+        </is>
+      </c>
+      <c r="F95" s="6" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra</t>
+        </is>
+      </c>
+      <c r="G95" s="6" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="H95" s="6" t="inlineStr">
+        <is>
+          <t>Link</t>
+        </is>
+      </c>
+      <c r="I95" s="7" t="inlineStr">
+        <is>
+          <t>https://moveon.global/BD_en/products/0000000BB811A2TJ-foreign-trade-cross-border-applicable-samsung-s26ultra-mobile-phone-case-frameless-wood-grain-magnetic-suction-s25u-anti-fall-24-protective-case/1AC6839645384080</t>
+        </is>
+      </c>
+      <c r="J95" s="7" t="inlineStr">
+        <is>
+          <t>Samsung Galaxy S26 Ultra/Hard PC/sku/S26U-PC-CB-W.jpg</t>
+        </is>
+      </c>
+      <c r="K95" s="8" t="n">
+        <v>215.93</v>
+      </c>
+      <c r="L95" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="M95" s="8" t="n">
+        <v>50</v>
+      </c>
+      <c r="N95" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="O95" s="8" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="P95" s="8" t="n">
+        <v>20</v>
+      </c>
+      <c r="Q95" s="8" t="n">
+        <v>0</v>
+      </c>
+      <c r="R95" s="8">
+        <f>SUM(K95:Q95)</f>
+        <v/>
+      </c>
+      <c r="S95" s="8">
+        <f>IF(R95&lt;300, R95*1.4, IF(R95&lt;400, R95*1.33, R95*1.25))</f>
+        <v/>
+      </c>
+      <c r="T95" s="9">
+        <f>INT(S95/100)*100 + IF(MOD(ROUND(S95,0),100)&lt;25, 0, IF(MOD(ROUND(S95,0),100)&lt;=74, 49, 99))</f>
+        <v/>
+      </c>
+      <c r="U95" s="8">
+        <f>IF(T95&lt;300, 0, MIN(99, IF(T95&lt;500, T95*7%, IF(T95&lt;700, T95*12%, T95*15%))))</f>
         <v/>
       </c>
     </row>

</xml_diff>